<commit_message>
added sd card support
</commit_message>
<xml_diff>
--- a/docs/HX35_menuItems.xlsx
+++ b/docs/HX35_menuItems.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="215">
   <si>
     <t>Index #</t>
   </si>
@@ -641,6 +641,30 @@
   </si>
   <si>
     <t>int8_t EditValues[MENU_ITEMCOUNT] = {</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>SD Card Init</t>
+  </si>
+  <si>
+    <t>Load SD Scan</t>
+  </si>
+  <si>
+    <t>Flash SD Scan</t>
+  </si>
+  <si>
+    <t>Flash FPGA</t>
+  </si>
+  <si>
+    <t>Reload FPGA</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Flash Other</t>
   </si>
 </sst>
 </file>
@@ -777,7 +801,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -814,6 +838,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -827,7 +857,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -938,6 +968,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1244,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="4" customWidth="1"/>
@@ -1320,7 +1353,7 @@
         <v>172</v>
       </c>
       <c r="C2" s="5" t="str">
-        <f>G10</f>
+        <f>G11</f>
         <v>m_upper_db_16</v>
       </c>
       <c r="D2" s="1">
@@ -1340,23 +1373,23 @@
         <v>199</v>
       </c>
       <c r="I2" s="18" t="str">
-        <f t="shared" ref="I2:I9" si="0">CONCATENATE("  ",G2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <f t="shared" ref="I2:I10" si="0">CONCATENATE("  ",G2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_upper_dbs, // #0 = Upper DBs</v>
       </c>
       <c r="J2" s="1" t="str">
-        <f t="shared" ref="J2:J9" si="1">CONCATENATE("  { """,B2,""" },  // #",A2," ",IF(C2&lt;0," EXIT SUBM",""))</f>
+        <f t="shared" ref="J2:J10" si="1">CONCATENATE("  { """,B2,""" },  // #",A2," ",IF(C2&lt;0," EXIT SUBM",""))</f>
         <v xml:space="preserve">  { "Upper DBs" },  // #0 </v>
       </c>
       <c r="K2" s="18" t="str">
-        <f t="shared" ref="K2:K9" si="2">CONCATENATE("  ",D2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <f t="shared" ref="K2:K10" si="2">CONCATENATE("  ",D2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  1, // #0 = Upper DBs</v>
       </c>
       <c r="L2" s="18" t="str">
-        <f t="shared" ref="L2:L9" si="3">CONCATENATE("  ",E2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <f t="shared" ref="L2:L10" si="3">CONCATENATE("  ",E2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #0 = Upper DBs</v>
       </c>
       <c r="M2" s="18" t="str">
-        <f t="shared" ref="M2:M9" si="4">CONCATENATE("  ",C2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <f t="shared" ref="M2:M10" si="4">CONCATENATE("  ",C2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_upper_db_16, // #0 = Upper DBs</v>
       </c>
       <c r="N2" s="18" t="str">
@@ -1364,21 +1397,21 @@
         <v xml:space="preserve">  ac_none, // Upper DBs</v>
       </c>
       <c r="O2" s="18" t="str">
-        <f t="shared" ref="O2:O40" si="5">CONCATENATE("  ",F2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <f t="shared" ref="O2:O49" si="5">CONCATENATE("  ",F2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #0 = Upper DBs</v>
       </c>
       <c r="P2" s="13"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <f t="shared" ref="A3:A38" si="6">A2+1</f>
+        <f t="shared" ref="A3:A47" si="6">A2+1</f>
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>173</v>
       </c>
       <c r="C3" s="5" t="str">
-        <f>G20</f>
+        <f>G21</f>
         <v>m_lower_db_16</v>
       </c>
       <c r="D3" s="1">
@@ -1391,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="12" t="str">
-        <f t="shared" ref="G3:G8" si="7">CONCATENATE("m_",LOWER(SUBSTITUTE(B3," ","_")))</f>
+        <f t="shared" ref="G3:G9" si="7">CONCATENATE("m_",LOWER(SUBSTITUTE(B3," ","_")))</f>
         <v>m_lower_dbs</v>
       </c>
       <c r="H3" s="12" t="s">
@@ -1418,7 +1451,7 @@
         <v xml:space="preserve">  m_lower_db_16, // #1 = Lower DBs</v>
       </c>
       <c r="N3" s="18" t="str">
-        <f t="shared" ref="N3:N40" si="8">CONCATENATE("  ",H3,", // ",B3)</f>
+        <f t="shared" ref="N3:N49" si="8">CONCATENATE("  ",H3,", // ",B3)</f>
         <v xml:space="preserve">  ac_none, // Lower DBs</v>
       </c>
       <c r="O3" s="18" t="str">
@@ -1436,7 +1469,7 @@
         <v>174</v>
       </c>
       <c r="C4" s="5" t="str">
-        <f>G30</f>
+        <f>G31</f>
         <v>m_pedal_db_16</v>
       </c>
       <c r="D4" s="1">
@@ -1599,1533 +1632,1534 @@
       </c>
       <c r="P6" s="17"/>
     </row>
-    <row r="7" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>61</v>
+      <c r="B7" s="33" t="s">
+        <v>207</v>
       </c>
       <c r="C7" s="5" t="str">
-        <f>G33</f>
-        <v>m_kbd_driver</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="19">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
+        <f>G34</f>
+        <v>m_sd_card_init</v>
+      </c>
+      <c r="D7" s="12">
+        <v>0</v>
+      </c>
+      <c r="E7" s="12">
+        <v>127</v>
+      </c>
+      <c r="F7" s="12">
+        <v>-47</v>
       </c>
       <c r="G7" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(B7," ","_")))</f>
-        <v>m_keyboard</v>
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B7,"/","")," ","_")))</f>
+        <v>m_utilities</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>199</v>
       </c>
       <c r="I7" s="18" t="str">
+        <f t="shared" ref="I7" si="10">CONCATENATE("  ",G7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_utilities, // #5 = Utilities</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <f t="shared" ref="J7" si="11">CONCATENATE("  { """,B7,""" },  // #",A7," ",IF(C7&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Utilities" },  // #5 </v>
+      </c>
+      <c r="K7" s="18" t="str">
+        <f t="shared" ref="K7" si="12">CONCATENATE("  ",D7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #5 = Utilities</v>
+      </c>
+      <c r="L7" s="18" t="str">
+        <f t="shared" ref="L7" si="13">CONCATENATE("  ",E7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  127, // #5 = Utilities</v>
+      </c>
+      <c r="M7" s="18" t="str">
+        <f t="shared" ref="M7" si="14">CONCATENATE("  ",C7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_sd_card_init, // #5 = Utilities</v>
+      </c>
+      <c r="N7" s="18" t="str">
+        <f>CONCATENATE("  ",H7,", // ",B7)</f>
+        <v xml:space="preserve">  ac_none, // Utilities</v>
+      </c>
+      <c r="O7" s="18" t="str">
+        <f t="shared" ref="O7" si="15">CONCATENATE("  ",F7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -47, // #5 = Utilities</v>
+      </c>
+      <c r="P7" s="17"/>
+    </row>
+    <row r="8" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="5" t="str">
+        <f>G42</f>
+        <v>m_kbd_driver</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="12" t="str">
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(B8," ","_")))</f>
+        <v>m_keyboard</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="I8" s="18" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  m_keyboard, // #5 = Keyboard</v>
-      </c>
-      <c r="J7" s="1" t="str">
+        <v xml:space="preserve">  m_keyboard, // #6 = Keyboard</v>
+      </c>
+      <c r="J8" s="1" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  { "Keyboard" },  // #5 </v>
-      </c>
-      <c r="K7" s="18" t="str">
+        <v xml:space="preserve">  { "Keyboard" },  // #6 </v>
+      </c>
+      <c r="K8" s="18" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  0, // #5 = Keyboard</v>
-      </c>
-      <c r="L7" s="18" t="str">
+        <v xml:space="preserve">  0, // #6 = Keyboard</v>
+      </c>
+      <c r="L8" s="18" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">  0, // #5 = Keyboard</v>
-      </c>
-      <c r="M7" s="18" t="str">
+        <v xml:space="preserve">  0, // #6 = Keyboard</v>
+      </c>
+      <c r="M8" s="18" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">  m_kbd_driver, // #5 = Keyboard</v>
-      </c>
-      <c r="N7" s="18" t="str">
+        <v xml:space="preserve">  m_kbd_driver, // #6 = Keyboard</v>
+      </c>
+      <c r="N8" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // Keyboard</v>
       </c>
-      <c r="O7" s="18" t="str">
+      <c r="O8" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #5 = Keyboard</v>
-      </c>
-      <c r="P7" s="13"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
-      <c r="B8" s="1" t="s">
+        <v xml:space="preserve">  0, // #6 = Keyboard</v>
+      </c>
+      <c r="P8" s="13"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <f t="shared" si="6"/>
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
+      <c r="C9" s="1">
+        <v>0</v>
+      </c>
+      <c r="D9" s="1">
         <v>-1</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E9" s="1">
         <v>31</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F9" s="1">
         <v>-1</v>
       </c>
-      <c r="G8" s="12" t="str">
+      <c r="G9" s="12" t="str">
         <f t="shared" si="7"/>
         <v>m_pitchwheel_pot</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H9" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I8" s="18" t="str">
+      <c r="I9" s="18" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  m_pitchwheel_pot, // #6 = Pitchwheel Pot</v>
-      </c>
-      <c r="J8" s="1" t="str">
+        <v xml:space="preserve">  m_pitchwheel_pot, // #7 = Pitchwheel Pot</v>
+      </c>
+      <c r="J9" s="1" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  { "Pitchwheel Pot" },  // #6 </v>
-      </c>
-      <c r="K8" s="18" t="str">
+        <v xml:space="preserve">  { "Pitchwheel Pot" },  // #7 </v>
+      </c>
+      <c r="K9" s="18" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  -1, // #6 = Pitchwheel Pot</v>
-      </c>
-      <c r="L8" s="18" t="str">
+        <v xml:space="preserve">  -1, // #7 = Pitchwheel Pot</v>
+      </c>
+      <c r="L9" s="18" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">  31, // #6 = Pitchwheel Pot</v>
-      </c>
-      <c r="M8" s="18" t="str">
+        <v xml:space="preserve">  31, // #7 = Pitchwheel Pot</v>
+      </c>
+      <c r="M9" s="18" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">  0, // #6 = Pitchwheel Pot</v>
-      </c>
-      <c r="N8" s="18" t="str">
+        <v xml:space="preserve">  0, // #7 = Pitchwheel Pot</v>
+      </c>
+      <c r="N9" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // Pitchwheel Pot</v>
       </c>
-      <c r="O8" s="18" t="str">
+      <c r="O9" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  -1, // #6 = Pitchwheel Pot</v>
-      </c>
-      <c r="P8" s="13"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <f t="shared" si="6"/>
-        <v>7</v>
-      </c>
-      <c r="B9" s="22" t="s">
+        <v xml:space="preserve">  -1, // #7 = Pitchwheel Pot</v>
+      </c>
+      <c r="P9" s="13"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>195</v>
       </c>
-      <c r="C9" s="22">
-        <v>0</v>
-      </c>
-      <c r="D9" s="22">
-        <v>0</v>
-      </c>
-      <c r="E9" s="22">
-        <v>0</v>
-      </c>
-      <c r="F9" s="22">
-        <v>0</v>
-      </c>
-      <c r="G9" s="34" t="s">
+      <c r="C10" s="22">
+        <v>0</v>
+      </c>
+      <c r="D10" s="22">
+        <v>0</v>
+      </c>
+      <c r="E10" s="22">
+        <v>0</v>
+      </c>
+      <c r="F10" s="22">
+        <v>0</v>
+      </c>
+      <c r="G10" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H10" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I9" s="26" t="str">
+      <c r="I10" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  m_end, // #7 = End</v>
-      </c>
-      <c r="J9" s="22" t="str">
+        <v xml:space="preserve">  m_end, // #8 = End</v>
+      </c>
+      <c r="J10" s="22" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve">  { "End" },  // #7 </v>
-      </c>
-      <c r="K9" s="26" t="str">
+        <v xml:space="preserve">  { "End" },  // #8 </v>
+      </c>
+      <c r="K10" s="26" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  0, // #7 = End</v>
-      </c>
-      <c r="L9" s="26" t="str">
+        <v xml:space="preserve">  0, // #8 = End</v>
+      </c>
+      <c r="L10" s="26" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve">  0, // #7 = End</v>
-      </c>
-      <c r="M9" s="26" t="str">
+        <v xml:space="preserve">  0, // #8 = End</v>
+      </c>
+      <c r="M10" s="26" t="str">
         <f t="shared" si="4"/>
-        <v xml:space="preserve">  0, // #7 = End</v>
-      </c>
-      <c r="N9" s="18" t="str">
+        <v xml:space="preserve">  0, // #8 = End</v>
+      </c>
+      <c r="N10" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // End</v>
       </c>
-      <c r="O9" s="26" t="str">
+      <c r="O10" s="26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #7 = End</v>
-      </c>
-      <c r="P9" s="13"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <f t="shared" si="6"/>
-        <v>8</v>
-      </c>
-      <c r="B10" s="35" t="s">
+        <v xml:space="preserve">  0, // #8 = End</v>
+      </c>
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <f t="shared" si="6"/>
+        <v>9</v>
+      </c>
+      <c r="B11" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="12">
-        <v>0</v>
-      </c>
-      <c r="E10" s="12">
+      <c r="C11" s="1">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0</v>
+      </c>
+      <c r="E11" s="12">
         <v>127</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F11" s="12">
         <v>127</v>
       </c>
-      <c r="G10" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B10,"/","")," ","_")))</f>
+      <c r="G11" s="12" t="str">
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B11,"/","")," ","_")))</f>
         <v>m_upper_db_16</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H11" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I10" s="18" t="str">
-        <f t="shared" ref="I10" si="10">CONCATENATE("  ",G10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_16, // #8 = Upper DB 16</v>
-      </c>
-      <c r="J10" s="1" t="str">
-        <f t="shared" ref="J10" si="11">CONCATENATE("  { """,B10,""" },  // #",A10," ",IF(C10&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 16" },  // #8 </v>
-      </c>
-      <c r="K10" s="18" t="str">
-        <f t="shared" ref="K10" si="12">CONCATENATE("  ",D10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #8 = Upper DB 16</v>
-      </c>
-      <c r="L10" s="18" t="str">
-        <f t="shared" ref="L10" si="13">CONCATENATE("  ",E10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #8 = Upper DB 16</v>
-      </c>
-      <c r="M10" s="18" t="str">
-        <f t="shared" ref="M10" si="14">CONCATENATE("  ",C10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #8 = Upper DB 16</v>
-      </c>
-      <c r="N10" s="18" t="str">
+      <c r="I11" s="18" t="str">
+        <f t="shared" ref="I11" si="16">CONCATENATE("  ",G11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_upper_db_16, // #9 = Upper DB 16</v>
+      </c>
+      <c r="J11" s="1" t="str">
+        <f t="shared" ref="J11" si="17">CONCATENATE("  { """,B11,""" },  // #",A11," ",IF(C11&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Upper DB 16" },  // #9 </v>
+      </c>
+      <c r="K11" s="18" t="str">
+        <f t="shared" ref="K11" si="18">CONCATENATE("  ",D11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #9 = Upper DB 16</v>
+      </c>
+      <c r="L11" s="18" t="str">
+        <f t="shared" ref="L11" si="19">CONCATENATE("  ",E11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  127, // #9 = Upper DB 16</v>
+      </c>
+      <c r="M11" s="18" t="str">
+        <f t="shared" ref="M11" si="20">CONCATENATE("  ",C11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #9 = Upper DB 16</v>
+      </c>
+      <c r="N11" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 16</v>
       </c>
-      <c r="O10" s="18" t="str">
+      <c r="O11" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #8 = Upper DB 16</v>
-      </c>
-      <c r="P10" s="13"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <f t="shared" si="6"/>
-        <v>9</v>
-      </c>
-      <c r="B11" s="29" t="s">
+        <v xml:space="preserve">  127, // #9 = Upper DB 16</v>
+      </c>
+      <c r="P11" s="13"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <f t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="B12" s="29" t="s">
         <v>176</v>
       </c>
-      <c r="C11" s="1">
-        <v>0</v>
-      </c>
-      <c r="D11" s="12">
-        <v>0</v>
-      </c>
-      <c r="E11" s="12">
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="12">
+        <v>0</v>
+      </c>
+      <c r="E12" s="12">
         <v>127</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F12" s="12">
         <v>127</v>
       </c>
-      <c r="G11" s="12" t="str">
-        <f t="shared" ref="G11:G18" si="15">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B11,"/","")," ","_")))</f>
+      <c r="G12" s="12" t="str">
+        <f t="shared" ref="G12:G19" si="21">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B12,"/","")," ","_")))</f>
         <v>m_upper_db_5_13</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H12" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I11" s="18" t="str">
-        <f t="shared" ref="I11:I18" si="16">CONCATENATE("  ",G11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_5_13, // #9 = Upper DB 5 1/3</v>
-      </c>
-      <c r="J11" s="1" t="str">
-        <f t="shared" ref="J11:J18" si="17">CONCATENATE("  { """,B11,""" },  // #",A11," ",IF(C11&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 5 1/3" },  // #9 </v>
-      </c>
-      <c r="K11" s="18" t="str">
-        <f t="shared" ref="K11:K18" si="18">CONCATENATE("  ",D11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #9 = Upper DB 5 1/3</v>
-      </c>
-      <c r="L11" s="18" t="str">
-        <f t="shared" ref="L11:L18" si="19">CONCATENATE("  ",E11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #9 = Upper DB 5 1/3</v>
-      </c>
-      <c r="M11" s="18" t="str">
-        <f t="shared" ref="M11:M18" si="20">CONCATENATE("  ",C11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #9 = Upper DB 5 1/3</v>
-      </c>
-      <c r="N11" s="18" t="str">
+      <c r="I12" s="18" t="str">
+        <f t="shared" ref="I12:I19" si="22">CONCATENATE("  ",G12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_upper_db_5_13, // #10 = Upper DB 5 1/3</v>
+      </c>
+      <c r="J12" s="1" t="str">
+        <f t="shared" ref="J12:J19" si="23">CONCATENATE("  { """,B12,""" },  // #",A12," ",IF(C12&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Upper DB 5 1/3" },  // #10 </v>
+      </c>
+      <c r="K12" s="18" t="str">
+        <f t="shared" ref="K12:K19" si="24">CONCATENATE("  ",D12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #10 = Upper DB 5 1/3</v>
+      </c>
+      <c r="L12" s="18" t="str">
+        <f t="shared" ref="L12:L19" si="25">CONCATENATE("  ",E12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  127, // #10 = Upper DB 5 1/3</v>
+      </c>
+      <c r="M12" s="18" t="str">
+        <f t="shared" ref="M12:M19" si="26">CONCATENATE("  ",C12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #10 = Upper DB 5 1/3</v>
+      </c>
+      <c r="N12" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 5 1/3</v>
       </c>
-      <c r="O11" s="18" t="str">
+      <c r="O12" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #9 = Upper DB 5 1/3</v>
-      </c>
-      <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <f t="shared" si="6"/>
-        <v>10</v>
-      </c>
-      <c r="B12" s="29" t="s">
+        <v xml:space="preserve">  127, // #10 = Upper DB 5 1/3</v>
+      </c>
+      <c r="P12" s="13"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <f t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="B13" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="C12" s="1">
-        <v>0</v>
-      </c>
-      <c r="D12" s="12">
-        <v>0</v>
-      </c>
-      <c r="E12" s="12">
+      <c r="C13" s="1">
+        <v>0</v>
+      </c>
+      <c r="D13" s="12">
+        <v>0</v>
+      </c>
+      <c r="E13" s="12">
         <v>127</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F13" s="12">
         <v>127</v>
       </c>
-      <c r="G12" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="G13" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_8</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H13" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I12" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_8, // #10 = Upper DB 8</v>
-      </c>
-      <c r="J12" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 8" },  // #10 </v>
-      </c>
-      <c r="K12" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #10 = Upper DB 8</v>
-      </c>
-      <c r="L12" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #10 = Upper DB 8</v>
-      </c>
-      <c r="M12" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #10 = Upper DB 8</v>
-      </c>
-      <c r="N12" s="18" t="str">
+      <c r="I13" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_8, // #11 = Upper DB 8</v>
+      </c>
+      <c r="J13" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 8" },  // #11 </v>
+      </c>
+      <c r="K13" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #11 = Upper DB 8</v>
+      </c>
+      <c r="L13" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #11 = Upper DB 8</v>
+      </c>
+      <c r="M13" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #11 = Upper DB 8</v>
+      </c>
+      <c r="N13" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 8</v>
       </c>
-      <c r="O12" s="18" t="str">
+      <c r="O13" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #10 = Upper DB 8</v>
-      </c>
-      <c r="P12" s="13"/>
-    </row>
-    <row r="13" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
-        <f t="shared" si="6"/>
-        <v>11</v>
-      </c>
-      <c r="B13" s="29" t="s">
+        <v xml:space="preserve">  127, // #11 = Upper DB 8</v>
+      </c>
+      <c r="P13" s="13"/>
+    </row>
+    <row r="14" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="B14" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="C13" s="1">
-        <v>0</v>
-      </c>
-      <c r="D13" s="12">
-        <v>0</v>
-      </c>
-      <c r="E13" s="12">
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="12">
+        <v>0</v>
+      </c>
+      <c r="E14" s="12">
         <v>127</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F14" s="12">
         <v>50</v>
       </c>
-      <c r="G13" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="G14" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_4</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="H14" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I13" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_4, // #11 = Upper DB 4</v>
-      </c>
-      <c r="J13" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 4" },  // #11 </v>
-      </c>
-      <c r="K13" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #11 = Upper DB 4</v>
-      </c>
-      <c r="L13" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #11 = Upper DB 4</v>
-      </c>
-      <c r="M13" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #11 = Upper DB 4</v>
-      </c>
-      <c r="N13" s="18" t="str">
+      <c r="I14" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_4, // #12 = Upper DB 4</v>
+      </c>
+      <c r="J14" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 4" },  // #12 </v>
+      </c>
+      <c r="K14" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #12 = Upper DB 4</v>
+      </c>
+      <c r="L14" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #12 = Upper DB 4</v>
+      </c>
+      <c r="M14" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #12 = Upper DB 4</v>
+      </c>
+      <c r="N14" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 4</v>
       </c>
-      <c r="O13" s="18" t="str">
+      <c r="O14" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  50, // #11 = Upper DB 4</v>
-      </c>
-      <c r="P13" s="13"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
-        <f t="shared" si="6"/>
-        <v>12</v>
-      </c>
-      <c r="B14" s="29" t="s">
+        <v xml:space="preserve">  50, // #12 = Upper DB 4</v>
+      </c>
+      <c r="P14" s="13"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="B15" s="29" t="s">
         <v>179</v>
       </c>
-      <c r="C14" s="1">
-        <v>0</v>
-      </c>
-      <c r="D14" s="12">
-        <v>0</v>
-      </c>
-      <c r="E14" s="12">
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12">
+        <v>0</v>
+      </c>
+      <c r="E15" s="12">
         <v>127</v>
       </c>
-      <c r="F14" s="12">
-        <v>0</v>
-      </c>
-      <c r="G14" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="F15" s="12">
+        <v>0</v>
+      </c>
+      <c r="G15" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_2_23</v>
       </c>
-      <c r="H14" s="12" t="s">
+      <c r="H15" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I14" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_2_23, // #12 = Upper DB 2 2/3</v>
-      </c>
-      <c r="J14" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 2 2/3" },  // #12 </v>
-      </c>
-      <c r="K14" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #12 = Upper DB 2 2/3</v>
-      </c>
-      <c r="L14" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #12 = Upper DB 2 2/3</v>
-      </c>
-      <c r="M14" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #12 = Upper DB 2 2/3</v>
-      </c>
-      <c r="N14" s="18" t="str">
+      <c r="I15" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_2_23, // #13 = Upper DB 2 2/3</v>
+      </c>
+      <c r="J15" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 2 2/3" },  // #13 </v>
+      </c>
+      <c r="K15" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #13 = Upper DB 2 2/3</v>
+      </c>
+      <c r="L15" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #13 = Upper DB 2 2/3</v>
+      </c>
+      <c r="M15" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #13 = Upper DB 2 2/3</v>
+      </c>
+      <c r="N15" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 2 2/3</v>
       </c>
-      <c r="O14" s="18" t="str">
+      <c r="O15" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #12 = Upper DB 2 2/3</v>
-      </c>
-      <c r="P14" s="13"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <f t="shared" si="6"/>
-        <v>13</v>
-      </c>
-      <c r="B15" s="29" t="s">
+        <v xml:space="preserve">  0, // #13 = Upper DB 2 2/3</v>
+      </c>
+      <c r="P15" s="13"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <f t="shared" si="6"/>
+        <v>14</v>
+      </c>
+      <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
-      <c r="C15" s="1">
-        <v>0</v>
-      </c>
-      <c r="D15" s="12">
-        <v>0</v>
-      </c>
-      <c r="E15" s="12">
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12">
+        <v>0</v>
+      </c>
+      <c r="E16" s="12">
         <v>127</v>
       </c>
-      <c r="F15" s="12">
-        <v>0</v>
-      </c>
-      <c r="G15" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="F16" s="12">
+        <v>0</v>
+      </c>
+      <c r="G16" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_2</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="H16" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I15" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_2, // #13 = Upper DB 2</v>
-      </c>
-      <c r="J15" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 2" },  // #13 </v>
-      </c>
-      <c r="K15" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #13 = Upper DB 2</v>
-      </c>
-      <c r="L15" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #13 = Upper DB 2</v>
-      </c>
-      <c r="M15" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #13 = Upper DB 2</v>
-      </c>
-      <c r="N15" s="18" t="str">
+      <c r="I16" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_2, // #14 = Upper DB 2</v>
+      </c>
+      <c r="J16" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 2" },  // #14 </v>
+      </c>
+      <c r="K16" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #14 = Upper DB 2</v>
+      </c>
+      <c r="L16" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #14 = Upper DB 2</v>
+      </c>
+      <c r="M16" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #14 = Upper DB 2</v>
+      </c>
+      <c r="N16" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 2</v>
       </c>
-      <c r="O15" s="18" t="str">
+      <c r="O16" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #13 = Upper DB 2</v>
-      </c>
-      <c r="P15" s="13"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
-        <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="B16" s="29" t="s">
+        <v xml:space="preserve">  0, // #14 = Upper DB 2</v>
+      </c>
+      <c r="P16" s="13"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
+      <c r="B17" s="29" t="s">
         <v>181</v>
       </c>
-      <c r="C16" s="1">
-        <v>0</v>
-      </c>
-      <c r="D16" s="12">
-        <v>0</v>
-      </c>
-      <c r="E16" s="12">
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="12">
+        <v>0</v>
+      </c>
+      <c r="E17" s="12">
         <v>127</v>
       </c>
-      <c r="F16" s="12">
-        <v>0</v>
-      </c>
-      <c r="G16" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="F17" s="12">
+        <v>0</v>
+      </c>
+      <c r="G17" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_1_35</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H17" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I16" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_1_35, // #14 = Upper DB 1 3/5</v>
-      </c>
-      <c r="J16" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 1 3/5" },  // #14 </v>
-      </c>
-      <c r="K16" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #14 = Upper DB 1 3/5</v>
-      </c>
-      <c r="L16" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #14 = Upper DB 1 3/5</v>
-      </c>
-      <c r="M16" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #14 = Upper DB 1 3/5</v>
-      </c>
-      <c r="N16" s="18" t="str">
+      <c r="I17" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_1_35, // #15 = Upper DB 1 3/5</v>
+      </c>
+      <c r="J17" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 1 3/5" },  // #15 </v>
+      </c>
+      <c r="K17" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #15 = Upper DB 1 3/5</v>
+      </c>
+      <c r="L17" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #15 = Upper DB 1 3/5</v>
+      </c>
+      <c r="M17" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #15 = Upper DB 1 3/5</v>
+      </c>
+      <c r="N17" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 1 3/5</v>
       </c>
-      <c r="O16" s="18" t="str">
+      <c r="O17" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #14 = Upper DB 1 3/5</v>
-      </c>
-      <c r="P16" s="13"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
-        <f t="shared" si="6"/>
-        <v>15</v>
-      </c>
-      <c r="B17" s="29" t="s">
+        <v xml:space="preserve">  0, // #15 = Upper DB 1 3/5</v>
+      </c>
+      <c r="P17" s="13"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="B18" s="29" t="s">
         <v>182</v>
       </c>
-      <c r="C17" s="1">
-        <v>0</v>
-      </c>
-      <c r="D17" s="12">
-        <v>0</v>
-      </c>
-      <c r="E17" s="12">
+      <c r="C18" s="1">
+        <v>0</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0</v>
+      </c>
+      <c r="E18" s="12">
         <v>127</v>
       </c>
-      <c r="F17" s="12">
-        <v>0</v>
-      </c>
-      <c r="G17" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="F18" s="12">
+        <v>0</v>
+      </c>
+      <c r="G18" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_1_13</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H18" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I17" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_1_13, // #15 = Upper DB 1 1/3</v>
-      </c>
-      <c r="J17" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 1 1/3" },  // #15 </v>
-      </c>
-      <c r="K17" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #15 = Upper DB 1 1/3</v>
-      </c>
-      <c r="L17" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #15 = Upper DB 1 1/3</v>
-      </c>
-      <c r="M17" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #15 = Upper DB 1 1/3</v>
-      </c>
-      <c r="N17" s="18" t="str">
+      <c r="I18" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_1_13, // #16 = Upper DB 1 1/3</v>
+      </c>
+      <c r="J18" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 1 1/3" },  // #16 </v>
+      </c>
+      <c r="K18" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #16 = Upper DB 1 1/3</v>
+      </c>
+      <c r="L18" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #16 = Upper DB 1 1/3</v>
+      </c>
+      <c r="M18" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #16 = Upper DB 1 1/3</v>
+      </c>
+      <c r="N18" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 1 1/3</v>
       </c>
-      <c r="O17" s="18" t="str">
+      <c r="O18" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #15 = Upper DB 1 1/3</v>
-      </c>
-      <c r="P17" s="13"/>
-    </row>
-    <row r="18" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
-        <f t="shared" si="6"/>
-        <v>16</v>
-      </c>
-      <c r="B18" s="29" t="s">
+        <v xml:space="preserve">  0, // #16 = Upper DB 1 1/3</v>
+      </c>
+      <c r="P18" s="13"/>
+    </row>
+    <row r="19" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="B19" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="1">
-        <v>0</v>
-      </c>
-      <c r="D18" s="12">
-        <v>0</v>
-      </c>
-      <c r="E18" s="12">
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0</v>
+      </c>
+      <c r="E19" s="12">
         <v>127</v>
       </c>
-      <c r="F18" s="12">
-        <v>0</v>
-      </c>
-      <c r="G18" s="12" t="str">
-        <f t="shared" si="15"/>
+      <c r="F19" s="12">
+        <v>0</v>
+      </c>
+      <c r="G19" s="12" t="str">
+        <f t="shared" si="21"/>
         <v>m_upper_db_1</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H19" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="I18" s="18" t="str">
-        <f t="shared" si="16"/>
-        <v xml:space="preserve">  m_upper_db_1, // #16 = Upper DB 1</v>
-      </c>
-      <c r="J18" s="1" t="str">
-        <f t="shared" si="17"/>
-        <v xml:space="preserve">  { "Upper DB 1" },  // #16 </v>
-      </c>
-      <c r="K18" s="18" t="str">
-        <f t="shared" si="18"/>
-        <v xml:space="preserve">  0, // #16 = Upper DB 1</v>
-      </c>
-      <c r="L18" s="18" t="str">
-        <f t="shared" si="19"/>
-        <v xml:space="preserve">  127, // #16 = Upper DB 1</v>
-      </c>
-      <c r="M18" s="18" t="str">
-        <f t="shared" si="20"/>
-        <v xml:space="preserve">  0, // #16 = Upper DB 1</v>
-      </c>
-      <c r="N18" s="18" t="str">
+      <c r="I19" s="18" t="str">
+        <f t="shared" si="22"/>
+        <v xml:space="preserve">  m_upper_db_1, // #17 = Upper DB 1</v>
+      </c>
+      <c r="J19" s="1" t="str">
+        <f t="shared" si="23"/>
+        <v xml:space="preserve">  { "Upper DB 1" },  // #17 </v>
+      </c>
+      <c r="K19" s="18" t="str">
+        <f t="shared" si="24"/>
+        <v xml:space="preserve">  0, // #17 = Upper DB 1</v>
+      </c>
+      <c r="L19" s="18" t="str">
+        <f t="shared" si="25"/>
+        <v xml:space="preserve">  127, // #17 = Upper DB 1</v>
+      </c>
+      <c r="M19" s="18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  0, // #17 = Upper DB 1</v>
+      </c>
+      <c r="N19" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_upper_db, // Upper DB 1</v>
       </c>
-      <c r="O18" s="18" t="str">
+      <c r="O19" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #16 = Upper DB 1</v>
-      </c>
-      <c r="P18" s="13"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
-        <f t="shared" si="6"/>
-        <v>17</v>
-      </c>
-      <c r="B19" s="22" t="s">
+        <v xml:space="preserve">  0, // #17 = Upper DB 1</v>
+      </c>
+      <c r="P19" s="13"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C20" s="22">
         <v>-1</v>
       </c>
-      <c r="D19" s="22">
-        <v>0</v>
-      </c>
-      <c r="E19" s="22">
-        <v>0</v>
-      </c>
-      <c r="F19" s="22">
-        <v>0</v>
-      </c>
-      <c r="G19" s="26" t="str">
-        <f>CONCATENATE("m_back_",A19)</f>
-        <v>m_back_17</v>
-      </c>
-      <c r="H19" s="12" t="s">
+      <c r="D20" s="22">
+        <v>0</v>
+      </c>
+      <c r="E20" s="22">
+        <v>0</v>
+      </c>
+      <c r="F20" s="22">
+        <v>0</v>
+      </c>
+      <c r="G20" s="26" t="str">
+        <f>CONCATENATE("m_back_",A20)</f>
+        <v>m_back_18</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I19" s="26" t="str">
-        <f t="shared" ref="I19:I28" si="21">CONCATENATE("  ",G19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_17, // #17 = Upper DB EXIT </v>
-      </c>
-      <c r="J19" s="22" t="str">
-        <f t="shared" ref="J19:J28" si="22">CONCATENATE("  { """,B19,""" },  // #",A19," ",IF(C19&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB" },  // #17  EXIT SUBM</v>
-      </c>
-      <c r="K19" s="26" t="str">
-        <f t="shared" ref="K19:K28" si="23">CONCATENATE("  ",D19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #17 = Upper DB EXIT </v>
-      </c>
-      <c r="L19" s="26" t="str">
-        <f t="shared" ref="L19:L28" si="24">CONCATENATE("  ",E19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #17 = Upper DB EXIT </v>
-      </c>
-      <c r="M19" s="26" t="str">
-        <f t="shared" ref="M19:M28" si="25">CONCATENATE("  ",C19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #17 = Upper DB EXIT </v>
-      </c>
-      <c r="N19" s="18" t="str">
+      <c r="I20" s="26" t="str">
+        <f t="shared" ref="I20:I29" si="27">CONCATENATE("  ",G20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_back_18, // #18 = Upper DB EXIT </v>
+      </c>
+      <c r="J20" s="22" t="str">
+        <f t="shared" ref="J20:J29" si="28">CONCATENATE("  { """,B20,""" },  // #",A20," ",IF(C20&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Upper DB" },  // #18  EXIT SUBM</v>
+      </c>
+      <c r="K20" s="26" t="str">
+        <f t="shared" ref="K20:K29" si="29">CONCATENATE("  ",D20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #18 = Upper DB EXIT </v>
+      </c>
+      <c r="L20" s="26" t="str">
+        <f t="shared" ref="L20:L29" si="30">CONCATENATE("  ",E20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #18 = Upper DB EXIT </v>
+      </c>
+      <c r="M20" s="26" t="str">
+        <f t="shared" ref="M20:M29" si="31">CONCATENATE("  ",C20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -1, // #18 = Upper DB EXIT </v>
+      </c>
+      <c r="N20" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // Upper DB</v>
       </c>
-      <c r="O19" s="26" t="str">
+      <c r="O20" s="26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #17 = Upper DB EXIT </v>
-      </c>
-      <c r="P19" s="13"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
-        <f t="shared" si="6"/>
-        <v>18</v>
-      </c>
-      <c r="B20" s="36" t="s">
+        <v xml:space="preserve">  0, // #18 = Upper DB EXIT </v>
+      </c>
+      <c r="P20" s="13"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <f t="shared" si="6"/>
+        <v>19</v>
+      </c>
+      <c r="B21" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="1">
-        <v>0</v>
-      </c>
-      <c r="D20" s="12">
-        <v>0</v>
-      </c>
-      <c r="E20" s="12">
+      <c r="C21" s="1">
+        <v>0</v>
+      </c>
+      <c r="D21" s="12">
+        <v>0</v>
+      </c>
+      <c r="E21" s="12">
         <v>127</v>
       </c>
-      <c r="F20" s="12">
-        <v>0</v>
-      </c>
-      <c r="G20" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B20,"/","")," ","_")))</f>
+      <c r="F21" s="12">
+        <v>0</v>
+      </c>
+      <c r="G21" s="12" t="str">
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B21,"/","")," ","_")))</f>
         <v>m_lower_db_16</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H21" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I20" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_16, // #18 = Lower DB 16</v>
-      </c>
-      <c r="J20" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 16" },  // #18 </v>
-      </c>
-      <c r="K20" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #18 = Lower DB 16</v>
-      </c>
-      <c r="L20" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #18 = Lower DB 16</v>
-      </c>
-      <c r="M20" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #18 = Lower DB 16</v>
-      </c>
-      <c r="N20" s="18" t="str">
+      <c r="I21" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_16, // #19 = Lower DB 16</v>
+      </c>
+      <c r="J21" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 16" },  // #19 </v>
+      </c>
+      <c r="K21" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #19 = Lower DB 16</v>
+      </c>
+      <c r="L21" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #19 = Lower DB 16</v>
+      </c>
+      <c r="M21" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #19 = Lower DB 16</v>
+      </c>
+      <c r="N21" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 16</v>
       </c>
-      <c r="O20" s="18" t="str">
+      <c r="O21" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #18 = Lower DB 16</v>
-      </c>
-      <c r="P20" s="13"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
-        <f t="shared" si="6"/>
-        <v>19</v>
-      </c>
-      <c r="B21" s="30" t="s">
+        <v xml:space="preserve">  0, // #19 = Lower DB 16</v>
+      </c>
+      <c r="P21" s="13"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="B22" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="C21" s="1">
-        <v>0</v>
-      </c>
-      <c r="D21" s="12">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12">
+      <c r="C22" s="1">
+        <v>0</v>
+      </c>
+      <c r="D22" s="12">
+        <v>0</v>
+      </c>
+      <c r="E22" s="12">
         <v>127</v>
       </c>
-      <c r="F21" s="12">
-        <v>0</v>
-      </c>
-      <c r="G21" s="12" t="str">
-        <f t="shared" ref="G21:G28" si="26">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B21,"/","")," ","_")))</f>
+      <c r="F22" s="12">
+        <v>0</v>
+      </c>
+      <c r="G22" s="12" t="str">
+        <f t="shared" ref="G22:G29" si="32">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B22,"/","")," ","_")))</f>
         <v>m_lower_db_5_13</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="H22" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I21" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_5_13, // #19 = Lower DB 5 1/3</v>
-      </c>
-      <c r="J21" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 5 1/3" },  // #19 </v>
-      </c>
-      <c r="K21" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #19 = Lower DB 5 1/3</v>
-      </c>
-      <c r="L21" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #19 = Lower DB 5 1/3</v>
-      </c>
-      <c r="M21" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #19 = Lower DB 5 1/3</v>
-      </c>
-      <c r="N21" s="18" t="str">
+      <c r="I22" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_5_13, // #20 = Lower DB 5 1/3</v>
+      </c>
+      <c r="J22" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 5 1/3" },  // #20 </v>
+      </c>
+      <c r="K22" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #20 = Lower DB 5 1/3</v>
+      </c>
+      <c r="L22" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #20 = Lower DB 5 1/3</v>
+      </c>
+      <c r="M22" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #20 = Lower DB 5 1/3</v>
+      </c>
+      <c r="N22" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 5 1/3</v>
       </c>
-      <c r="O21" s="18" t="str">
+      <c r="O22" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #19 = Lower DB 5 1/3</v>
-      </c>
-      <c r="P21" s="13"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
-        <f t="shared" si="6"/>
-        <v>20</v>
-      </c>
-      <c r="B22" s="30" t="s">
+        <v xml:space="preserve">  0, // #20 = Lower DB 5 1/3</v>
+      </c>
+      <c r="P22" s="13"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <f t="shared" si="6"/>
+        <v>21</v>
+      </c>
+      <c r="B23" s="30" t="s">
         <v>186</v>
       </c>
-      <c r="C22" s="1">
-        <v>0</v>
-      </c>
-      <c r="D22" s="12">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12">
+      <c r="C23" s="1">
+        <v>0</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
+      </c>
+      <c r="E23" s="12">
         <v>127</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F23" s="12">
         <v>127</v>
       </c>
-      <c r="G22" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="G23" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_8</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H23" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I22" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_8, // #20 = Lower DB 8</v>
-      </c>
-      <c r="J22" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 8" },  // #20 </v>
-      </c>
-      <c r="K22" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #20 = Lower DB 8</v>
-      </c>
-      <c r="L22" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #20 = Lower DB 8</v>
-      </c>
-      <c r="M22" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #20 = Lower DB 8</v>
-      </c>
-      <c r="N22" s="18" t="str">
+      <c r="I23" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_8, // #21 = Lower DB 8</v>
+      </c>
+      <c r="J23" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 8" },  // #21 </v>
+      </c>
+      <c r="K23" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #21 = Lower DB 8</v>
+      </c>
+      <c r="L23" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #21 = Lower DB 8</v>
+      </c>
+      <c r="M23" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #21 = Lower DB 8</v>
+      </c>
+      <c r="N23" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 8</v>
       </c>
-      <c r="O22" s="18" t="str">
+      <c r="O23" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #20 = Lower DB 8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
-        <f t="shared" si="6"/>
-        <v>21</v>
-      </c>
-      <c r="B23" s="30" t="s">
+        <v xml:space="preserve">  127, // #21 = Lower DB 8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <f t="shared" si="6"/>
+        <v>22</v>
+      </c>
+      <c r="B24" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="C23" s="1">
-        <v>0</v>
-      </c>
-      <c r="D23" s="12">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12">
+      <c r="C24" s="1">
+        <v>0</v>
+      </c>
+      <c r="D24" s="12">
+        <v>0</v>
+      </c>
+      <c r="E24" s="12">
         <v>127</v>
       </c>
-      <c r="F23" s="12">
+      <c r="F24" s="12">
         <v>127</v>
       </c>
-      <c r="G23" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="G24" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_4</v>
       </c>
-      <c r="H23" s="12" t="s">
+      <c r="H24" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I23" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_4, // #21 = Lower DB 4</v>
-      </c>
-      <c r="J23" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 4" },  // #21 </v>
-      </c>
-      <c r="K23" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #21 = Lower DB 4</v>
-      </c>
-      <c r="L23" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #21 = Lower DB 4</v>
-      </c>
-      <c r="M23" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #21 = Lower DB 4</v>
-      </c>
-      <c r="N23" s="18" t="str">
+      <c r="I24" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_4, // #22 = Lower DB 4</v>
+      </c>
+      <c r="J24" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 4" },  // #22 </v>
+      </c>
+      <c r="K24" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #22 = Lower DB 4</v>
+      </c>
+      <c r="L24" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #22 = Lower DB 4</v>
+      </c>
+      <c r="M24" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #22 = Lower DB 4</v>
+      </c>
+      <c r="N24" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 4</v>
       </c>
-      <c r="O23" s="18" t="str">
+      <c r="O24" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #21 = Lower DB 4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
-        <f t="shared" si="6"/>
-        <v>22</v>
-      </c>
-      <c r="B24" s="30" t="s">
+        <v xml:space="preserve">  127, // #22 = Lower DB 4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <f t="shared" si="6"/>
+        <v>23</v>
+      </c>
+      <c r="B25" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="C24" s="1">
-        <v>0</v>
-      </c>
-      <c r="D24" s="12">
-        <v>0</v>
-      </c>
-      <c r="E24" s="12">
+      <c r="C25" s="1">
+        <v>0</v>
+      </c>
+      <c r="D25" s="12">
+        <v>0</v>
+      </c>
+      <c r="E25" s="12">
         <v>127</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F25" s="12">
         <v>40</v>
       </c>
-      <c r="G24" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="G25" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_2_23</v>
       </c>
-      <c r="H24" s="12" t="s">
+      <c r="H25" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I24" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_2_23, // #22 = Lower DB 2 2/3</v>
-      </c>
-      <c r="J24" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 2 2/3" },  // #22 </v>
-      </c>
-      <c r="K24" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #22 = Lower DB 2 2/3</v>
-      </c>
-      <c r="L24" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #22 = Lower DB 2 2/3</v>
-      </c>
-      <c r="M24" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #22 = Lower DB 2 2/3</v>
-      </c>
-      <c r="N24" s="18" t="str">
+      <c r="I25" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_2_23, // #23 = Lower DB 2 2/3</v>
+      </c>
+      <c r="J25" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 2 2/3" },  // #23 </v>
+      </c>
+      <c r="K25" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #23 = Lower DB 2 2/3</v>
+      </c>
+      <c r="L25" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #23 = Lower DB 2 2/3</v>
+      </c>
+      <c r="M25" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #23 = Lower DB 2 2/3</v>
+      </c>
+      <c r="N25" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 2 2/3</v>
       </c>
-      <c r="O24" s="18" t="str">
+      <c r="O25" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  40, // #22 = Lower DB 2 2/3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
-        <f t="shared" si="6"/>
-        <v>23</v>
-      </c>
-      <c r="B25" s="30" t="s">
+        <v xml:space="preserve">  40, // #23 = Lower DB 2 2/3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <f t="shared" si="6"/>
+        <v>24</v>
+      </c>
+      <c r="B26" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="C25" s="1">
-        <v>0</v>
-      </c>
-      <c r="D25" s="12">
-        <v>0</v>
-      </c>
-      <c r="E25" s="12">
+      <c r="C26" s="1">
+        <v>0</v>
+      </c>
+      <c r="D26" s="12">
+        <v>0</v>
+      </c>
+      <c r="E26" s="12">
         <v>127</v>
       </c>
-      <c r="F25" s="12">
-        <v>0</v>
-      </c>
-      <c r="G25" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="F26" s="12">
+        <v>0</v>
+      </c>
+      <c r="G26" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_2</v>
       </c>
-      <c r="H25" s="12" t="s">
+      <c r="H26" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I25" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_2, // #23 = Lower DB 2</v>
-      </c>
-      <c r="J25" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 2" },  // #23 </v>
-      </c>
-      <c r="K25" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #23 = Lower DB 2</v>
-      </c>
-      <c r="L25" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #23 = Lower DB 2</v>
-      </c>
-      <c r="M25" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #23 = Lower DB 2</v>
-      </c>
-      <c r="N25" s="18" t="str">
+      <c r="I26" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_2, // #24 = Lower DB 2</v>
+      </c>
+      <c r="J26" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 2" },  // #24 </v>
+      </c>
+      <c r="K26" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #24 = Lower DB 2</v>
+      </c>
+      <c r="L26" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #24 = Lower DB 2</v>
+      </c>
+      <c r="M26" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #24 = Lower DB 2</v>
+      </c>
+      <c r="N26" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 2</v>
       </c>
-      <c r="O25" s="18" t="str">
+      <c r="O26" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #23 = Lower DB 2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
-        <f t="shared" si="6"/>
-        <v>24</v>
-      </c>
-      <c r="B26" s="30" t="s">
+        <v xml:space="preserve">  0, // #24 = Lower DB 2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <f t="shared" si="6"/>
+        <v>25</v>
+      </c>
+      <c r="B27" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="C26" s="1">
-        <v>0</v>
-      </c>
-      <c r="D26" s="12">
-        <v>0</v>
-      </c>
-      <c r="E26" s="12">
+      <c r="C27" s="1">
+        <v>0</v>
+      </c>
+      <c r="D27" s="12">
+        <v>0</v>
+      </c>
+      <c r="E27" s="12">
         <v>127</v>
       </c>
-      <c r="F26" s="12">
-        <v>0</v>
-      </c>
-      <c r="G26" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="F27" s="12">
+        <v>0</v>
+      </c>
+      <c r="G27" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_1_35</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="H27" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I26" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_1_35, // #24 = Lower DB 1 3/5</v>
-      </c>
-      <c r="J26" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 1 3/5" },  // #24 </v>
-      </c>
-      <c r="K26" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #24 = Lower DB 1 3/5</v>
-      </c>
-      <c r="L26" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #24 = Lower DB 1 3/5</v>
-      </c>
-      <c r="M26" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #24 = Lower DB 1 3/5</v>
-      </c>
-      <c r="N26" s="18" t="str">
+      <c r="I27" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_1_35, // #25 = Lower DB 1 3/5</v>
+      </c>
+      <c r="J27" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 1 3/5" },  // #25 </v>
+      </c>
+      <c r="K27" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #25 = Lower DB 1 3/5</v>
+      </c>
+      <c r="L27" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #25 = Lower DB 1 3/5</v>
+      </c>
+      <c r="M27" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #25 = Lower DB 1 3/5</v>
+      </c>
+      <c r="N27" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 1 3/5</v>
       </c>
-      <c r="O26" s="18" t="str">
+      <c r="O27" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #24 = Lower DB 1 3/5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
-        <f t="shared" si="6"/>
-        <v>25</v>
-      </c>
-      <c r="B27" s="30" t="s">
+        <v xml:space="preserve">  0, // #25 = Lower DB 1 3/5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <f t="shared" si="6"/>
+        <v>26</v>
+      </c>
+      <c r="B28" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="C27" s="1">
-        <v>0</v>
-      </c>
-      <c r="D27" s="12">
-        <v>0</v>
-      </c>
-      <c r="E27" s="12">
+      <c r="C28" s="1">
+        <v>0</v>
+      </c>
+      <c r="D28" s="12">
+        <v>0</v>
+      </c>
+      <c r="E28" s="12">
         <v>127</v>
       </c>
-      <c r="F27" s="12">
-        <v>0</v>
-      </c>
-      <c r="G27" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="F28" s="12">
+        <v>0</v>
+      </c>
+      <c r="G28" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_1_13</v>
       </c>
-      <c r="H27" s="12" t="s">
+      <c r="H28" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I27" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_1_13, // #25 = Lower DB 1 1/3</v>
-      </c>
-      <c r="J27" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 1 1/3" },  // #25 </v>
-      </c>
-      <c r="K27" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #25 = Lower DB 1 1/3</v>
-      </c>
-      <c r="L27" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #25 = Lower DB 1 1/3</v>
-      </c>
-      <c r="M27" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #25 = Lower DB 1 1/3</v>
-      </c>
-      <c r="N27" s="18" t="str">
+      <c r="I28" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_1_13, // #26 = Lower DB 1 1/3</v>
+      </c>
+      <c r="J28" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 1 1/3" },  // #26 </v>
+      </c>
+      <c r="K28" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #26 = Lower DB 1 1/3</v>
+      </c>
+      <c r="L28" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #26 = Lower DB 1 1/3</v>
+      </c>
+      <c r="M28" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #26 = Lower DB 1 1/3</v>
+      </c>
+      <c r="N28" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 1 1/3</v>
       </c>
-      <c r="O27" s="18" t="str">
+      <c r="O28" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #25 = Lower DB 1 1/3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
-        <f t="shared" si="6"/>
-        <v>26</v>
-      </c>
-      <c r="B28" s="30" t="s">
+        <v xml:space="preserve">  0, // #26 = Lower DB 1 1/3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <f t="shared" si="6"/>
+        <v>27</v>
+      </c>
+      <c r="B29" s="30" t="s">
         <v>192</v>
       </c>
-      <c r="C28" s="1">
-        <v>0</v>
-      </c>
-      <c r="D28" s="12">
-        <v>0</v>
-      </c>
-      <c r="E28" s="12">
+      <c r="C29" s="1">
+        <v>0</v>
+      </c>
+      <c r="D29" s="12">
+        <v>0</v>
+      </c>
+      <c r="E29" s="12">
         <v>127</v>
       </c>
-      <c r="F28" s="12">
-        <v>0</v>
-      </c>
-      <c r="G28" s="12" t="str">
-        <f t="shared" si="26"/>
+      <c r="F29" s="12">
+        <v>0</v>
+      </c>
+      <c r="G29" s="12" t="str">
+        <f t="shared" si="32"/>
         <v>m_lower_db_1</v>
       </c>
-      <c r="H28" s="12" t="s">
+      <c r="H29" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="I28" s="18" t="str">
-        <f t="shared" si="21"/>
-        <v xml:space="preserve">  m_lower_db_1, // #26 = Lower DB 1</v>
-      </c>
-      <c r="J28" s="1" t="str">
-        <f t="shared" si="22"/>
-        <v xml:space="preserve">  { "Lower DB 1" },  // #26 </v>
-      </c>
-      <c r="K28" s="18" t="str">
-        <f t="shared" si="23"/>
-        <v xml:space="preserve">  0, // #26 = Lower DB 1</v>
-      </c>
-      <c r="L28" s="18" t="str">
-        <f t="shared" si="24"/>
-        <v xml:space="preserve">  127, // #26 = Lower DB 1</v>
-      </c>
-      <c r="M28" s="18" t="str">
-        <f t="shared" si="25"/>
-        <v xml:space="preserve">  0, // #26 = Lower DB 1</v>
-      </c>
-      <c r="N28" s="18" t="str">
+      <c r="I29" s="18" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  m_lower_db_1, // #27 = Lower DB 1</v>
+      </c>
+      <c r="J29" s="1" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  { "Lower DB 1" },  // #27 </v>
+      </c>
+      <c r="K29" s="18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">  0, // #27 = Lower DB 1</v>
+      </c>
+      <c r="L29" s="18" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">  127, // #27 = Lower DB 1</v>
+      </c>
+      <c r="M29" s="18" t="str">
+        <f t="shared" si="31"/>
+        <v xml:space="preserve">  0, // #27 = Lower DB 1</v>
+      </c>
+      <c r="N29" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_lower_db, // Lower DB 1</v>
       </c>
-      <c r="O28" s="18" t="str">
+      <c r="O29" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #26 = Lower DB 1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
-        <f t="shared" si="6"/>
-        <v>27</v>
-      </c>
-      <c r="B29" s="22" t="s">
+        <v xml:space="preserve">  0, // #27 = Lower DB 1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <f t="shared" si="6"/>
+        <v>28</v>
+      </c>
+      <c r="B30" s="22" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="22">
+      <c r="C30" s="22">
         <v>-1</v>
       </c>
-      <c r="D29" s="22">
-        <v>0</v>
-      </c>
-      <c r="E29" s="22">
-        <v>0</v>
-      </c>
-      <c r="F29" s="22">
-        <v>0</v>
-      </c>
-      <c r="G29" s="26" t="str">
-        <f>CONCATENATE("m_back_",A29)</f>
-        <v>m_back_27</v>
-      </c>
-      <c r="H29" s="12" t="s">
+      <c r="D30" s="22">
+        <v>0</v>
+      </c>
+      <c r="E30" s="22">
+        <v>0</v>
+      </c>
+      <c r="F30" s="22">
+        <v>0</v>
+      </c>
+      <c r="G30" s="26" t="str">
+        <f>CONCATENATE("m_back_",A30)</f>
+        <v>m_back_28</v>
+      </c>
+      <c r="H30" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I29" s="26" t="str">
-        <f t="shared" ref="I29:I31" si="27">CONCATENATE("  ",G29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_27, // #27 = Lower DB EXIT </v>
-      </c>
-      <c r="J29" s="22" t="str">
-        <f t="shared" ref="J29:J31" si="28">CONCATENATE("  { """,B29,""" },  // #",A29," ",IF(C29&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB" },  // #27  EXIT SUBM</v>
-      </c>
-      <c r="K29" s="26" t="str">
-        <f t="shared" ref="K29:K31" si="29">CONCATENATE("  ",D29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #27 = Lower DB EXIT </v>
-      </c>
-      <c r="L29" s="26" t="str">
-        <f t="shared" ref="L29:L31" si="30">CONCATENATE("  ",E29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #27 = Lower DB EXIT </v>
-      </c>
-      <c r="M29" s="26" t="str">
-        <f t="shared" ref="M29:M31" si="31">CONCATENATE("  ",C29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #27 = Lower DB EXIT </v>
-      </c>
-      <c r="N29" s="18" t="str">
+      <c r="I30" s="26" t="str">
+        <f t="shared" ref="I30:I32" si="33">CONCATENATE("  ",G30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_back_28, // #28 = Lower DB EXIT </v>
+      </c>
+      <c r="J30" s="22" t="str">
+        <f t="shared" ref="J30:J32" si="34">CONCATENATE("  { """,B30,""" },  // #",A30," ",IF(C30&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Lower DB" },  // #28  EXIT SUBM</v>
+      </c>
+      <c r="K30" s="26" t="str">
+        <f t="shared" ref="K30:K32" si="35">CONCATENATE("  ",D30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #28 = Lower DB EXIT </v>
+      </c>
+      <c r="L30" s="26" t="str">
+        <f t="shared" ref="L30:L32" si="36">CONCATENATE("  ",E30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #28 = Lower DB EXIT </v>
+      </c>
+      <c r="M30" s="26" t="str">
+        <f t="shared" ref="M30:M32" si="37">CONCATENATE("  ",C30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -1, // #28 = Lower DB EXIT </v>
+      </c>
+      <c r="N30" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // Lower DB</v>
       </c>
-      <c r="O29" s="26" t="str">
+      <c r="O30" s="26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #27 = Lower DB EXIT </v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
-        <f t="shared" si="6"/>
-        <v>28</v>
-      </c>
-      <c r="B30" s="37" t="s">
+        <v xml:space="preserve">  0, // #28 = Lower DB EXIT </v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <f t="shared" si="6"/>
+        <v>29</v>
+      </c>
+      <c r="B31" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="C30" s="1">
-        <v>0</v>
-      </c>
-      <c r="D30" s="12">
-        <v>0</v>
-      </c>
-      <c r="E30" s="12">
+      <c r="C31" s="1">
+        <v>0</v>
+      </c>
+      <c r="D31" s="12">
+        <v>0</v>
+      </c>
+      <c r="E31" s="12">
         <v>127</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F31" s="12">
         <v>127</v>
       </c>
-      <c r="G30" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B30,"/","")," ","_")))</f>
+      <c r="G31" s="12" t="str">
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B31,"/","")," ","_")))</f>
         <v>m_pedal_db_16</v>
       </c>
-      <c r="H30" s="12" t="s">
+      <c r="H31" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="I30" s="18" t="str">
-        <f t="shared" si="27"/>
-        <v xml:space="preserve">  m_pedal_db_16, // #28 = Pedal DB 16</v>
-      </c>
-      <c r="J30" s="1" t="str">
-        <f t="shared" si="28"/>
-        <v xml:space="preserve">  { "Pedal DB 16" },  // #28 </v>
-      </c>
-      <c r="K30" s="18" t="str">
-        <f t="shared" si="29"/>
-        <v xml:space="preserve">  0, // #28 = Pedal DB 16</v>
-      </c>
-      <c r="L30" s="18" t="str">
-        <f t="shared" si="30"/>
-        <v xml:space="preserve">  127, // #28 = Pedal DB 16</v>
-      </c>
-      <c r="M30" s="18" t="str">
-        <f t="shared" si="31"/>
-        <v xml:space="preserve">  0, // #28 = Pedal DB 16</v>
-      </c>
-      <c r="N30" s="18" t="str">
+      <c r="I31" s="18" t="str">
+        <f t="shared" si="33"/>
+        <v xml:space="preserve">  m_pedal_db_16, // #29 = Pedal DB 16</v>
+      </c>
+      <c r="J31" s="1" t="str">
+        <f t="shared" si="34"/>
+        <v xml:space="preserve">  { "Pedal DB 16" },  // #29 </v>
+      </c>
+      <c r="K31" s="18" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">  0, // #29 = Pedal DB 16</v>
+      </c>
+      <c r="L31" s="18" t="str">
+        <f t="shared" si="36"/>
+        <v xml:space="preserve">  127, // #29 = Pedal DB 16</v>
+      </c>
+      <c r="M31" s="18" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">  0, // #29 = Pedal DB 16</v>
+      </c>
+      <c r="N31" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_pedal_db, // Pedal DB 16</v>
       </c>
-      <c r="O30" s="18" t="str">
+      <c r="O31" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  127, // #28 = Pedal DB 16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
-        <f t="shared" si="6"/>
-        <v>29</v>
-      </c>
-      <c r="B31" s="31" t="s">
+        <v xml:space="preserve">  127, // #29 = Pedal DB 16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <f t="shared" si="6"/>
+        <v>30</v>
+      </c>
+      <c r="B32" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="C31" s="1">
-        <v>0</v>
-      </c>
-      <c r="D31" s="12">
-        <v>0</v>
-      </c>
-      <c r="E31" s="12">
+      <c r="C32" s="1">
+        <v>0</v>
+      </c>
+      <c r="D32" s="12">
+        <v>0</v>
+      </c>
+      <c r="E32" s="12">
         <v>127</v>
       </c>
-      <c r="F31" s="12">
+      <c r="F32" s="12">
         <v>60</v>
       </c>
-      <c r="G31" s="12" t="str">
-        <f t="shared" ref="G31" si="32">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B31,"/","")," ","_")))</f>
+      <c r="G32" s="12" t="str">
+        <f t="shared" ref="G32" si="38">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B32,"/","")," ","_")))</f>
         <v>m_pedal_db_8</v>
       </c>
-      <c r="H31" s="12" t="s">
+      <c r="H32" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="I31" s="18" t="str">
-        <f t="shared" si="27"/>
-        <v xml:space="preserve">  m_pedal_db_8, // #29 = Pedal DB 8</v>
-      </c>
-      <c r="J31" s="1" t="str">
-        <f t="shared" si="28"/>
-        <v xml:space="preserve">  { "Pedal DB 8" },  // #29 </v>
-      </c>
-      <c r="K31" s="18" t="str">
-        <f t="shared" si="29"/>
-        <v xml:space="preserve">  0, // #29 = Pedal DB 8</v>
-      </c>
-      <c r="L31" s="18" t="str">
-        <f t="shared" si="30"/>
-        <v xml:space="preserve">  127, // #29 = Pedal DB 8</v>
-      </c>
-      <c r="M31" s="18" t="str">
-        <f t="shared" si="31"/>
-        <v xml:space="preserve">  0, // #29 = Pedal DB 8</v>
-      </c>
-      <c r="N31" s="18" t="str">
+      <c r="I32" s="18" t="str">
+        <f t="shared" si="33"/>
+        <v xml:space="preserve">  m_pedal_db_8, // #30 = Pedal DB 8</v>
+      </c>
+      <c r="J32" s="1" t="str">
+        <f t="shared" si="34"/>
+        <v xml:space="preserve">  { "Pedal DB 8" },  // #30 </v>
+      </c>
+      <c r="K32" s="18" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">  0, // #30 = Pedal DB 8</v>
+      </c>
+      <c r="L32" s="18" t="str">
+        <f t="shared" si="36"/>
+        <v xml:space="preserve">  127, // #30 = Pedal DB 8</v>
+      </c>
+      <c r="M32" s="18" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">  0, // #30 = Pedal DB 8</v>
+      </c>
+      <c r="N32" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_pedal_db, // Pedal DB 8</v>
       </c>
-      <c r="O31" s="18" t="str">
+      <c r="O32" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  60, // #29 = Pedal DB 8</v>
-      </c>
-      <c r="P31" s="13"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
-        <f t="shared" si="6"/>
-        <v>30</v>
-      </c>
-      <c r="B32" s="22" t="s">
+        <v xml:space="preserve">  60, // #30 = Pedal DB 8</v>
+      </c>
+      <c r="P32" s="13"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <f t="shared" si="6"/>
+        <v>31</v>
+      </c>
+      <c r="B33" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C33" s="22">
         <v>-1</v>
       </c>
-      <c r="D32" s="22">
-        <v>0</v>
-      </c>
-      <c r="E32" s="22">
-        <v>0</v>
-      </c>
-      <c r="F32" s="22">
-        <v>0</v>
-      </c>
-      <c r="G32" s="26" t="str">
-        <f>CONCATENATE("m_back_",A32)</f>
-        <v>m_back_30</v>
-      </c>
-      <c r="H32" s="12" t="s">
+      <c r="D33" s="22">
+        <v>0</v>
+      </c>
+      <c r="E33" s="22">
+        <v>0</v>
+      </c>
+      <c r="F33" s="22">
+        <v>0</v>
+      </c>
+      <c r="G33" s="26" t="str">
+        <f>CONCATENATE("m_back_",A33)</f>
+        <v>m_back_31</v>
+      </c>
+      <c r="H33" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I32" s="26" t="str">
-        <f t="shared" ref="I32" si="33">CONCATENATE("  ",G32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_30, // #30 = Pedal DB EXIT </v>
-      </c>
-      <c r="J32" s="22" t="str">
-        <f t="shared" ref="J32" si="34">CONCATENATE("  { """,B32,""" },  // #",A32," ",IF(C32&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pedal DB" },  // #30  EXIT SUBM</v>
-      </c>
-      <c r="K32" s="26" t="str">
-        <f t="shared" ref="K32" si="35">CONCATENATE("  ",D32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #30 = Pedal DB EXIT </v>
-      </c>
-      <c r="L32" s="26" t="str">
-        <f t="shared" ref="L32" si="36">CONCATENATE("  ",E32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #30 = Pedal DB EXIT </v>
-      </c>
-      <c r="M32" s="26" t="str">
-        <f t="shared" ref="M32" si="37">CONCATENATE("  ",C32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #30 = Pedal DB EXIT </v>
-      </c>
-      <c r="N32" s="18" t="str">
+      <c r="I33" s="26" t="str">
+        <f t="shared" ref="I33:I34" si="39">CONCATENATE("  ",G33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_back_31, // #31 = Pedal DB EXIT </v>
+      </c>
+      <c r="J33" s="22" t="str">
+        <f t="shared" ref="J33:J34" si="40">CONCATENATE("  { """,B33,""" },  // #",A33," ",IF(C33&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Pedal DB" },  // #31  EXIT SUBM</v>
+      </c>
+      <c r="K33" s="26" t="str">
+        <f t="shared" ref="K33:K34" si="41">CONCATENATE("  ",D33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #31 = Pedal DB EXIT </v>
+      </c>
+      <c r="L33" s="26" t="str">
+        <f t="shared" ref="L33:L34" si="42">CONCATENATE("  ",E33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #31 = Pedal DB EXIT </v>
+      </c>
+      <c r="M33" s="26" t="str">
+        <f t="shared" ref="M33:M34" si="43">CONCATENATE("  ",C33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -1, // #31 = Pedal DB EXIT </v>
+      </c>
+      <c r="N33" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // Pedal DB</v>
       </c>
-      <c r="O32" s="26" t="str">
+      <c r="O33" s="26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #30 = Pedal DB EXIT </v>
-      </c>
-      <c r="P32" s="13"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
-        <f t="shared" si="6"/>
-        <v>31</v>
-      </c>
-      <c r="B33" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="C33" s="20">
-        <v>0</v>
-      </c>
-      <c r="D33" s="20">
-        <v>0</v>
-      </c>
-      <c r="E33" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G33" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B33,"/","")," ","_")))</f>
-        <v>m_kbd_driver</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="I33" s="18" t="str">
-        <f t="shared" ref="I33:I40" si="38">CONCATENATE("  ",G33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_kbd_driver, // #31 = Kbd Driver</v>
-      </c>
-      <c r="J33" s="1" t="str">
-        <f t="shared" ref="J33:J40" si="39">CONCATENATE("  { """,B33,""" },  // #",A33," ",IF(C33&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Kbd Driver" },  // #31 </v>
-      </c>
-      <c r="K33" s="18" t="str">
-        <f t="shared" ref="K33:K40" si="40">CONCATENATE("  ",D33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #31 = Kbd Driver</v>
-      </c>
-      <c r="L33" s="18" t="str">
-        <f t="shared" ref="L33:L40" si="41">CONCATENATE("  ",E33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  drv_custom, // #31 = Kbd Driver</v>
-      </c>
-      <c r="M33" s="18" t="str">
-        <f t="shared" ref="M33:M40" si="42">CONCATENATE("  ",C33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #31 = Kbd Driver</v>
-      </c>
-      <c r="N33" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Kbd Driver</v>
-      </c>
-      <c r="O33" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  drv_fatar1, // #31 = Kbd Driver</v>
+        <v xml:space="preserve">  0, // #31 = Pedal DB EXIT </v>
       </c>
       <c r="P33" s="13"/>
     </row>
@@ -3134,226 +3168,228 @@
         <f t="shared" si="6"/>
         <v>32</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>5</v>
+      <c r="B34" s="38" t="s">
+        <v>208</v>
       </c>
       <c r="C34" s="1">
         <v>0</v>
       </c>
-      <c r="D34" s="1">
-        <v>1</v>
-      </c>
-      <c r="E34" s="1">
-        <v>40</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>35</v>
+      <c r="D34" s="12">
+        <v>0</v>
+      </c>
+      <c r="E34" s="12">
+        <v>0</v>
+      </c>
+      <c r="F34" s="12">
+        <v>0</v>
       </c>
       <c r="G34" s="12" t="str">
-        <f t="shared" ref="G34:G39" si="43">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B34,"/","")," ","_")))</f>
-        <v>m_velocity_min</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>199</v>
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B34,"/","")," ","_")))</f>
+        <v>m_sd_card_init</v>
+      </c>
+      <c r="H34" s="12" t="str">
+        <f>CONCATENATE("ac_",LOWER(SUBSTITUTE(SUBSTITUTE(B34,"/","")," ","_")))</f>
+        <v>ac_sd_card_init</v>
       </c>
       <c r="I34" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_velocity_min, // #32 = Velocity Min</v>
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">  m_sd_card_init, // #32 = SD Card Init</v>
       </c>
       <c r="J34" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Velocity Min" },  // #32 </v>
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">  { "SD Card Init" },  // #32 </v>
       </c>
       <c r="K34" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  1, // #32 = Velocity Min</v>
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">  0, // #32 = SD Card Init</v>
       </c>
       <c r="L34" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  40, // #32 = Velocity Min</v>
+        <f t="shared" si="42"/>
+        <v xml:space="preserve">  0, // #32 = SD Card Init</v>
       </c>
       <c r="M34" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #32 = Velocity Min</v>
+        <f t="shared" si="43"/>
+        <v xml:space="preserve">  0, // #32 = SD Card Init</v>
       </c>
       <c r="N34" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Velocity Min</v>
+        <v xml:space="preserve">  ac_sd_card_init, // SD Card Init</v>
       </c>
       <c r="O34" s="18" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_MINDYN, // #32 = Velocity Min</v>
-      </c>
-      <c r="P34" s="13"/>
+        <v xml:space="preserve">  0, // #32 = SD Card Init</v>
+      </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <f t="shared" si="6"/>
         <v>33</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>60</v>
+      <c r="B35" s="38" t="s">
+        <v>209</v>
       </c>
       <c r="C35" s="1">
         <v>0</v>
       </c>
-      <c r="D35" s="1">
-        <v>1</v>
-      </c>
-      <c r="E35" s="1">
-        <v>40</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>36</v>
+      <c r="D35" s="12">
+        <v>0</v>
+      </c>
+      <c r="E35" s="12">
+        <v>0</v>
+      </c>
+      <c r="F35" s="12">
+        <v>0</v>
       </c>
       <c r="G35" s="12" t="str">
-        <f t="shared" si="43"/>
-        <v>m_velocity_maxadj</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>199</v>
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B35,"/","")," ","_")))</f>
+        <v>m_load_sd_scan</v>
+      </c>
+      <c r="H35" s="12" t="str">
+        <f t="shared" ref="H35:H40" si="44">CONCATENATE("ac_",LOWER(SUBSTITUTE(SUBSTITUTE(B35,"/","")," ","_")))</f>
+        <v>ac_load_sd_scan</v>
       </c>
       <c r="I35" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_velocity_maxadj, // #33 = Velocity MaxAdj</v>
+        <f t="shared" ref="I35" si="45">CONCATENATE("  ",G35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_load_sd_scan, // #33 = Load SD Scan</v>
       </c>
       <c r="J35" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Velocity MaxAdj" },  // #33 </v>
+        <f t="shared" ref="J35" si="46">CONCATENATE("  { """,B35,""" },  // #",A35," ",IF(C35&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Load SD Scan" },  // #33 </v>
       </c>
       <c r="K35" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  1, // #33 = Velocity MaxAdj</v>
+        <f t="shared" ref="K35" si="47">CONCATENATE("  ",D35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
       </c>
       <c r="L35" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  40, // #33 = Velocity MaxAdj</v>
+        <f t="shared" ref="L35" si="48">CONCATENATE("  ",E35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
       </c>
       <c r="M35" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #33 = Velocity MaxAdj</v>
+        <f t="shared" ref="M35" si="49">CONCATENATE("  ",C35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
       </c>
       <c r="N35" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Velocity MaxAdj</v>
+        <f t="shared" ref="N35" si="50">CONCATENATE("  ",H35,", // ",B35)</f>
+        <v xml:space="preserve">  ac_load_sd_scan, // Load SD Scan</v>
       </c>
       <c r="O35" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_MAXDYNADJ, // #33 = Velocity MaxAdj</v>
-      </c>
-      <c r="P35" s="13"/>
+        <f t="shared" ref="O35" si="51">CONCATENATE("  ",F35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
+      </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <f t="shared" si="6"/>
         <v>34</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>6</v>
+      <c r="B36" s="38" t="s">
+        <v>210</v>
       </c>
       <c r="C36" s="1">
         <v>0</v>
       </c>
-      <c r="D36" s="1">
-        <v>1</v>
-      </c>
-      <c r="E36" s="1">
-        <v>30</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>37</v>
+      <c r="D36" s="12">
+        <v>0</v>
+      </c>
+      <c r="E36" s="12">
+        <v>0</v>
+      </c>
+      <c r="F36" s="12">
+        <v>0</v>
       </c>
       <c r="G36" s="12" t="str">
-        <f t="shared" si="43"/>
-        <v>m_velocity_slope</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>199</v>
+        <f t="shared" ref="G36:G40" si="52">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B36,"/","")," ","_")))</f>
+        <v>m_flash_sd_scan</v>
+      </c>
+      <c r="H36" s="12" t="str">
+        <f t="shared" si="44"/>
+        <v>ac_flash_sd_scan</v>
       </c>
       <c r="I36" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_velocity_slope, // #34 = Velocity Slope</v>
+        <f t="shared" ref="I36:I40" si="53">CONCATENATE("  ",G36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_flash_sd_scan, // #34 = Flash SD Scan</v>
       </c>
       <c r="J36" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Velocity Slope" },  // #34 </v>
+        <f t="shared" ref="J36:J40" si="54">CONCATENATE("  { """,B36,""" },  // #",A36," ",IF(C36&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Flash SD Scan" },  // #34 </v>
       </c>
       <c r="K36" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  1, // #34 = Velocity Slope</v>
+        <f t="shared" ref="K36:K40" si="55">CONCATENATE("  ",D36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
       </c>
       <c r="L36" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  30, // #34 = Velocity Slope</v>
+        <f t="shared" ref="L36:L40" si="56">CONCATENATE("  ",E36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
       </c>
       <c r="M36" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #34 = Velocity Slope</v>
+        <f t="shared" ref="M36:M40" si="57">CONCATENATE("  ",C36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
       </c>
       <c r="N36" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Velocity Slope</v>
+        <f t="shared" ref="N36:N40" si="58">CONCATENATE("  ",H36,", // ",B36)</f>
+        <v xml:space="preserve">  ac_flash_sd_scan, // Flash SD Scan</v>
       </c>
       <c r="O36" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_DYNSLOPE, // #34 = Velocity Slope</v>
+        <f t="shared" ref="O36:O40" si="59">CONCATENATE("  ",F36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
       </c>
       <c r="P36" s="13"/>
     </row>
-    <row r="37" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <f t="shared" si="6"/>
         <v>35</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>15</v>
+      <c r="B37" s="38" t="s">
+        <v>211</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
       </c>
-      <c r="D37" s="1">
-        <v>12</v>
-      </c>
-      <c r="E37" s="1">
-        <v>60</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>32</v>
+      <c r="D37" s="12">
+        <v>0</v>
+      </c>
+      <c r="E37" s="12">
+        <v>0</v>
+      </c>
+      <c r="F37" s="12">
+        <v>0</v>
       </c>
       <c r="G37" s="12" t="str">
-        <f t="shared" si="43"/>
-        <v>m_upper_base</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>199</v>
+        <f t="shared" si="52"/>
+        <v>m_flash_fpga</v>
+      </c>
+      <c r="H37" s="12" t="str">
+        <f t="shared" si="44"/>
+        <v>ac_flash_fpga</v>
       </c>
       <c r="I37" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_upper_base, // #35 = Upper Base</v>
+        <f t="shared" si="53"/>
+        <v xml:space="preserve">  m_flash_fpga, // #35 = Flash FPGA</v>
       </c>
       <c r="J37" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Upper Base" },  // #35 </v>
+        <f t="shared" si="54"/>
+        <v xml:space="preserve">  { "Flash FPGA" },  // #35 </v>
       </c>
       <c r="K37" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  12, // #35 = Upper Base</v>
+        <f t="shared" si="55"/>
+        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
       </c>
       <c r="L37" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  60, // #35 = Upper Base</v>
+        <f t="shared" si="56"/>
+        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
       </c>
       <c r="M37" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #35 = Upper Base</v>
+        <f t="shared" si="57"/>
+        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
       </c>
       <c r="N37" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Upper Base</v>
+        <f t="shared" si="58"/>
+        <v xml:space="preserve">  ac_flash_fpga, // Flash FPGA</v>
       </c>
       <c r="O37" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_BASE_UPR, // #35 = Upper Base</v>
+        <f t="shared" si="59"/>
+        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
       </c>
       <c r="P37" s="13"/>
     </row>
@@ -3362,192 +3398,715 @@
         <f t="shared" si="6"/>
         <v>36</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>16</v>
+      <c r="B38" s="38" t="s">
+        <v>214</v>
       </c>
       <c r="C38" s="1">
         <v>0</v>
       </c>
-      <c r="D38" s="1">
-        <v>12</v>
-      </c>
-      <c r="E38" s="1">
-        <v>60</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>33</v>
+      <c r="D38" s="12">
+        <v>0</v>
+      </c>
+      <c r="E38" s="12">
+        <v>0</v>
+      </c>
+      <c r="F38" s="12">
+        <v>0</v>
       </c>
       <c r="G38" s="12" t="str">
-        <f t="shared" si="43"/>
-        <v>m_lower_base</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>199</v>
+        <f t="shared" si="52"/>
+        <v>m_flash_other</v>
+      </c>
+      <c r="H38" s="12" t="str">
+        <f t="shared" si="44"/>
+        <v>ac_flash_other</v>
       </c>
       <c r="I38" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_lower_base, // #36 = Lower Base</v>
+        <f t="shared" si="53"/>
+        <v xml:space="preserve">  m_flash_other, // #36 = Flash Other</v>
       </c>
       <c r="J38" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Lower Base" },  // #36 </v>
+        <f t="shared" si="54"/>
+        <v xml:space="preserve">  { "Flash Other" },  // #36 </v>
       </c>
       <c r="K38" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  12, // #36 = Lower Base</v>
+        <f t="shared" si="55"/>
+        <v xml:space="preserve">  0, // #36 = Flash Other</v>
       </c>
       <c r="L38" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  60, // #36 = Lower Base</v>
+        <f t="shared" si="56"/>
+        <v xml:space="preserve">  0, // #36 = Flash Other</v>
       </c>
       <c r="M38" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #36 = Lower Base</v>
+        <f t="shared" si="57"/>
+        <v xml:space="preserve">  0, // #36 = Flash Other</v>
       </c>
       <c r="N38" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Lower Base</v>
+        <f t="shared" si="58"/>
+        <v xml:space="preserve">  ac_flash_other, // Flash Other</v>
       </c>
       <c r="O38" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_BASE_LWR, // #36 = Lower Base</v>
+        <f t="shared" si="59"/>
+        <v xml:space="preserve">  0, // #36 = Flash Other</v>
       </c>
       <c r="P38" s="13"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
-        <f>A38+1</f>
+        <f t="shared" si="6"/>
         <v>37</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>17</v>
+      <c r="B39" s="38" t="s">
+        <v>212</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
       </c>
-      <c r="D39" s="1">
-        <v>12</v>
-      </c>
-      <c r="E39" s="1">
-        <v>60</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>34</v>
+      <c r="D39" s="12">
+        <v>0</v>
+      </c>
+      <c r="E39" s="12">
+        <v>0</v>
+      </c>
+      <c r="F39" s="12">
+        <v>0</v>
       </c>
       <c r="G39" s="12" t="str">
-        <f t="shared" si="43"/>
-        <v>m_pedal_base</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>199</v>
+        <f t="shared" si="52"/>
+        <v>m_reload_fpga</v>
+      </c>
+      <c r="H39" s="12" t="str">
+        <f t="shared" si="44"/>
+        <v>ac_reload_fpga</v>
       </c>
       <c r="I39" s="18" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_pedal_base, // #37 = Pedal Base</v>
+        <f t="shared" si="53"/>
+        <v xml:space="preserve">  m_reload_fpga, // #37 = Reload FPGA</v>
       </c>
       <c r="J39" s="1" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "Pedal Base" },  // #37 </v>
+        <f t="shared" si="54"/>
+        <v xml:space="preserve">  { "Reload FPGA" },  // #37 </v>
       </c>
       <c r="K39" s="18" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  12, // #37 = Pedal Base</v>
+        <f t="shared" si="55"/>
+        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
       </c>
       <c r="L39" s="18" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  60, // #37 = Pedal Base</v>
+        <f t="shared" si="56"/>
+        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
       </c>
       <c r="M39" s="18" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  0, // #37 = Pedal Base</v>
+        <f t="shared" si="57"/>
+        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
       </c>
       <c r="N39" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">  ac_none, // Pedal Base</v>
+        <f t="shared" si="58"/>
+        <v xml:space="preserve">  ac_reload_fpga, // Reload FPGA</v>
       </c>
       <c r="O39" s="18" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">  MIDI_BASE_PED, // #37 = Pedal Base</v>
+        <f t="shared" si="59"/>
+        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
       </c>
       <c r="P39" s="13"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
-        <f>A39+1</f>
+        <f t="shared" si="6"/>
         <v>38</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="38" t="s">
+        <v>213</v>
+      </c>
+      <c r="C40" s="1">
+        <v>0</v>
+      </c>
+      <c r="D40" s="12">
+        <v>0</v>
+      </c>
+      <c r="E40" s="12">
+        <v>0</v>
+      </c>
+      <c r="F40" s="12">
+        <v>0</v>
+      </c>
+      <c r="G40" s="12" t="str">
+        <f t="shared" si="52"/>
+        <v>m_test</v>
+      </c>
+      <c r="H40" s="12" t="str">
+        <f t="shared" si="44"/>
+        <v>ac_test</v>
+      </c>
+      <c r="I40" s="18" t="str">
+        <f t="shared" si="53"/>
+        <v xml:space="preserve">  m_test, // #38 = Test</v>
+      </c>
+      <c r="J40" s="1" t="str">
+        <f t="shared" si="54"/>
+        <v xml:space="preserve">  { "Test" },  // #38 </v>
+      </c>
+      <c r="K40" s="18" t="str">
+        <f t="shared" si="55"/>
+        <v xml:space="preserve">  0, // #38 = Test</v>
+      </c>
+      <c r="L40" s="18" t="str">
+        <f t="shared" si="56"/>
+        <v xml:space="preserve">  0, // #38 = Test</v>
+      </c>
+      <c r="M40" s="18" t="str">
+        <f t="shared" si="57"/>
+        <v xml:space="preserve">  0, // #38 = Test</v>
+      </c>
+      <c r="N40" s="18" t="str">
+        <f t="shared" si="58"/>
+        <v xml:space="preserve">  ac_test, // Test</v>
+      </c>
+      <c r="O40" s="18" t="str">
+        <f t="shared" si="59"/>
+        <v xml:space="preserve">  0, // #38 = Test</v>
+      </c>
+      <c r="P40" s="13"/>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <f t="shared" si="6"/>
+        <v>39</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="C41" s="22">
+        <v>-1</v>
+      </c>
+      <c r="D41" s="22">
+        <v>0</v>
+      </c>
+      <c r="E41" s="22">
+        <v>0</v>
+      </c>
+      <c r="F41" s="22">
+        <v>0</v>
+      </c>
+      <c r="G41" s="26" t="str">
+        <f>CONCATENATE("m_back_",A41)</f>
+        <v>m_back_39</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="I41" s="26" t="str">
+        <f t="shared" ref="I41" si="60">CONCATENATE("  ",G41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_back_39, // #39 = Utilities EXIT </v>
+      </c>
+      <c r="J41" s="22" t="str">
+        <f t="shared" ref="J41" si="61">CONCATENATE("  { """,B41,""" },  // #",A41," ",IF(C41&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Utilities" },  // #39  EXIT SUBM</v>
+      </c>
+      <c r="K41" s="26" t="str">
+        <f t="shared" ref="K41" si="62">CONCATENATE("  ",D41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #39 = Utilities EXIT </v>
+      </c>
+      <c r="L41" s="26" t="str">
+        <f t="shared" ref="L41" si="63">CONCATENATE("  ",E41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #39 = Utilities EXIT </v>
+      </c>
+      <c r="M41" s="26" t="str">
+        <f t="shared" ref="M41" si="64">CONCATENATE("  ",C41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -1, // #39 = Utilities EXIT </v>
+      </c>
+      <c r="N41" s="18" t="str">
+        <f t="shared" ref="N41" si="65">CONCATENATE("  ",H41,", // ",B41)</f>
+        <v xml:space="preserve">  ac_none, // Utilities</v>
+      </c>
+      <c r="O41" s="26" t="str">
+        <f t="shared" ref="O41" si="66">CONCATENATE("  ",F41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #39 = Utilities EXIT </v>
+      </c>
+      <c r="P41" s="13"/>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <f t="shared" si="6"/>
+        <v>40</v>
+      </c>
+      <c r="B42" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="20">
+        <v>0</v>
+      </c>
+      <c r="D42" s="20">
+        <v>0</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G42" s="12" t="str">
+        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B42,"/","")," ","_")))</f>
+        <v>m_kbd_driver</v>
+      </c>
+      <c r="H42" s="12" t="str">
+        <f>CONCATENATE("ac_",LOWER(SUBSTITUTE(SUBSTITUTE(B42,"/","")," ","_")))</f>
+        <v>ac_kbd_driver</v>
+      </c>
+      <c r="I42" s="18" t="str">
+        <f t="shared" ref="I42:I49" si="67">CONCATENATE("  ",G42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  m_kbd_driver, // #40 = Kbd Driver</v>
+      </c>
+      <c r="J42" s="1" t="str">
+        <f t="shared" ref="J42:J49" si="68">CONCATENATE("  { """,B42,""" },  // #",A42," ",IF(C42&lt;0," EXIT SUBM",""))</f>
+        <v xml:space="preserve">  { "Kbd Driver" },  // #40 </v>
+      </c>
+      <c r="K42" s="18" t="str">
+        <f t="shared" ref="K42:K49" si="69">CONCATENATE("  ",D42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #40 = Kbd Driver</v>
+      </c>
+      <c r="L42" s="18" t="str">
+        <f t="shared" ref="L42:L49" si="70">CONCATENATE("  ",E42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  drv_custom, // #40 = Kbd Driver</v>
+      </c>
+      <c r="M42" s="18" t="str">
+        <f t="shared" ref="M42:M49" si="71">CONCATENATE("  ",C42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #40 = Kbd Driver</v>
+      </c>
+      <c r="N42" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_kbd_driver, // Kbd Driver</v>
+      </c>
+      <c r="O42" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  drv_fatar1, // #40 = Kbd Driver</v>
+      </c>
+      <c r="P42" s="13"/>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <f t="shared" si="6"/>
+        <v>41</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" s="1">
+        <v>0</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1</v>
+      </c>
+      <c r="E43" s="1">
+        <v>40</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G43" s="12" t="str">
+        <f t="shared" ref="G43:G48" si="72">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B43,"/","")," ","_")))</f>
+        <v>m_velocity_min</v>
+      </c>
+      <c r="H43" s="12" t="str">
+        <f t="shared" ref="H43:H48" si="73">CONCATENATE("ac_",LOWER(SUBSTITUTE(SUBSTITUTE(B43,"/","")," ","_")))</f>
+        <v>ac_velocity_min</v>
+      </c>
+      <c r="I43" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_velocity_min, // #41 = Velocity Min</v>
+      </c>
+      <c r="J43" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Velocity Min" },  // #41 </v>
+      </c>
+      <c r="K43" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  1, // #41 = Velocity Min</v>
+      </c>
+      <c r="L43" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  40, // #41 = Velocity Min</v>
+      </c>
+      <c r="M43" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #41 = Velocity Min</v>
+      </c>
+      <c r="N43" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_velocity_min, // Velocity Min</v>
+      </c>
+      <c r="O43" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_MINDYN, // #41 = Velocity Min</v>
+      </c>
+      <c r="P43" s="13"/>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <f t="shared" si="6"/>
+        <v>42</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0</v>
+      </c>
+      <c r="D44" s="1">
+        <v>1</v>
+      </c>
+      <c r="E44" s="1">
+        <v>40</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44" s="12" t="str">
+        <f t="shared" si="72"/>
+        <v>m_velocity_maxadj</v>
+      </c>
+      <c r="H44" s="12" t="str">
+        <f t="shared" si="73"/>
+        <v>ac_velocity_maxadj</v>
+      </c>
+      <c r="I44" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_velocity_maxadj, // #42 = Velocity MaxAdj</v>
+      </c>
+      <c r="J44" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Velocity MaxAdj" },  // #42 </v>
+      </c>
+      <c r="K44" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  1, // #42 = Velocity MaxAdj</v>
+      </c>
+      <c r="L44" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  40, // #42 = Velocity MaxAdj</v>
+      </c>
+      <c r="M44" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #42 = Velocity MaxAdj</v>
+      </c>
+      <c r="N44" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_velocity_maxadj, // Velocity MaxAdj</v>
+      </c>
+      <c r="O44" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_MAXDYNADJ, // #42 = Velocity MaxAdj</v>
+      </c>
+      <c r="P44" s="13"/>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <f t="shared" si="6"/>
+        <v>43</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0</v>
+      </c>
+      <c r="D45" s="1">
+        <v>1</v>
+      </c>
+      <c r="E45" s="1">
+        <v>30</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G45" s="12" t="str">
+        <f t="shared" si="72"/>
+        <v>m_velocity_slope</v>
+      </c>
+      <c r="H45" s="12" t="str">
+        <f t="shared" si="73"/>
+        <v>ac_velocity_slope</v>
+      </c>
+      <c r="I45" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_velocity_slope, // #43 = Velocity Slope</v>
+      </c>
+      <c r="J45" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Velocity Slope" },  // #43 </v>
+      </c>
+      <c r="K45" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  1, // #43 = Velocity Slope</v>
+      </c>
+      <c r="L45" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  30, // #43 = Velocity Slope</v>
+      </c>
+      <c r="M45" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #43 = Velocity Slope</v>
+      </c>
+      <c r="N45" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_velocity_slope, // Velocity Slope</v>
+      </c>
+      <c r="O45" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_DYNSLOPE, // #43 = Velocity Slope</v>
+      </c>
+      <c r="P45" s="13"/>
+    </row>
+    <row r="46" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <f t="shared" si="6"/>
+        <v>44</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="1">
+        <v>0</v>
+      </c>
+      <c r="D46" s="1">
+        <v>12</v>
+      </c>
+      <c r="E46" s="1">
+        <v>60</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G46" s="12" t="str">
+        <f t="shared" si="72"/>
+        <v>m_upper_base</v>
+      </c>
+      <c r="H46" s="12" t="str">
+        <f t="shared" si="73"/>
+        <v>ac_upper_base</v>
+      </c>
+      <c r="I46" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_upper_base, // #44 = Upper Base</v>
+      </c>
+      <c r="J46" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Upper Base" },  // #44 </v>
+      </c>
+      <c r="K46" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  12, // #44 = Upper Base</v>
+      </c>
+      <c r="L46" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  60, // #44 = Upper Base</v>
+      </c>
+      <c r="M46" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #44 = Upper Base</v>
+      </c>
+      <c r="N46" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_upper_base, // Upper Base</v>
+      </c>
+      <c r="O46" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_BASE_UPR, // #44 = Upper Base</v>
+      </c>
+      <c r="P46" s="13"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <f t="shared" si="6"/>
+        <v>45</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="1">
+        <v>0</v>
+      </c>
+      <c r="D47" s="1">
+        <v>12</v>
+      </c>
+      <c r="E47" s="1">
+        <v>60</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G47" s="12" t="str">
+        <f t="shared" si="72"/>
+        <v>m_lower_base</v>
+      </c>
+      <c r="H47" s="12" t="str">
+        <f t="shared" si="73"/>
+        <v>ac_lower_base</v>
+      </c>
+      <c r="I47" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_lower_base, // #45 = Lower Base</v>
+      </c>
+      <c r="J47" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Lower Base" },  // #45 </v>
+      </c>
+      <c r="K47" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  12, // #45 = Lower Base</v>
+      </c>
+      <c r="L47" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  60, // #45 = Lower Base</v>
+      </c>
+      <c r="M47" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #45 = Lower Base</v>
+      </c>
+      <c r="N47" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_lower_base, // Lower Base</v>
+      </c>
+      <c r="O47" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_BASE_LWR, // #45 = Lower Base</v>
+      </c>
+      <c r="P47" s="13"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <f>A47+1</f>
+        <v>46</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0</v>
+      </c>
+      <c r="D48" s="1">
+        <v>12</v>
+      </c>
+      <c r="E48" s="1">
+        <v>60</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G48" s="12" t="str">
+        <f t="shared" si="72"/>
+        <v>m_pedal_base</v>
+      </c>
+      <c r="H48" s="12" t="str">
+        <f t="shared" si="73"/>
+        <v>ac_pedal_base</v>
+      </c>
+      <c r="I48" s="18" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_pedal_base, // #46 = Pedal Base</v>
+      </c>
+      <c r="J48" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "Pedal Base" },  // #46 </v>
+      </c>
+      <c r="K48" s="18" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  12, // #46 = Pedal Base</v>
+      </c>
+      <c r="L48" s="18" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  60, // #46 = Pedal Base</v>
+      </c>
+      <c r="M48" s="18" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  0, // #46 = Pedal Base</v>
+      </c>
+      <c r="N48" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">  ac_pedal_base, // Pedal Base</v>
+      </c>
+      <c r="O48" s="18" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve">  MIDI_BASE_PED, // #46 = Pedal Base</v>
+      </c>
+      <c r="P48" s="13"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <f>A48+1</f>
+        <v>47</v>
+      </c>
+      <c r="B49" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C40" s="22">
+      <c r="C49" s="22">
         <v>-1</v>
       </c>
-      <c r="D40" s="22">
-        <v>0</v>
-      </c>
-      <c r="E40" s="22">
-        <v>0</v>
-      </c>
-      <c r="F40" s="22">
-        <v>0</v>
-      </c>
-      <c r="G40" s="26" t="str">
-        <f>CONCATENATE("m_back_",A40)</f>
-        <v>m_back_38</v>
-      </c>
-      <c r="H40" s="12" t="s">
+      <c r="D49" s="22">
+        <v>0</v>
+      </c>
+      <c r="E49" s="22">
+        <v>0</v>
+      </c>
+      <c r="F49" s="22">
+        <v>0</v>
+      </c>
+      <c r="G49" s="26" t="str">
+        <f>CONCATENATE("m_back_",A49)</f>
+        <v>m_back_47</v>
+      </c>
+      <c r="H49" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="I40" s="26" t="str">
-        <f t="shared" si="38"/>
-        <v xml:space="preserve">  m_back_38, // #38 = (Keyboard) EXIT </v>
-      </c>
-      <c r="J40" s="22" t="str">
-        <f t="shared" si="39"/>
-        <v xml:space="preserve">  { "(Keyboard)" },  // #38  EXIT SUBM</v>
-      </c>
-      <c r="K40" s="26" t="str">
-        <f t="shared" si="40"/>
-        <v xml:space="preserve">  0, // #38 = (Keyboard) EXIT </v>
-      </c>
-      <c r="L40" s="26" t="str">
-        <f t="shared" si="41"/>
-        <v xml:space="preserve">  0, // #38 = (Keyboard) EXIT </v>
-      </c>
-      <c r="M40" s="26" t="str">
-        <f t="shared" si="42"/>
-        <v xml:space="preserve">  -1, // #38 = (Keyboard) EXIT </v>
-      </c>
-      <c r="N40" s="18" t="str">
+      <c r="I49" s="26" t="str">
+        <f t="shared" si="67"/>
+        <v xml:space="preserve">  m_back_47, // #47 = (Keyboard) EXIT </v>
+      </c>
+      <c r="J49" s="22" t="str">
+        <f t="shared" si="68"/>
+        <v xml:space="preserve">  { "(Keyboard)" },  // #47  EXIT SUBM</v>
+      </c>
+      <c r="K49" s="26" t="str">
+        <f t="shared" si="69"/>
+        <v xml:space="preserve">  0, // #47 = (Keyboard) EXIT </v>
+      </c>
+      <c r="L49" s="26" t="str">
+        <f t="shared" si="70"/>
+        <v xml:space="preserve">  0, // #47 = (Keyboard) EXIT </v>
+      </c>
+      <c r="M49" s="26" t="str">
+        <f t="shared" si="71"/>
+        <v xml:space="preserve">  -1, // #47 = (Keyboard) EXIT </v>
+      </c>
+      <c r="N49" s="18" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">  ac_none, // (Keyboard)</v>
       </c>
-      <c r="O40" s="26" t="str">
+      <c r="O49" s="26" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">  0, // #38 = (Keyboard) EXIT </v>
-      </c>
-      <c r="P40" s="13"/>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="I41" s="15" t="s">
+        <v xml:space="preserve">  0, // #47 = (Keyboard) EXIT </v>
+      </c>
+      <c r="P49" s="13"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I50" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="J50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="K50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="L41" s="1" t="s">
+      <c r="L50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M41" s="1" t="s">
+      <c r="M50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N41" s="1" t="s">
+      <c r="N50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="O41" s="1" t="s">
+      <c r="O50" s="1" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added organ/speaker load from DF
</commit_message>
<xml_diff>
--- a/docs/HX35_menuItems.xlsx
+++ b/docs/HX35_menuItems.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="265">
   <si>
     <t>Index #</t>
   </si>
@@ -643,12 +643,6 @@
     <t>SD Flash Tools</t>
   </si>
   <si>
-    <t>int8_t * EditValueLinks[MENU_ITEMCOUNT] = {</t>
-  </si>
-  <si>
-    <t>Zuweisung</t>
-  </si>
-  <si>
     <t>NULL</t>
   </si>
   <si>
@@ -751,17 +745,83 @@
     <t>setAmpVolume</t>
   </si>
   <si>
-    <t>&amp;preset.masterVolume</t>
-  </si>
-  <si>
-    <t>&amp;preset.ampVolume</t>
+    <t>Organ Model</t>
+  </si>
+  <si>
+    <t>menuOrganModel</t>
+  </si>
+  <si>
+    <t>Speaker Model</t>
+  </si>
+  <si>
+    <t>menuSpeakerModel</t>
+  </si>
+  <si>
+    <t>m_upper_db_16</t>
+  </si>
+  <si>
+    <t>m_lower_db_16</t>
+  </si>
+  <si>
+    <t>m_pedal_db_16</t>
+  </si>
+  <si>
+    <t>m_sd_card_info</t>
+  </si>
+  <si>
+    <t>m_kbd_driver</t>
+  </si>
+  <si>
+    <t>MenuLink-Konstanten für Submenus</t>
+  </si>
+  <si>
+    <t>zeigt auf</t>
+  </si>
+  <si>
+    <t>C++</t>
+  </si>
+  <si>
+    <t>&amp;preamp.masterVolume</t>
+  </si>
+  <si>
+    <t>&amp;preamp.ampVolume</t>
+  </si>
+  <si>
+    <t>uint8_t * EditValuePtrs[MENU_ITEMCOUNT] = {</t>
+  </si>
+  <si>
+    <t>m_menu_end</t>
+  </si>
+  <si>
+    <t>Zuweisung Edit-Variable</t>
+  </si>
+  <si>
+    <t>&amp;boardInfo.scan_driverIdx</t>
+  </si>
+  <si>
+    <t>&amp;midiSettings.channelLower</t>
+  </si>
+  <si>
+    <t>&amp;midiSettings.channelPedal</t>
+  </si>
+  <si>
+    <t>&amp;organModel.fatarVelocityFac</t>
+  </si>
+  <si>
+    <t>&amp;midiSettings.channel</t>
+  </si>
+  <si>
+    <t>&amp;tabs.organModel</t>
+  </si>
+  <si>
+    <t>&amp;tabs.speakerModel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -884,8 +944,22 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color theme="8" tint="-0.249977111117893"/>
+      <name val="Lucida Console"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF00B0F0"/>
+      <color indexed="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -947,7 +1021,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1048,7 +1122,7 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1071,6 +1145,39 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1376,28 +1483,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P50"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
     <col min="4" max="5" width="12.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19" style="12" customWidth="1"/>
-    <col min="8" max="8" width="29.7109375" style="12" customWidth="1"/>
-    <col min="9" max="9" width="27.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.85546875" style="12" customWidth="1"/>
+    <col min="7" max="8" width="26" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" style="12" customWidth="1"/>
+    <col min="10" max="10" width="25.42578125" style="12" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" style="13" customWidth="1"/>
     <col min="12" max="12" width="25.42578125" style="12" customWidth="1"/>
-    <col min="13" max="13" width="25.42578125" style="13" customWidth="1"/>
-    <col min="14" max="14" width="25.42578125" style="12" customWidth="1"/>
-    <col min="15" max="15" width="21.28515625" style="13" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" style="12" customWidth="1"/>
-    <col min="17" max="16384" width="11.42578125" style="12"/>
+    <col min="13" max="13" width="21.28515625" style="13" customWidth="1"/>
+    <col min="14" max="14" width="41.5703125" style="12" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" style="12" customWidth="1"/>
+    <col min="16" max="16" width="9.7109375" style="12" customWidth="1"/>
+    <col min="17" max="17" width="39.7109375" style="12" customWidth="1"/>
+    <col min="18" max="16384" width="11.42578125" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="7" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="7" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1416,38 +1523,37 @@
       <c r="F1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="11" t="s">
-        <v>39</v>
+      <c r="G1" s="48" t="s">
+        <v>13</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>13</v>
+        <v>25</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>27</v>
+        <v>21</v>
+      </c>
+      <c r="K1" s="40" t="s">
+        <v>228</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>21</v>
+        <v>232</v>
       </c>
       <c r="M1" s="40" t="s">
-        <v>230</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="O1" s="40" t="s">
-        <v>208</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="O1" s="46" t="s">
+        <v>250</v>
+      </c>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -1455,7 +1561,7 @@
         <v>172</v>
       </c>
       <c r="C2" s="5" t="str">
-        <f>G11</f>
+        <f>O3</f>
         <v>m_upper_db_16</v>
       </c>
       <c r="D2" s="1">
@@ -1467,55 +1573,56 @@
       <c r="F2" s="1">
         <v>0</v>
       </c>
-      <c r="G2" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(B2," ","_")))</f>
-        <v>m_upper_dbs</v>
-      </c>
-      <c r="H2" s="18" t="str">
-        <f>CONCATENATE("  ",G2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_dbs, // #0 = Upper DBs</v>
-      </c>
-      <c r="I2" s="1" t="str">
+      <c r="G2" s="50" t="str">
         <f>CONCATENATE("  { """,B2,""" },  // #",A2," ",IF(C2&lt;0," EXIT SUBM",""))</f>
         <v xml:space="preserve">  { "Upper DBs" },  // #0 </v>
       </c>
-      <c r="J2" s="18" t="str">
+      <c r="H2" s="51" t="str">
         <f>CONCATENATE("  ",D2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  1, // #0 = Upper DBs</v>
       </c>
-      <c r="K2" s="18" t="str">
+      <c r="I2" s="51" t="str">
         <f>CONCATENATE("  ",E2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #0 = Upper DBs</v>
       </c>
-      <c r="L2" s="18" t="str">
+      <c r="J2" s="51" t="str">
         <f>CONCATENATE("  ",C2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_upper_db_16, // #0 = Upper DBs</v>
       </c>
+      <c r="K2" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L2" s="51" t="str">
+        <f>IF(K2 = "NULL",CONCATENATE("  ",K2,", // #",A2," = ",B2),CONCATENATE("  &amp;",K2,", // ",B2))</f>
+        <v xml:space="preserve">  NULL, // #0 = Upper DBs</v>
+      </c>
       <c r="M2" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N2" s="18" t="str">
-        <f>IF(M2 = "NULL",CONCATENATE("  ",M2,","),CONCATENATE("  &amp;",M2,", // ",B2))</f>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P2" s="13" t="str">
-        <f>CONCATENATE("  ",O2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
+        <v>207</v>
+      </c>
+      <c r="N2" s="51" t="str">
+        <f>CONCATENATE("  ",M2,", // #",A2," = ",B2,IF(C2&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  NULL, // #0 = Upper DBs</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O2" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="44" t="s">
+        <v>251</v>
+      </c>
+      <c r="Q2" s="44" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <f t="shared" ref="A3:A47" si="0">A2+1</f>
+        <f t="shared" ref="A3:A49" si="0">A2+1</f>
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>173</v>
       </c>
       <c r="C3" s="5" t="str">
-        <f>G21</f>
+        <f>O4</f>
         <v>m_lower_db_16</v>
       </c>
       <c r="D3" s="1">
@@ -1527,46 +1634,49 @@
       <c r="F3" s="1">
         <v>0</v>
       </c>
-      <c r="G3" s="12" t="str">
-        <f t="shared" ref="G3:G9" si="1">CONCATENATE("m_",LOWER(SUBSTITUTE(B3," ","_")))</f>
-        <v>m_lower_dbs</v>
-      </c>
-      <c r="H3" s="18" t="str">
-        <f>CONCATENATE("  ",G3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_dbs, // #1 = Lower DBs</v>
-      </c>
-      <c r="I3" s="1" t="str">
-        <f>CONCATENATE("  { """,B3,""" },  // #",A3," ",IF(C3&lt;0," EXIT SUBM",""))</f>
+      <c r="G3" s="50" t="str">
+        <f t="shared" ref="G3:G51" si="1">CONCATENATE("  { """,B3,""" },  // #",A3," ",IF(C3&lt;0," EXIT SUBM",""))</f>
         <v xml:space="preserve">  { "Lower DBs" },  // #1 </v>
       </c>
-      <c r="J3" s="18" t="str">
+      <c r="H3" s="51" t="str">
         <f>CONCATENATE("  ",D3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  1, // #1 = Lower DBs</v>
       </c>
-      <c r="K3" s="18" t="str">
+      <c r="I3" s="51" t="str">
         <f>CONCATENATE("  ",E3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  16, // #1 = Lower DBs</v>
       </c>
-      <c r="L3" s="18" t="str">
+      <c r="J3" s="51" t="str">
         <f>CONCATENATE("  ",C3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_lower_db_16, // #1 = Lower DBs</v>
       </c>
+      <c r="K3" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L3" s="51" t="str">
+        <f t="shared" ref="L3:L51" si="2">IF(K3 = "NULL",CONCATENATE("  ",K3,", // #",A3," = ",B3),CONCATENATE("  &amp;",K3,", // ",B3))</f>
+        <v xml:space="preserve">  NULL, // #1 = Lower DBs</v>
+      </c>
       <c r="M3" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N3" s="18" t="str">
-        <f t="shared" ref="N3:N49" si="2">IF(M3 = "NULL",CONCATENATE("  ",M3,","),CONCATENATE("  &amp;",M3,", // ",B3))</f>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O3" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P3" s="13" t="str">
-        <f>CONCATENATE("  ",O3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
+        <v>207</v>
+      </c>
+      <c r="N3" s="51" t="str">
+        <f>CONCATENATE("  ",M3,", // #",A3," = ",B3,IF(C3&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  NULL, // #1 = Lower DBs</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O3" s="42" t="s">
+        <v>245</v>
+      </c>
+      <c r="P3" s="1">
+        <f>A13</f>
+        <v>11</v>
+      </c>
+      <c r="Q3" s="20" t="str">
+        <f>CONCATENATE("const uint8_t ",O3," = ",P3,";")</f>
+        <v>const uint8_t m_upper_db_16 = 11;</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1575,7 +1685,7 @@
         <v>174</v>
       </c>
       <c r="C4" s="5" t="str">
-        <f>G31</f>
+        <f>O5</f>
         <v>m_pedal_db_16</v>
       </c>
       <c r="D4" s="1">
@@ -1587,46 +1697,49 @@
       <c r="F4" s="1">
         <v>0</v>
       </c>
-      <c r="G4" s="12" t="str">
+      <c r="G4" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>m_pedal_dbs</v>
-      </c>
-      <c r="H4" s="18" t="str">
-        <f>CONCATENATE("  ",G4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_pedal_dbs, // #2 = Pedal DBs</v>
-      </c>
-      <c r="I4" s="1" t="str">
-        <f>CONCATENATE("  { """,B4,""" },  // #",A4," ",IF(C4&lt;0," EXIT SUBM",""))</f>
         <v xml:space="preserve">  { "Pedal DBs" },  // #2 </v>
       </c>
-      <c r="J4" s="18" t="str">
+      <c r="H4" s="51" t="str">
         <f>CONCATENATE("  ",D4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  1, // #2 = Pedal DBs</v>
       </c>
-      <c r="K4" s="18" t="str">
+      <c r="I4" s="51" t="str">
         <f>CONCATENATE("  ",E4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  16, // #2 = Pedal DBs</v>
       </c>
-      <c r="L4" s="18" t="str">
+      <c r="J4" s="51" t="str">
         <f>CONCATENATE("  ",C4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_pedal_db_16, // #2 = Pedal DBs</v>
       </c>
+      <c r="K4" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L4" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #2 = Pedal DBs</v>
+      </c>
       <c r="M4" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N4" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O4" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P4" s="13" t="str">
-        <f>CONCATENATE("  ",O4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
+        <v>207</v>
+      </c>
+      <c r="N4" s="51" t="str">
+        <f>CONCATENATE("  ",M4,", // #",A4," = ",B4,IF(C4&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  NULL, // #2 = Pedal DBs</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O4" s="42" t="s">
+        <v>246</v>
+      </c>
+      <c r="P4" s="1">
+        <f>A23</f>
+        <v>21</v>
+      </c>
+      <c r="Q4" s="20" t="str">
+        <f t="shared" ref="Q4:Q8" si="3">CONCATENATE("const uint8_t ",O4," = ",P4,";")</f>
+        <v>const uint8_t m_lower_db_16 = 21;</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1646,46 +1759,49 @@
       <c r="F5" s="12">
         <v>127</v>
       </c>
-      <c r="G5" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B5,"/","")," ","_")))</f>
-        <v>m_master_volume</v>
-      </c>
-      <c r="H5" s="18" t="str">
-        <f>CONCATENATE("  ",G5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_master_volume, // #3 = Master Volume</v>
-      </c>
-      <c r="I5" s="1" t="str">
-        <f>CONCATENATE("  { """,B5,""" },  // #",A5," ",IF(C5&lt;0," EXIT SUBM",""))</f>
+      <c r="G5" s="50" t="str">
+        <f t="shared" si="1"/>
         <v xml:space="preserve">  { "Master Volume" },  // #3 </v>
       </c>
-      <c r="J5" s="18" t="str">
+      <c r="H5" s="51" t="str">
         <f>CONCATENATE("  ",D5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #3 = Master Volume</v>
       </c>
-      <c r="K5" s="18" t="str">
+      <c r="I5" s="51" t="str">
         <f>CONCATENATE("  ",E5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  127, // #3 = Master Volume</v>
       </c>
-      <c r="L5" s="18" t="str">
+      <c r="J5" s="51" t="str">
         <f>CONCATENATE("  ",C5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #3 = Master Volume</v>
       </c>
-      <c r="M5" s="41" t="s">
-        <v>231</v>
-      </c>
-      <c r="N5" s="18" t="str">
+      <c r="K5" s="41" t="s">
+        <v>229</v>
+      </c>
+      <c r="L5" s="51" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">  &amp;setOrganVolumes, // Master Volume</v>
       </c>
-      <c r="O5" s="39" t="s">
-        <v>243</v>
-      </c>
-      <c r="P5" s="13" t="str">
-        <f>CONCATENATE("  ",O5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;preset.masterVolume, // #3 = Master Volume</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="39" t="s">
+        <v>253</v>
+      </c>
+      <c r="N5" s="51" t="str">
+        <f>CONCATENATE("  ",M5,", // #",A5," = ",B5,IF(C5&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;preamp.masterVolume, // #3 = Master Volume</v>
+      </c>
+      <c r="O5" s="42" t="s">
+        <v>247</v>
+      </c>
+      <c r="P5" s="1">
+        <f>A33</f>
+        <v>31</v>
+      </c>
+      <c r="Q5" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>const uint8_t m_pedal_db_16 = 31;</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1705,46 +1821,49 @@
       <c r="F6" s="12">
         <v>40</v>
       </c>
-      <c r="G6" s="12" t="str">
-        <f t="shared" ref="G6" si="3">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B6,"/","")," ","_")))</f>
-        <v>m_amp_gain</v>
-      </c>
-      <c r="H6" s="18" t="str">
-        <f>CONCATENATE("  ",G6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_amp_gain, // #4 = Amp Gain</v>
-      </c>
-      <c r="I6" s="1" t="str">
-        <f>CONCATENATE("  { """,B6,""" },  // #",A6," ",IF(C6&lt;0," EXIT SUBM",""))</f>
+      <c r="G6" s="50" t="str">
+        <f t="shared" si="1"/>
         <v xml:space="preserve">  { "Amp Gain" },  // #4 </v>
       </c>
-      <c r="J6" s="18" t="str">
+      <c r="H6" s="51" t="str">
         <f>CONCATENATE("  ",D6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #4 = Amp Gain</v>
       </c>
-      <c r="K6" s="18" t="str">
+      <c r="I6" s="51" t="str">
         <f>CONCATENATE("  ",E6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  127, // #4 = Amp Gain</v>
       </c>
-      <c r="L6" s="18" t="str">
+      <c r="J6" s="51" t="str">
         <f>CONCATENATE("  ",C6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #4 = Amp Gain</v>
       </c>
-      <c r="M6" s="41" t="s">
-        <v>242</v>
-      </c>
-      <c r="N6" s="18" t="str">
+      <c r="K6" s="41" t="s">
+        <v>240</v>
+      </c>
+      <c r="L6" s="51" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">  &amp;setAmpVolume, // Amp Gain</v>
       </c>
-      <c r="O6" s="39" t="s">
-        <v>244</v>
-      </c>
-      <c r="P6" s="13" t="str">
-        <f>CONCATENATE("  ",O6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;preset.ampVolume, // #4 = Amp Gain</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M6" s="39" t="s">
+        <v>254</v>
+      </c>
+      <c r="N6" s="51" t="str">
+        <f>CONCATENATE("  ",M6,", // #",A6," = ",B6,IF(C6&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;preamp.ampVolume, // #4 = Amp Gain</v>
+      </c>
+      <c r="O6" s="42" t="s">
+        <v>248</v>
+      </c>
+      <c r="P6" s="1">
+        <f>A36</f>
+        <v>34</v>
+      </c>
+      <c r="Q6" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>const uint8_t m_sd_card_info = 34;</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1753,7 +1872,7 @@
         <v>206</v>
       </c>
       <c r="C7" s="5" t="str">
-        <f>G34</f>
+        <f>O6</f>
         <v>m_sd_card_info</v>
       </c>
       <c r="D7" s="12">
@@ -1765,46 +1884,49 @@
       <c r="F7" s="12">
         <v>-47</v>
       </c>
-      <c r="G7" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B7,"/","")," ","_")))</f>
-        <v>m_sd_flash_tools</v>
-      </c>
-      <c r="H7" s="18" t="str">
-        <f>CONCATENATE("  ",G7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_sd_flash_tools, // #5 = SD Flash Tools</v>
-      </c>
-      <c r="I7" s="1" t="str">
-        <f>CONCATENATE("  { """,B7,""" },  // #",A7," ",IF(C7&lt;0," EXIT SUBM",""))</f>
+      <c r="G7" s="50" t="str">
+        <f t="shared" si="1"/>
         <v xml:space="preserve">  { "SD Flash Tools" },  // #5 </v>
       </c>
-      <c r="J7" s="18" t="str">
+      <c r="H7" s="51" t="str">
         <f>CONCATENATE("  ",D7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #5 = SD Flash Tools</v>
       </c>
-      <c r="K7" s="18" t="str">
+      <c r="I7" s="51" t="str">
         <f>CONCATENATE("  ",E7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  127, // #5 = SD Flash Tools</v>
       </c>
-      <c r="L7" s="18" t="str">
+      <c r="J7" s="51" t="str">
         <f>CONCATENATE("  ",C7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_sd_card_info, // #5 = SD Flash Tools</v>
       </c>
+      <c r="K7" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L7" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #5 = SD Flash Tools</v>
+      </c>
       <c r="M7" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N7" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O7" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P7" s="13" t="str">
-        <f>CONCATENATE("  ",O7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
+        <v>207</v>
+      </c>
+      <c r="N7" s="51" t="str">
+        <f>CONCATENATE("  ",M7,", // #",A7," = ",B7,IF(C7&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  NULL, // #5 = SD Flash Tools</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="O7" s="42" t="s">
+        <v>249</v>
+      </c>
+      <c r="P7" s="1">
+        <f>A44</f>
+        <v>42</v>
+      </c>
+      <c r="Q7" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>const uint8_t m_kbd_driver = 42;</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1813,7 +1935,7 @@
         <v>61</v>
       </c>
       <c r="C8" s="5" t="str">
-        <f>G42</f>
+        <f>O7</f>
         <v>m_kbd_driver</v>
       </c>
       <c r="D8" s="1">
@@ -1825,287 +1947,259 @@
       <c r="F8" s="1">
         <v>0</v>
       </c>
-      <c r="G8" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(B8," ","_")))</f>
-        <v>m_keyboard</v>
-      </c>
-      <c r="H8" s="18" t="str">
-        <f>CONCATENATE("  ",G8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_keyboard, // #6 = Keyboard</v>
-      </c>
-      <c r="I8" s="1" t="str">
-        <f>CONCATENATE("  { """,B8,""" },  // #",A8," ",IF(C8&lt;0," EXIT SUBM",""))</f>
+      <c r="G8" s="50" t="str">
+        <f t="shared" si="1"/>
         <v xml:space="preserve">  { "Keyboard" },  // #6 </v>
       </c>
-      <c r="J8" s="18" t="str">
+      <c r="H8" s="51" t="str">
         <f>CONCATENATE("  ",D8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #6 = Keyboard</v>
       </c>
-      <c r="K8" s="18" t="str">
+      <c r="I8" s="51" t="str">
         <f>CONCATENATE("  ",E8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  0, // #6 = Keyboard</v>
       </c>
-      <c r="L8" s="18" t="str">
+      <c r="J8" s="51" t="str">
         <f>CONCATENATE("  ",C8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  m_kbd_driver, // #6 = Keyboard</v>
       </c>
+      <c r="K8" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L8" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #6 = Keyboard</v>
+      </c>
       <c r="M8" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N8" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O8" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P8" s="13" t="str">
-        <f>CONCATENATE("  ",O8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
+        <v>207</v>
+      </c>
+      <c r="N8" s="51" t="str">
+        <f>CONCATENATE("  ",M8,", // #",A8," = ",B8,IF(C8&lt;0," EXIT ",""))</f>
         <v xml:space="preserve">  NULL, // #6 = Keyboard</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O8" s="42" t="s">
+        <v>256</v>
+      </c>
+      <c r="P8" s="14">
+        <f>A12</f>
+        <v>10</v>
+      </c>
+      <c r="Q8" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>const uint8_t m_menu_end = 10;</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="1">
+        <v>241</v>
+      </c>
+      <c r="C9" s="47">
         <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>-1</v>
-      </c>
-      <c r="E9" s="1">
-        <v>31</v>
+        <v>0</v>
+      </c>
+      <c r="E9" s="19">
+        <v>15</v>
       </c>
       <c r="F9" s="1">
-        <v>-1</v>
-      </c>
-      <c r="G9" s="12" t="str">
+        <v>0</v>
+      </c>
+      <c r="G9" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>m_pitchwheel_pot</v>
-      </c>
-      <c r="H9" s="18" t="str">
-        <f>CONCATENATE("  ",G9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_pitchwheel_pot, // #7 = Pitchwheel Pot</v>
-      </c>
-      <c r="I9" s="1" t="str">
-        <f>CONCATENATE("  { """,B9,""" },  // #",A9," ",IF(C9&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pitchwheel Pot" },  // #7 </v>
-      </c>
-      <c r="J9" s="18" t="str">
+        <v xml:space="preserve">  { "Organ Model" },  // #7 </v>
+      </c>
+      <c r="H9" s="51" t="str">
         <f>CONCATENATE("  ",D9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #7 = Pitchwheel Pot</v>
-      </c>
-      <c r="K9" s="18" t="str">
+        <v xml:space="preserve">  0, // #7 = Organ Model</v>
+      </c>
+      <c r="I9" s="51" t="str">
         <f>CONCATENATE("  ",E9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  31, // #7 = Pitchwheel Pot</v>
-      </c>
-      <c r="L9" s="18" t="str">
+        <v xml:space="preserve">  15, // #7 = Organ Model</v>
+      </c>
+      <c r="J9" s="51" t="str">
         <f>CONCATENATE("  ",C9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #7 = Pitchwheel Pot</v>
+        <v xml:space="preserve">  0, // #7 = Organ Model</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="L9" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;menuOrganModel, // Organ Model</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N9" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O9" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P9" s="13" t="str">
-        <f>CONCATENATE("  ",O9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #7 = Pitchwheel Pot</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+      <c r="N9" s="51" t="str">
+        <f>CONCATENATE("  ",M9,", // #",A9," = ",B9,IF(C9&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;tabs.speakerModel, // #7 = Organ Model</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" s="22">
-        <v>0</v>
-      </c>
-      <c r="D10" s="22">
-        <v>0</v>
-      </c>
-      <c r="E10" s="22">
-        <v>0</v>
-      </c>
-      <c r="F10" s="22">
-        <v>0</v>
-      </c>
-      <c r="G10" s="34" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="26" t="str">
-        <f>CONCATENATE("  ",G10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_end, // #8 = End</v>
-      </c>
-      <c r="I10" s="22" t="str">
-        <f>CONCATENATE("  { """,B10,""" },  // #",A10," ",IF(C10&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "End" },  // #8 </v>
-      </c>
-      <c r="J10" s="26" t="str">
+      <c r="B10" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="47">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="19">
+        <v>15</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Speaker Model" },  // #8 </v>
+      </c>
+      <c r="H10" s="51" t="str">
         <f>CONCATENATE("  ",D10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #8 = End</v>
-      </c>
-      <c r="K10" s="26" t="str">
+        <v xml:space="preserve">  0, // #8 = Speaker Model</v>
+      </c>
+      <c r="I10" s="51" t="str">
         <f>CONCATENATE("  ",E10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #8 = End</v>
-      </c>
-      <c r="L10" s="26" t="str">
+        <v xml:space="preserve">  15, // #8 = Speaker Model</v>
+      </c>
+      <c r="J10" s="51" t="str">
         <f>CONCATENATE("  ",C10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #8 = End</v>
-      </c>
-      <c r="M10" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N10" s="18" t="str">
+        <v xml:space="preserve">  0, // #8 = Speaker Model</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="L10" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O10" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P10" s="13" t="str">
-        <f>CONCATENATE("  ",O10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #8 = End</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <v xml:space="preserve">  &amp;menuSpeakerModel, // Speaker Model</v>
+      </c>
+      <c r="M10" s="49" t="s">
+        <v>263</v>
+      </c>
+      <c r="N10" s="51" t="str">
+        <f>CONCATENATE("  ",M10,", // #",A10," = ",B10,IF(C10&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;tabs.organModel, // #8 = Speaker Model</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B11" s="35" t="s">
-        <v>175</v>
+      <c r="B11" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
-      <c r="D11" s="12">
-        <v>0</v>
-      </c>
-      <c r="E11" s="12">
-        <v>127</v>
-      </c>
-      <c r="F11" s="12">
-        <v>127</v>
-      </c>
-      <c r="G11" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B11,"/","")," ","_")))</f>
-        <v>m_upper_db_16</v>
-      </c>
-      <c r="H11" s="18" t="str">
-        <f>CONCATENATE("  ",G11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_16, // #9 = Upper DB 16</v>
-      </c>
-      <c r="I11" s="1" t="str">
-        <f>CONCATENATE("  { """,B11,""" },  // #",A11," ",IF(C11&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 16" },  // #9 </v>
-      </c>
-      <c r="J11" s="18" t="str">
+      <c r="D11" s="1">
+        <v>-1</v>
+      </c>
+      <c r="E11" s="1">
+        <v>31</v>
+      </c>
+      <c r="F11" s="1">
+        <v>-1</v>
+      </c>
+      <c r="G11" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Pitchwheel Pot" },  // #9 </v>
+      </c>
+      <c r="H11" s="51" t="str">
         <f>CONCATENATE("  ",D11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #9 = Upper DB 16</v>
-      </c>
-      <c r="K11" s="18" t="str">
+        <v xml:space="preserve">  -1, // #9 = Pitchwheel Pot</v>
+      </c>
+      <c r="I11" s="51" t="str">
         <f>CONCATENATE("  ",E11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #9 = Upper DB 16</v>
-      </c>
-      <c r="L11" s="18" t="str">
+        <v xml:space="preserve">  31, // #9 = Pitchwheel Pot</v>
+      </c>
+      <c r="J11" s="51" t="str">
         <f>CONCATENATE("  ",C11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #9 = Upper DB 16</v>
+        <v xml:space="preserve">  0, // #9 = Pitchwheel Pot</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L11" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #9 = Pitchwheel Pot</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N11" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 16</v>
-      </c>
-      <c r="O11" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="P11" s="13" t="str">
-        <f>CONCATENATE("  ",O11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[0], // #9 = Upper DB 16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N11" s="51" t="str">
+        <f>CONCATENATE("  ",M11,", // #",A11," = ",B11,IF(C11&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #9 = Pitchwheel Pot</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B12" s="29" t="s">
-        <v>176</v>
-      </c>
-      <c r="C12" s="1">
-        <v>0</v>
-      </c>
-      <c r="D12" s="12">
-        <v>0</v>
-      </c>
-      <c r="E12" s="12">
-        <v>127</v>
-      </c>
-      <c r="F12" s="12">
-        <v>127</v>
-      </c>
-      <c r="G12" s="12" t="str">
-        <f t="shared" ref="G12:G19" si="4">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B12,"/","")," ","_")))</f>
-        <v>m_upper_db_5_13</v>
-      </c>
-      <c r="H12" s="18" t="str">
-        <f>CONCATENATE("  ",G12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_5_13, // #10 = Upper DB 5 1/3</v>
-      </c>
-      <c r="I12" s="1" t="str">
-        <f>CONCATENATE("  { """,B12,""" },  // #",A12," ",IF(C12&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 5 1/3" },  // #10 </v>
-      </c>
-      <c r="J12" s="18" t="str">
+      <c r="B12" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="C12" s="22">
+        <v>0</v>
+      </c>
+      <c r="D12" s="22">
+        <v>0</v>
+      </c>
+      <c r="E12" s="22">
+        <v>0</v>
+      </c>
+      <c r="F12" s="22">
+        <v>0</v>
+      </c>
+      <c r="G12" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "End" },  // #10 </v>
+      </c>
+      <c r="H12" s="52" t="str">
         <f>CONCATENATE("  ",D12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #10 = Upper DB 5 1/3</v>
-      </c>
-      <c r="K12" s="18" t="str">
+        <v xml:space="preserve">  0, // #10 = End</v>
+      </c>
+      <c r="I12" s="52" t="str">
         <f>CONCATENATE("  ",E12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #10 = Upper DB 5 1/3</v>
-      </c>
-      <c r="L12" s="18" t="str">
+        <v xml:space="preserve">  0, // #10 = End</v>
+      </c>
+      <c r="J12" s="52" t="str">
         <f>CONCATENATE("  ",C12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #10 = Upper DB 5 1/3</v>
+        <v xml:space="preserve">  0, // #10 = End</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L12" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #10 = End</v>
       </c>
       <c r="M12" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N12" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 5 1/3</v>
-      </c>
-      <c r="O12" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="P12" s="13" t="str">
-        <f>CONCATENATE("  ",O12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[1], // #10 = Upper DB 5 1/3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N12" s="51" t="str">
+        <f>CONCATENATE("  ",M12,", // #",A12," = ",B12,IF(C12&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #10 = End</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B13" s="29" t="s">
-        <v>177</v>
+      <c r="B13" s="35" t="s">
+        <v>175</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
@@ -2119,52 +2213,44 @@
       <c r="F13" s="12">
         <v>127</v>
       </c>
-      <c r="G13" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_8</v>
-      </c>
-      <c r="H13" s="18" t="str">
-        <f>CONCATENATE("  ",G13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_8, // #11 = Upper DB 8</v>
-      </c>
-      <c r="I13" s="1" t="str">
-        <f>CONCATENATE("  { """,B13,""" },  // #",A13," ",IF(C13&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 8" },  // #11 </v>
-      </c>
-      <c r="J13" s="18" t="str">
+      <c r="G13" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 16" },  // #11 </v>
+      </c>
+      <c r="H13" s="51" t="str">
         <f>CONCATENATE("  ",D13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #11 = Upper DB 8</v>
-      </c>
-      <c r="K13" s="18" t="str">
+        <v xml:space="preserve">  0, // #11 = Upper DB 16</v>
+      </c>
+      <c r="I13" s="51" t="str">
         <f>CONCATENATE("  ",E13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #11 = Upper DB 8</v>
-      </c>
-      <c r="L13" s="18" t="str">
+        <v xml:space="preserve">  127, // #11 = Upper DB 16</v>
+      </c>
+      <c r="J13" s="51" t="str">
         <f>CONCATENATE("  ",C13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #11 = Upper DB 8</v>
+        <v xml:space="preserve">  0, // #11 = Upper DB 16</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L13" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 16</v>
       </c>
       <c r="M13" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N13" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 8</v>
-      </c>
-      <c r="O13" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="P13" s="13" t="str">
-        <f>CONCATENATE("  ",O13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[2], // #11 = Upper DB 8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+      <c r="N13" s="51" t="str">
+        <f>CONCATENATE("  ",M13,", // #",A13," = ",B13,IF(C13&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[0], // #11 = Upper DB 16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C14" s="1">
         <v>0</v>
@@ -2176,54 +2262,46 @@
         <v>127</v>
       </c>
       <c r="F14" s="12">
-        <v>50</v>
-      </c>
-      <c r="G14" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_4</v>
-      </c>
-      <c r="H14" s="18" t="str">
-        <f>CONCATENATE("  ",G14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_4, // #12 = Upper DB 4</v>
-      </c>
-      <c r="I14" s="1" t="str">
-        <f>CONCATENATE("  { """,B14,""" },  // #",A14," ",IF(C14&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 4" },  // #12 </v>
-      </c>
-      <c r="J14" s="18" t="str">
+        <v>127</v>
+      </c>
+      <c r="G14" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 5 1/3" },  // #12 </v>
+      </c>
+      <c r="H14" s="51" t="str">
         <f>CONCATENATE("  ",D14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #12 = Upper DB 4</v>
-      </c>
-      <c r="K14" s="18" t="str">
+        <v xml:space="preserve">  0, // #12 = Upper DB 5 1/3</v>
+      </c>
+      <c r="I14" s="51" t="str">
         <f>CONCATENATE("  ",E14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #12 = Upper DB 4</v>
-      </c>
-      <c r="L14" s="18" t="str">
+        <v xml:space="preserve">  127, // #12 = Upper DB 5 1/3</v>
+      </c>
+      <c r="J14" s="51" t="str">
         <f>CONCATENATE("  ",C14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #12 = Upper DB 4</v>
+        <v xml:space="preserve">  0, // #12 = Upper DB 5 1/3</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L14" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 5 1/3</v>
       </c>
       <c r="M14" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N14" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 4</v>
-      </c>
-      <c r="O14" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="P14" s="13" t="str">
-        <f>CONCATENATE("  ",O14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[3], // #12 = Upper DB 4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+      <c r="N14" s="51" t="str">
+        <f>CONCATENATE("  ",M14,", // #",A14," = ",B14,IF(C14&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[1], // #12 = Upper DB 5 1/3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C15" s="1">
         <v>0</v>
@@ -2235,54 +2313,46 @@
         <v>127</v>
       </c>
       <c r="F15" s="12">
-        <v>0</v>
-      </c>
-      <c r="G15" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_2_23</v>
-      </c>
-      <c r="H15" s="18" t="str">
-        <f>CONCATENATE("  ",G15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_2_23, // #13 = Upper DB 2 2/3</v>
-      </c>
-      <c r="I15" s="1" t="str">
-        <f>CONCATENATE("  { """,B15,""" },  // #",A15," ",IF(C15&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 2 2/3" },  // #13 </v>
-      </c>
-      <c r="J15" s="18" t="str">
+        <v>127</v>
+      </c>
+      <c r="G15" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 8" },  // #13 </v>
+      </c>
+      <c r="H15" s="51" t="str">
         <f>CONCATENATE("  ",D15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #13 = Upper DB 2 2/3</v>
-      </c>
-      <c r="K15" s="18" t="str">
+        <v xml:space="preserve">  0, // #13 = Upper DB 8</v>
+      </c>
+      <c r="I15" s="51" t="str">
         <f>CONCATENATE("  ",E15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #13 = Upper DB 2 2/3</v>
-      </c>
-      <c r="L15" s="18" t="str">
+        <v xml:space="preserve">  127, // #13 = Upper DB 8</v>
+      </c>
+      <c r="J15" s="51" t="str">
         <f>CONCATENATE("  ",C15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #13 = Upper DB 2 2/3</v>
+        <v xml:space="preserve">  0, // #13 = Upper DB 8</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L15" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 8</v>
       </c>
       <c r="M15" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N15" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 2 2/3</v>
-      </c>
-      <c r="O15" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="P15" s="13" t="str">
-        <f>CONCATENATE("  ",O15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[4], // #13 = Upper DB 2 2/3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+      <c r="N15" s="51" t="str">
+        <f>CONCATENATE("  ",M15,", // #",A15," = ",B15,IF(C15&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[2], // #13 = Upper DB 8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C16" s="1">
         <v>0</v>
@@ -2294,54 +2364,46 @@
         <v>127</v>
       </c>
       <c r="F16" s="12">
-        <v>0</v>
-      </c>
-      <c r="G16" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_2</v>
-      </c>
-      <c r="H16" s="18" t="str">
-        <f>CONCATENATE("  ",G16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_2, // #14 = Upper DB 2</v>
-      </c>
-      <c r="I16" s="1" t="str">
-        <f>CONCATENATE("  { """,B16,""" },  // #",A16," ",IF(C16&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 2" },  // #14 </v>
-      </c>
-      <c r="J16" s="18" t="str">
+        <v>50</v>
+      </c>
+      <c r="G16" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 4" },  // #14 </v>
+      </c>
+      <c r="H16" s="51" t="str">
         <f>CONCATENATE("  ",D16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #14 = Upper DB 2</v>
-      </c>
-      <c r="K16" s="18" t="str">
+        <v xml:space="preserve">  0, // #14 = Upper DB 4</v>
+      </c>
+      <c r="I16" s="51" t="str">
         <f>CONCATENATE("  ",E16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #14 = Upper DB 2</v>
-      </c>
-      <c r="L16" s="18" t="str">
+        <v xml:space="preserve">  127, // #14 = Upper DB 4</v>
+      </c>
+      <c r="J16" s="51" t="str">
         <f>CONCATENATE("  ",C16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #14 = Upper DB 2</v>
+        <v xml:space="preserve">  0, // #14 = Upper DB 4</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L16" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 4</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N16" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 2</v>
-      </c>
-      <c r="O16" s="18" t="s">
-        <v>215</v>
-      </c>
-      <c r="P16" s="13" t="str">
-        <f>CONCATENATE("  ",O16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[5], // #14 = Upper DB 2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+      <c r="N16" s="51" t="str">
+        <f>CONCATENATE("  ",M16,", // #",A16," = ",B16,IF(C16&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[3], // #14 = Upper DB 4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C17" s="1">
         <v>0</v>
@@ -2355,52 +2417,44 @@
       <c r="F17" s="12">
         <v>0</v>
       </c>
-      <c r="G17" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_1_35</v>
-      </c>
-      <c r="H17" s="18" t="str">
-        <f>CONCATENATE("  ",G17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_1_35, // #15 = Upper DB 1 3/5</v>
-      </c>
-      <c r="I17" s="1" t="str">
-        <f>CONCATENATE("  { """,B17,""" },  // #",A17," ",IF(C17&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 1 3/5" },  // #15 </v>
-      </c>
-      <c r="J17" s="18" t="str">
+      <c r="G17" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 2 2/3" },  // #15 </v>
+      </c>
+      <c r="H17" s="51" t="str">
         <f>CONCATENATE("  ",D17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #15 = Upper DB 1 3/5</v>
-      </c>
-      <c r="K17" s="18" t="str">
+        <v xml:space="preserve">  0, // #15 = Upper DB 2 2/3</v>
+      </c>
+      <c r="I17" s="51" t="str">
         <f>CONCATENATE("  ",E17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #15 = Upper DB 1 3/5</v>
-      </c>
-      <c r="L17" s="18" t="str">
+        <v xml:space="preserve">  127, // #15 = Upper DB 2 2/3</v>
+      </c>
+      <c r="J17" s="51" t="str">
         <f>CONCATENATE("  ",C17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #15 = Upper DB 1 3/5</v>
+        <v xml:space="preserve">  0, // #15 = Upper DB 2 2/3</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L17" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 2 2/3</v>
       </c>
       <c r="M17" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N17" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1 3/5</v>
-      </c>
-      <c r="O17" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="P17" s="13" t="str">
-        <f>CONCATENATE("  ",O17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[6], // #15 = Upper DB 1 3/5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+      <c r="N17" s="51" t="str">
+        <f>CONCATENATE("  ",M17,", // #",A17," = ",B17,IF(C17&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[4], // #15 = Upper DB 2 2/3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C18" s="1">
         <v>0</v>
@@ -2414,52 +2468,44 @@
       <c r="F18" s="12">
         <v>0</v>
       </c>
-      <c r="G18" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_1_13</v>
-      </c>
-      <c r="H18" s="18" t="str">
-        <f>CONCATENATE("  ",G18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_1_13, // #16 = Upper DB 1 1/3</v>
-      </c>
-      <c r="I18" s="1" t="str">
-        <f>CONCATENATE("  { """,B18,""" },  // #",A18," ",IF(C18&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 1 1/3" },  // #16 </v>
-      </c>
-      <c r="J18" s="18" t="str">
+      <c r="G18" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 2" },  // #16 </v>
+      </c>
+      <c r="H18" s="51" t="str">
         <f>CONCATENATE("  ",D18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #16 = Upper DB 1 1/3</v>
-      </c>
-      <c r="K18" s="18" t="str">
+        <v xml:space="preserve">  0, // #16 = Upper DB 2</v>
+      </c>
+      <c r="I18" s="51" t="str">
         <f>CONCATENATE("  ",E18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #16 = Upper DB 1 1/3</v>
-      </c>
-      <c r="L18" s="18" t="str">
+        <v xml:space="preserve">  127, // #16 = Upper DB 2</v>
+      </c>
+      <c r="J18" s="51" t="str">
         <f>CONCATENATE("  ",C18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #16 = Upper DB 1 1/3</v>
+        <v xml:space="preserve">  0, // #16 = Upper DB 2</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L18" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 2</v>
       </c>
       <c r="M18" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N18" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1 1/3</v>
-      </c>
-      <c r="O18" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="P18" s="13" t="str">
-        <f>CONCATENATE("  ",O18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[7], // #16 = Upper DB 1 1/3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+      <c r="N18" s="51" t="str">
+        <f>CONCATENATE("  ",M18,", // #",A18," = ",B18,IF(C18&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[5], // #16 = Upper DB 2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C19" s="1">
         <v>0</v>
@@ -2473,111 +2519,95 @@
       <c r="F19" s="12">
         <v>0</v>
       </c>
-      <c r="G19" s="12" t="str">
-        <f t="shared" si="4"/>
-        <v>m_upper_db_1</v>
-      </c>
-      <c r="H19" s="18" t="str">
-        <f>CONCATENATE("  ",G19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_db_1, // #17 = Upper DB 1</v>
-      </c>
-      <c r="I19" s="1" t="str">
-        <f>CONCATENATE("  { """,B19,""" },  // #",A19," ",IF(C19&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB 1" },  // #17 </v>
-      </c>
-      <c r="J19" s="18" t="str">
+      <c r="G19" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 1 3/5" },  // #17 </v>
+      </c>
+      <c r="H19" s="51" t="str">
         <f>CONCATENATE("  ",D19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #17 = Upper DB 1</v>
-      </c>
-      <c r="K19" s="18" t="str">
+        <v xml:space="preserve">  0, // #17 = Upper DB 1 3/5</v>
+      </c>
+      <c r="I19" s="51" t="str">
         <f>CONCATENATE("  ",E19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #17 = Upper DB 1</v>
-      </c>
-      <c r="L19" s="18" t="str">
+        <v xml:space="preserve">  127, // #17 = Upper DB 1 3/5</v>
+      </c>
+      <c r="J19" s="51" t="str">
         <f>CONCATENATE("  ",C19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #17 = Upper DB 1</v>
+        <v xml:space="preserve">  0, // #17 = Upper DB 1 3/5</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L19" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1 3/5</v>
       </c>
       <c r="M19" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="N19" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1</v>
-      </c>
-      <c r="O19" s="18" t="s">
-        <v>218</v>
-      </c>
-      <c r="P19" s="13" t="str">
-        <f>CONCATENATE("  ",O19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.upper[8], // #17 = Upper DB 1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+      <c r="N19" s="51" t="str">
+        <f>CONCATENATE("  ",M19,", // #",A19," = ",B19,IF(C19&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[6], // #17 = Upper DB 1 3/5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>196</v>
-      </c>
-      <c r="C20" s="22">
-        <v>-1</v>
-      </c>
-      <c r="D20" s="22">
-        <v>0</v>
-      </c>
-      <c r="E20" s="22">
-        <v>0</v>
-      </c>
-      <c r="F20" s="22">
-        <v>0</v>
-      </c>
-      <c r="G20" s="26" t="str">
-        <f>CONCATENATE("m_back_",A20)</f>
-        <v>m_back_18</v>
-      </c>
-      <c r="H20" s="26" t="str">
-        <f>CONCATENATE("  ",G20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_18, // #18 = Upper DB EXIT </v>
-      </c>
-      <c r="I20" s="22" t="str">
-        <f>CONCATENATE("  { """,B20,""" },  // #",A20," ",IF(C20&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper DB" },  // #18  EXIT SUBM</v>
-      </c>
-      <c r="J20" s="26" t="str">
+      <c r="B20" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0</v>
+      </c>
+      <c r="D20" s="12">
+        <v>0</v>
+      </c>
+      <c r="E20" s="12">
+        <v>127</v>
+      </c>
+      <c r="F20" s="12">
+        <v>0</v>
+      </c>
+      <c r="G20" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 1 1/3" },  // #18 </v>
+      </c>
+      <c r="H20" s="51" t="str">
         <f>CONCATENATE("  ",D20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #18 = Upper DB EXIT </v>
-      </c>
-      <c r="K20" s="26" t="str">
+        <v xml:space="preserve">  0, // #18 = Upper DB 1 1/3</v>
+      </c>
+      <c r="I20" s="51" t="str">
         <f>CONCATENATE("  ",E20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #18 = Upper DB EXIT </v>
-      </c>
-      <c r="L20" s="26" t="str">
+        <v xml:space="preserve">  127, // #18 = Upper DB 1 1/3</v>
+      </c>
+      <c r="J20" s="51" t="str">
         <f>CONCATENATE("  ",C20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #18 = Upper DB EXIT </v>
+        <v xml:space="preserve">  0, // #18 = Upper DB 1 1/3</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L20" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1 1/3</v>
       </c>
       <c r="M20" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N20" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O20" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P20" s="13" t="str">
-        <f>CONCATENATE("  ",O20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #18 = Upper DB EXIT </v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+      <c r="N20" s="51" t="str">
+        <f>CONCATENATE("  ",M20,", // #",A20," = ",B20,IF(C20&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[7], // #18 = Upper DB 1 1/3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B21" s="36" t="s">
-        <v>184</v>
+      <c r="B21" s="29" t="s">
+        <v>183</v>
       </c>
       <c r="C21" s="1">
         <v>0</v>
@@ -2591,111 +2621,95 @@
       <c r="F21" s="12">
         <v>0</v>
       </c>
-      <c r="G21" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B21,"/","")," ","_")))</f>
-        <v>m_lower_db_16</v>
-      </c>
-      <c r="H21" s="18" t="str">
-        <f>CONCATENATE("  ",G21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_16, // #19 = Lower DB 16</v>
-      </c>
-      <c r="I21" s="1" t="str">
-        <f>CONCATENATE("  { """,B21,""" },  // #",A21," ",IF(C21&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 16" },  // #19 </v>
-      </c>
-      <c r="J21" s="18" t="str">
+      <c r="G21" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB 1" },  // #19 </v>
+      </c>
+      <c r="H21" s="51" t="str">
         <f>CONCATENATE("  ",D21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #19 = Lower DB 16</v>
-      </c>
-      <c r="K21" s="18" t="str">
+        <v xml:space="preserve">  0, // #19 = Upper DB 1</v>
+      </c>
+      <c r="I21" s="51" t="str">
         <f>CONCATENATE("  ",E21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #19 = Lower DB 16</v>
-      </c>
-      <c r="L21" s="18" t="str">
+        <v xml:space="preserve">  127, // #19 = Upper DB 1</v>
+      </c>
+      <c r="J21" s="51" t="str">
         <f>CONCATENATE("  ",C21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #19 = Lower DB 16</v>
+        <v xml:space="preserve">  0, // #19 = Upper DB 1</v>
+      </c>
+      <c r="K21" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="L21" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_upper_db, // Upper DB 1</v>
       </c>
       <c r="M21" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N21" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 16</v>
-      </c>
-      <c r="O21" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="P21" s="13" t="str">
-        <f>CONCATENATE("  ",O21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[0], // #19 = Lower DB 16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+      <c r="N21" s="51" t="str">
+        <f>CONCATENATE("  ",M21,", // #",A21," = ",B21,IF(C21&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.upper[8], // #19 = Upper DB 1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B22" s="30" t="s">
-        <v>185</v>
-      </c>
-      <c r="C22" s="1">
-        <v>0</v>
-      </c>
-      <c r="D22" s="12">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12">
-        <v>127</v>
-      </c>
-      <c r="F22" s="12">
-        <v>0</v>
-      </c>
-      <c r="G22" s="12" t="str">
-        <f t="shared" ref="G22:G29" si="5">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B22,"/","")," ","_")))</f>
-        <v>m_lower_db_5_13</v>
-      </c>
-      <c r="H22" s="18" t="str">
-        <f>CONCATENATE("  ",G22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_5_13, // #20 = Lower DB 5 1/3</v>
-      </c>
-      <c r="I22" s="1" t="str">
-        <f>CONCATENATE("  { """,B22,""" },  // #",A22," ",IF(C22&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 5 1/3" },  // #20 </v>
-      </c>
-      <c r="J22" s="18" t="str">
+      <c r="B22" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="C22" s="22">
+        <v>-1</v>
+      </c>
+      <c r="D22" s="22">
+        <v>0</v>
+      </c>
+      <c r="E22" s="22">
+        <v>0</v>
+      </c>
+      <c r="F22" s="22">
+        <v>0</v>
+      </c>
+      <c r="G22" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper DB" },  // #20  EXIT SUBM</v>
+      </c>
+      <c r="H22" s="52" t="str">
         <f>CONCATENATE("  ",D22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #20 = Lower DB 5 1/3</v>
-      </c>
-      <c r="K22" s="18" t="str">
+        <v xml:space="preserve">  0, // #20 = Upper DB EXIT </v>
+      </c>
+      <c r="I22" s="52" t="str">
         <f>CONCATENATE("  ",E22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #20 = Lower DB 5 1/3</v>
-      </c>
-      <c r="L22" s="18" t="str">
+        <v xml:space="preserve">  0, // #20 = Upper DB EXIT </v>
+      </c>
+      <c r="J22" s="52" t="str">
         <f>CONCATENATE("  ",C22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #20 = Lower DB 5 1/3</v>
+        <v xml:space="preserve">  -1, // #20 = Upper DB EXIT </v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L22" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #20 = Upper DB</v>
       </c>
       <c r="M22" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N22" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 5 1/3</v>
-      </c>
-      <c r="O22" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="P22" s="13" t="str">
-        <f>CONCATENATE("  ",O22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[1], // #20 = Lower DB 5 1/3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N22" s="51" t="str">
+        <f>CONCATENATE("  ",M22,", // #",A22," = ",B22,IF(C22&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #20 = Upper DB EXIT </v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B23" s="30" t="s">
-        <v>186</v>
+      <c r="B23" s="36" t="s">
+        <v>184</v>
       </c>
       <c r="C23" s="1">
         <v>0</v>
@@ -2707,54 +2721,46 @@
         <v>127</v>
       </c>
       <c r="F23" s="12">
-        <v>127</v>
-      </c>
-      <c r="G23" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_8</v>
-      </c>
-      <c r="H23" s="18" t="str">
-        <f>CONCATENATE("  ",G23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_8, // #21 = Lower DB 8</v>
-      </c>
-      <c r="I23" s="1" t="str">
-        <f>CONCATENATE("  { """,B23,""" },  // #",A23," ",IF(C23&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 8" },  // #21 </v>
-      </c>
-      <c r="J23" s="18" t="str">
+        <v>0</v>
+      </c>
+      <c r="G23" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 16" },  // #21 </v>
+      </c>
+      <c r="H23" s="51" t="str">
         <f>CONCATENATE("  ",D23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #21 = Lower DB 8</v>
-      </c>
-      <c r="K23" s="18" t="str">
+        <v xml:space="preserve">  0, // #21 = Lower DB 16</v>
+      </c>
+      <c r="I23" s="51" t="str">
         <f>CONCATENATE("  ",E23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #21 = Lower DB 8</v>
-      </c>
-      <c r="L23" s="18" t="str">
+        <v xml:space="preserve">  127, // #21 = Lower DB 16</v>
+      </c>
+      <c r="J23" s="51" t="str">
         <f>CONCATENATE("  ",C23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #21 = Lower DB 8</v>
+        <v xml:space="preserve">  0, // #21 = Lower DB 16</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L23" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 16</v>
       </c>
       <c r="M23" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N23" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 8</v>
-      </c>
-      <c r="O23" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="P23" s="13" t="str">
-        <f>CONCATENATE("  ",O23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[2], // #21 = Lower DB 8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+      <c r="N23" s="51" t="str">
+        <f>CONCATENATE("  ",M23,", // #",A23," = ",B23,IF(C23&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[0], // #21 = Lower DB 16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C24" s="1">
         <v>0</v>
@@ -2766,54 +2772,46 @@
         <v>127</v>
       </c>
       <c r="F24" s="12">
-        <v>127</v>
-      </c>
-      <c r="G24" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_4</v>
-      </c>
-      <c r="H24" s="18" t="str">
-        <f>CONCATENATE("  ",G24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_4, // #22 = Lower DB 4</v>
-      </c>
-      <c r="I24" s="1" t="str">
-        <f>CONCATENATE("  { """,B24,""" },  // #",A24," ",IF(C24&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 4" },  // #22 </v>
-      </c>
-      <c r="J24" s="18" t="str">
+        <v>0</v>
+      </c>
+      <c r="G24" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 5 1/3" },  // #22 </v>
+      </c>
+      <c r="H24" s="51" t="str">
         <f>CONCATENATE("  ",D24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #22 = Lower DB 4</v>
-      </c>
-      <c r="K24" s="18" t="str">
+        <v xml:space="preserve">  0, // #22 = Lower DB 5 1/3</v>
+      </c>
+      <c r="I24" s="51" t="str">
         <f>CONCATENATE("  ",E24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #22 = Lower DB 4</v>
-      </c>
-      <c r="L24" s="18" t="str">
+        <v xml:space="preserve">  127, // #22 = Lower DB 5 1/3</v>
+      </c>
+      <c r="J24" s="51" t="str">
         <f>CONCATENATE("  ",C24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #22 = Lower DB 4</v>
+        <v xml:space="preserve">  0, // #22 = Lower DB 5 1/3</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L24" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 5 1/3</v>
       </c>
       <c r="M24" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N24" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 4</v>
-      </c>
-      <c r="O24" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="P24" s="13" t="str">
-        <f>CONCATENATE("  ",O24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[3], // #22 = Lower DB 4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="N24" s="51" t="str">
+        <f>CONCATENATE("  ",M24,", // #",A24," = ",B24,IF(C24&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[1], // #22 = Lower DB 5 1/3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C25" s="1">
         <v>0</v>
@@ -2825,54 +2823,46 @@
         <v>127</v>
       </c>
       <c r="F25" s="12">
-        <v>40</v>
-      </c>
-      <c r="G25" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_2_23</v>
-      </c>
-      <c r="H25" s="18" t="str">
-        <f>CONCATENATE("  ",G25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_2_23, // #23 = Lower DB 2 2/3</v>
-      </c>
-      <c r="I25" s="1" t="str">
-        <f>CONCATENATE("  { """,B25,""" },  // #",A25," ",IF(C25&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 2 2/3" },  // #23 </v>
-      </c>
-      <c r="J25" s="18" t="str">
+        <v>127</v>
+      </c>
+      <c r="G25" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 8" },  // #23 </v>
+      </c>
+      <c r="H25" s="51" t="str">
         <f>CONCATENATE("  ",D25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #23 = Lower DB 2 2/3</v>
-      </c>
-      <c r="K25" s="18" t="str">
+        <v xml:space="preserve">  0, // #23 = Lower DB 8</v>
+      </c>
+      <c r="I25" s="51" t="str">
         <f>CONCATENATE("  ",E25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #23 = Lower DB 2 2/3</v>
-      </c>
-      <c r="L25" s="18" t="str">
+        <v xml:space="preserve">  127, // #23 = Lower DB 8</v>
+      </c>
+      <c r="J25" s="51" t="str">
         <f>CONCATENATE("  ",C25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #23 = Lower DB 2 2/3</v>
+        <v xml:space="preserve">  0, // #23 = Lower DB 8</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L25" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 8</v>
       </c>
       <c r="M25" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N25" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 2 2/3</v>
-      </c>
-      <c r="O25" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="P25" s="13" t="str">
-        <f>CONCATENATE("  ",O25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[4], // #23 = Lower DB 2 2/3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+      <c r="N25" s="51" t="str">
+        <f>CONCATENATE("  ",M25,", // #",A25," = ",B25,IF(C25&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[2], // #23 = Lower DB 8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C26" s="1">
         <v>0</v>
@@ -2884,54 +2874,46 @@
         <v>127</v>
       </c>
       <c r="F26" s="12">
-        <v>0</v>
-      </c>
-      <c r="G26" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_2</v>
-      </c>
-      <c r="H26" s="18" t="str">
-        <f>CONCATENATE("  ",G26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_2, // #24 = Lower DB 2</v>
-      </c>
-      <c r="I26" s="1" t="str">
-        <f>CONCATENATE("  { """,B26,""" },  // #",A26," ",IF(C26&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 2" },  // #24 </v>
-      </c>
-      <c r="J26" s="18" t="str">
+        <v>127</v>
+      </c>
+      <c r="G26" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 4" },  // #24 </v>
+      </c>
+      <c r="H26" s="51" t="str">
         <f>CONCATENATE("  ",D26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #24 = Lower DB 2</v>
-      </c>
-      <c r="K26" s="18" t="str">
+        <v xml:space="preserve">  0, // #24 = Lower DB 4</v>
+      </c>
+      <c r="I26" s="51" t="str">
         <f>CONCATENATE("  ",E26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #24 = Lower DB 2</v>
-      </c>
-      <c r="L26" s="18" t="str">
+        <v xml:space="preserve">  127, // #24 = Lower DB 4</v>
+      </c>
+      <c r="J26" s="51" t="str">
         <f>CONCATENATE("  ",C26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #24 = Lower DB 2</v>
+        <v xml:space="preserve">  0, // #24 = Lower DB 4</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L26" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 4</v>
       </c>
       <c r="M26" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N26" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 2</v>
-      </c>
-      <c r="O26" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="P26" s="13" t="str">
-        <f>CONCATENATE("  ",O26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[5], // #24 = Lower DB 2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="N26" s="51" t="str">
+        <f>CONCATENATE("  ",M26,", // #",A26," = ",B26,IF(C26&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[3], // #24 = Lower DB 4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C27" s="1">
         <v>0</v>
@@ -2943,54 +2925,46 @@
         <v>127</v>
       </c>
       <c r="F27" s="12">
-        <v>0</v>
-      </c>
-      <c r="G27" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_1_35</v>
-      </c>
-      <c r="H27" s="18" t="str">
-        <f>CONCATENATE("  ",G27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_1_35, // #25 = Lower DB 1 3/5</v>
-      </c>
-      <c r="I27" s="1" t="str">
-        <f>CONCATENATE("  { """,B27,""" },  // #",A27," ",IF(C27&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 1 3/5" },  // #25 </v>
-      </c>
-      <c r="J27" s="18" t="str">
+        <v>40</v>
+      </c>
+      <c r="G27" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 2 2/3" },  // #25 </v>
+      </c>
+      <c r="H27" s="51" t="str">
         <f>CONCATENATE("  ",D27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #25 = Lower DB 1 3/5</v>
-      </c>
-      <c r="K27" s="18" t="str">
+        <v xml:space="preserve">  0, // #25 = Lower DB 2 2/3</v>
+      </c>
+      <c r="I27" s="51" t="str">
         <f>CONCATENATE("  ",E27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #25 = Lower DB 1 3/5</v>
-      </c>
-      <c r="L27" s="18" t="str">
+        <v xml:space="preserve">  127, // #25 = Lower DB 2 2/3</v>
+      </c>
+      <c r="J27" s="51" t="str">
         <f>CONCATENATE("  ",C27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #25 = Lower DB 1 3/5</v>
+        <v xml:space="preserve">  0, // #25 = Lower DB 2 2/3</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L27" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 2 2/3</v>
       </c>
       <c r="M27" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N27" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1 3/5</v>
-      </c>
-      <c r="O27" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="P27" s="13" t="str">
-        <f>CONCATENATE("  ",O27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[6], // #25 = Lower DB 1 3/5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+      <c r="N27" s="51" t="str">
+        <f>CONCATENATE("  ",M27,", // #",A27," = ",B27,IF(C27&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[4], // #25 = Lower DB 2 2/3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C28" s="1">
         <v>0</v>
@@ -3004,52 +2978,44 @@
       <c r="F28" s="12">
         <v>0</v>
       </c>
-      <c r="G28" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_1_13</v>
-      </c>
-      <c r="H28" s="18" t="str">
-        <f>CONCATENATE("  ",G28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_1_13, // #26 = Lower DB 1 1/3</v>
-      </c>
-      <c r="I28" s="1" t="str">
-        <f>CONCATENATE("  { """,B28,""" },  // #",A28," ",IF(C28&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 1 1/3" },  // #26 </v>
-      </c>
-      <c r="J28" s="18" t="str">
+      <c r="G28" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 2" },  // #26 </v>
+      </c>
+      <c r="H28" s="51" t="str">
         <f>CONCATENATE("  ",D28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #26 = Lower DB 1 1/3</v>
-      </c>
-      <c r="K28" s="18" t="str">
+        <v xml:space="preserve">  0, // #26 = Lower DB 2</v>
+      </c>
+      <c r="I28" s="51" t="str">
         <f>CONCATENATE("  ",E28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #26 = Lower DB 1 1/3</v>
-      </c>
-      <c r="L28" s="18" t="str">
+        <v xml:space="preserve">  127, // #26 = Lower DB 2</v>
+      </c>
+      <c r="J28" s="51" t="str">
         <f>CONCATENATE("  ",C28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #26 = Lower DB 1 1/3</v>
+        <v xml:space="preserve">  0, // #26 = Lower DB 2</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L28" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 2</v>
       </c>
       <c r="M28" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N28" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1 1/3</v>
-      </c>
-      <c r="O28" s="18" t="s">
-        <v>226</v>
-      </c>
-      <c r="P28" s="13" t="str">
-        <f>CONCATENATE("  ",O28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[7], // #26 = Lower DB 1 1/3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+      <c r="N28" s="51" t="str">
+        <f>CONCATENATE("  ",M28,", // #",A28," = ",B28,IF(C28&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[5], // #26 = Lower DB 2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C29" s="1">
         <v>0</v>
@@ -3063,111 +3029,95 @@
       <c r="F29" s="12">
         <v>0</v>
       </c>
-      <c r="G29" s="12" t="str">
-        <f t="shared" si="5"/>
-        <v>m_lower_db_1</v>
-      </c>
-      <c r="H29" s="18" t="str">
-        <f>CONCATENATE("  ",G29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_db_1, // #27 = Lower DB 1</v>
-      </c>
-      <c r="I29" s="1" t="str">
-        <f>CONCATENATE("  { """,B29,""" },  // #",A29," ",IF(C29&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB 1" },  // #27 </v>
-      </c>
-      <c r="J29" s="18" t="str">
+      <c r="G29" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 1 3/5" },  // #27 </v>
+      </c>
+      <c r="H29" s="51" t="str">
         <f>CONCATENATE("  ",D29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #27 = Lower DB 1</v>
-      </c>
-      <c r="K29" s="18" t="str">
+        <v xml:space="preserve">  0, // #27 = Lower DB 1 3/5</v>
+      </c>
+      <c r="I29" s="51" t="str">
         <f>CONCATENATE("  ",E29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #27 = Lower DB 1</v>
-      </c>
-      <c r="L29" s="18" t="str">
+        <v xml:space="preserve">  127, // #27 = Lower DB 1 3/5</v>
+      </c>
+      <c r="J29" s="51" t="str">
         <f>CONCATENATE("  ",C29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #27 = Lower DB 1</v>
+        <v xml:space="preserve">  0, // #27 = Lower DB 1 3/5</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L29" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1 3/5</v>
       </c>
       <c r="M29" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="N29" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1</v>
-      </c>
-      <c r="O29" s="18" t="s">
-        <v>227</v>
-      </c>
-      <c r="P29" s="13" t="str">
-        <f>CONCATENATE("  ",O29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.lower[8], // #27 = Lower DB 1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="N29" s="51" t="str">
+        <f>CONCATENATE("  ",M29,", // #",A29," = ",B29,IF(C29&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[6], // #27 = Lower DB 1 3/5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B30" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="C30" s="22">
-        <v>-1</v>
-      </c>
-      <c r="D30" s="22">
-        <v>0</v>
-      </c>
-      <c r="E30" s="22">
-        <v>0</v>
-      </c>
-      <c r="F30" s="22">
-        <v>0</v>
-      </c>
-      <c r="G30" s="26" t="str">
-        <f>CONCATENATE("m_back_",A30)</f>
-        <v>m_back_28</v>
-      </c>
-      <c r="H30" s="26" t="str">
-        <f>CONCATENATE("  ",G30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_28, // #28 = Lower DB EXIT </v>
-      </c>
-      <c r="I30" s="22" t="str">
-        <f>CONCATENATE("  { """,B30,""" },  // #",A30," ",IF(C30&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower DB" },  // #28  EXIT SUBM</v>
-      </c>
-      <c r="J30" s="26" t="str">
+      <c r="B30" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0</v>
+      </c>
+      <c r="D30" s="12">
+        <v>0</v>
+      </c>
+      <c r="E30" s="12">
+        <v>127</v>
+      </c>
+      <c r="F30" s="12">
+        <v>0</v>
+      </c>
+      <c r="G30" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 1 1/3" },  // #28 </v>
+      </c>
+      <c r="H30" s="51" t="str">
         <f>CONCATENATE("  ",D30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #28 = Lower DB EXIT </v>
-      </c>
-      <c r="K30" s="26" t="str">
+        <v xml:space="preserve">  0, // #28 = Lower DB 1 1/3</v>
+      </c>
+      <c r="I30" s="51" t="str">
         <f>CONCATENATE("  ",E30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #28 = Lower DB EXIT </v>
-      </c>
-      <c r="L30" s="26" t="str">
+        <v xml:space="preserve">  127, // #28 = Lower DB 1 1/3</v>
+      </c>
+      <c r="J30" s="51" t="str">
         <f>CONCATENATE("  ",C30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #28 = Lower DB EXIT </v>
+        <v xml:space="preserve">  0, // #28 = Lower DB 1 1/3</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L30" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1 1/3</v>
       </c>
       <c r="M30" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N30" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O30" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P30" s="13" t="str">
-        <f>CONCATENATE("  ",O30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #28 = Lower DB EXIT </v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+      <c r="N30" s="51" t="str">
+        <f>CONCATENATE("  ",M30,", // #",A30," = ",B30,IF(C30&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[7], // #28 = Lower DB 1 1/3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B31" s="37" t="s">
-        <v>193</v>
+      <c r="B31" s="30" t="s">
+        <v>192</v>
       </c>
       <c r="C31" s="1">
         <v>0</v>
@@ -3179,172 +3129,148 @@
         <v>127</v>
       </c>
       <c r="F31" s="12">
-        <v>127</v>
-      </c>
-      <c r="G31" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B31,"/","")," ","_")))</f>
-        <v>m_pedal_db_16</v>
-      </c>
-      <c r="H31" s="18" t="str">
-        <f>CONCATENATE("  ",G31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_pedal_db_16, // #29 = Pedal DB 16</v>
-      </c>
-      <c r="I31" s="1" t="str">
-        <f>CONCATENATE("  { """,B31,""" },  // #",A31," ",IF(C31&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pedal DB 16" },  // #29 </v>
-      </c>
-      <c r="J31" s="18" t="str">
+        <v>0</v>
+      </c>
+      <c r="G31" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB 1" },  // #29 </v>
+      </c>
+      <c r="H31" s="51" t="str">
         <f>CONCATENATE("  ",D31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #29 = Pedal DB 16</v>
-      </c>
-      <c r="K31" s="18" t="str">
+        <v xml:space="preserve">  0, // #29 = Lower DB 1</v>
+      </c>
+      <c r="I31" s="51" t="str">
         <f>CONCATENATE("  ",E31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #29 = Pedal DB 16</v>
-      </c>
-      <c r="L31" s="18" t="str">
+        <v xml:space="preserve">  127, // #29 = Lower DB 1</v>
+      </c>
+      <c r="J31" s="51" t="str">
         <f>CONCATENATE("  ",C31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #29 = Pedal DB 16</v>
+        <v xml:space="preserve">  0, // #29 = Lower DB 1</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="L31" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;fpga_send_lower_db, // Lower DB 1</v>
       </c>
       <c r="M31" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N31" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O31" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="P31" s="13" t="str">
-        <f>CONCATENATE("  ",O31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.pedal[0], // #29 = Pedal DB 16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+      <c r="N31" s="51" t="str">
+        <f>CONCATENATE("  ",M31,", // #",A31," = ",B31,IF(C31&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.lower[8], // #29 = Lower DB 1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B32" s="31" t="s">
-        <v>194</v>
-      </c>
-      <c r="C32" s="1">
-        <v>0</v>
-      </c>
-      <c r="D32" s="12">
-        <v>0</v>
-      </c>
-      <c r="E32" s="12">
-        <v>127</v>
-      </c>
-      <c r="F32" s="12">
-        <v>60</v>
-      </c>
-      <c r="G32" s="12" t="str">
-        <f t="shared" ref="G32" si="6">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B32,"/","")," ","_")))</f>
-        <v>m_pedal_db_8</v>
-      </c>
-      <c r="H32" s="18" t="str">
-        <f>CONCATENATE("  ",G32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_pedal_db_8, // #30 = Pedal DB 8</v>
-      </c>
-      <c r="I32" s="1" t="str">
-        <f>CONCATENATE("  { """,B32,""" },  // #",A32," ",IF(C32&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pedal DB 8" },  // #30 </v>
-      </c>
-      <c r="J32" s="18" t="str">
+      <c r="B32" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" s="22">
+        <v>-1</v>
+      </c>
+      <c r="D32" s="22">
+        <v>0</v>
+      </c>
+      <c r="E32" s="22">
+        <v>0</v>
+      </c>
+      <c r="F32" s="22">
+        <v>0</v>
+      </c>
+      <c r="G32" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower DB" },  // #30  EXIT SUBM</v>
+      </c>
+      <c r="H32" s="52" t="str">
         <f>CONCATENATE("  ",D32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #30 = Pedal DB 8</v>
-      </c>
-      <c r="K32" s="18" t="str">
+        <v xml:space="preserve">  0, // #30 = Lower DB EXIT </v>
+      </c>
+      <c r="I32" s="52" t="str">
         <f>CONCATENATE("  ",E32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  127, // #30 = Pedal DB 8</v>
-      </c>
-      <c r="L32" s="18" t="str">
+        <v xml:space="preserve">  0, // #30 = Lower DB EXIT </v>
+      </c>
+      <c r="J32" s="52" t="str">
         <f>CONCATENATE("  ",C32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #30 = Pedal DB 8</v>
+        <v xml:space="preserve">  -1, // #30 = Lower DB EXIT </v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L32" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #30 = Lower DB</v>
       </c>
       <c r="M32" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N32" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O32" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="P32" s="13" t="str">
-        <f>CONCATENATE("  ",O32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  &amp;drawbars.pedal[1], // #30 = Pedal DB 8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N32" s="51" t="str">
+        <f>CONCATENATE("  ",M32,", // #",A32," = ",B32,IF(C32&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #30 = Lower DB EXIT </v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B33" s="22" t="s">
-        <v>198</v>
-      </c>
-      <c r="C33" s="22">
-        <v>-1</v>
-      </c>
-      <c r="D33" s="22">
-        <v>0</v>
-      </c>
-      <c r="E33" s="22">
-        <v>0</v>
-      </c>
-      <c r="F33" s="22">
-        <v>0</v>
-      </c>
-      <c r="G33" s="26" t="str">
-        <f>CONCATENATE("m_back_",A33)</f>
-        <v>m_back_31</v>
-      </c>
-      <c r="H33" s="26" t="str">
-        <f>CONCATENATE("  ",G33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_31, // #31 = Pedal DB EXIT </v>
-      </c>
-      <c r="I33" s="22" t="str">
-        <f>CONCATENATE("  { """,B33,""" },  // #",A33," ",IF(C33&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pedal DB" },  // #31  EXIT SUBM</v>
-      </c>
-      <c r="J33" s="26" t="str">
+      <c r="B33" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" s="1">
+        <v>0</v>
+      </c>
+      <c r="D33" s="12">
+        <v>0</v>
+      </c>
+      <c r="E33" s="12">
+        <v>127</v>
+      </c>
+      <c r="F33" s="12">
+        <v>127</v>
+      </c>
+      <c r="G33" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Pedal DB 16" },  // #31 </v>
+      </c>
+      <c r="H33" s="51" t="str">
         <f>CONCATENATE("  ",D33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #31 = Pedal DB EXIT </v>
-      </c>
-      <c r="K33" s="26" t="str">
+        <v xml:space="preserve">  0, // #31 = Pedal DB 16</v>
+      </c>
+      <c r="I33" s="51" t="str">
         <f>CONCATENATE("  ",E33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #31 = Pedal DB EXIT </v>
-      </c>
-      <c r="L33" s="26" t="str">
+        <v xml:space="preserve">  127, // #31 = Pedal DB 16</v>
+      </c>
+      <c r="J33" s="51" t="str">
         <f>CONCATENATE("  ",C33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #31 = Pedal DB EXIT </v>
+        <v xml:space="preserve">  0, // #31 = Pedal DB 16</v>
+      </c>
+      <c r="K33" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L33" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #31 = Pedal DB 16</v>
       </c>
       <c r="M33" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N33" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O33" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P33" s="13" t="str">
-        <f>CONCATENATE("  ",O33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #31 = Pedal DB EXIT </v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="N33" s="51" t="str">
+        <f>CONCATENATE("  ",M33,", // #",A33," = ",B33,IF(C33&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.pedal[0], // #31 = Pedal DB 16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B34" s="38" t="s">
-        <v>240</v>
+      <c r="B34" s="31" t="s">
+        <v>194</v>
       </c>
       <c r="C34" s="1">
         <v>0</v>
@@ -3353,116 +3279,100 @@
         <v>0</v>
       </c>
       <c r="E34" s="12">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="F34" s="12">
-        <v>0</v>
-      </c>
-      <c r="G34" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B34,"/","")," ","_")))</f>
-        <v>m_sd_card_info</v>
-      </c>
-      <c r="H34" s="18" t="str">
-        <f>CONCATENATE("  ",G34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_sd_card_info, // #32 = SD Card Info</v>
-      </c>
-      <c r="I34" s="1" t="str">
-        <f>CONCATENATE("  { """,B34,""" },  // #",A34," ",IF(C34&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "SD Card Info" },  // #32 </v>
-      </c>
-      <c r="J34" s="18" t="str">
+        <v>60</v>
+      </c>
+      <c r="G34" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Pedal DB 8" },  // #32 </v>
+      </c>
+      <c r="H34" s="51" t="str">
         <f>CONCATENATE("  ",D34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #32 = SD Card Info</v>
-      </c>
-      <c r="K34" s="18" t="str">
+        <v xml:space="preserve">  0, // #32 = Pedal DB 8</v>
+      </c>
+      <c r="I34" s="51" t="str">
         <f>CONCATENATE("  ",E34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #32 = SD Card Info</v>
-      </c>
-      <c r="L34" s="18" t="str">
+        <v xml:space="preserve">  127, // #32 = Pedal DB 8</v>
+      </c>
+      <c r="J34" s="51" t="str">
         <f>CONCATENATE("  ",C34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #32 = SD Card Info</v>
+        <v xml:space="preserve">  0, // #32 = Pedal DB 8</v>
+      </c>
+      <c r="K34" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L34" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #32 = Pedal DB 8</v>
       </c>
       <c r="M34" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="N34" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;sdCardInfo, // SD Card Info</v>
-      </c>
-      <c r="O34" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P34" s="13" t="str">
-        <f>CONCATENATE("  ",O34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #32 = SD Card Info</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+      <c r="N34" s="51" t="str">
+        <f>CONCATENATE("  ",M34,", // #",A34," = ",B34,IF(C34&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;drawbars.pedal[1], // #32 = Pedal DB 8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="B35" s="38" t="s">
-        <v>200</v>
-      </c>
-      <c r="C35" s="1">
-        <v>0</v>
-      </c>
-      <c r="D35" s="12">
-        <v>0</v>
-      </c>
-      <c r="E35" s="12">
-        <v>0</v>
-      </c>
-      <c r="F35" s="12">
-        <v>0</v>
-      </c>
-      <c r="G35" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B35,"/","")," ","_")))</f>
-        <v>m_load_sd_scan</v>
-      </c>
-      <c r="H35" s="18" t="str">
-        <f>CONCATENATE("  ",G35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_load_sd_scan, // #33 = Load SD Scan</v>
-      </c>
-      <c r="I35" s="1" t="str">
-        <f>CONCATENATE("  { """,B35,""" },  // #",A35," ",IF(C35&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Load SD Scan" },  // #33 </v>
-      </c>
-      <c r="J35" s="18" t="str">
+      <c r="B35" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="C35" s="22">
+        <v>-1</v>
+      </c>
+      <c r="D35" s="22">
+        <v>0</v>
+      </c>
+      <c r="E35" s="22">
+        <v>0</v>
+      </c>
+      <c r="F35" s="22">
+        <v>0</v>
+      </c>
+      <c r="G35" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Pedal DB" },  // #33  EXIT SUBM</v>
+      </c>
+      <c r="H35" s="52" t="str">
         <f>CONCATENATE("  ",D35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
-      </c>
-      <c r="K35" s="18" t="str">
+        <v xml:space="preserve">  0, // #33 = Pedal DB EXIT </v>
+      </c>
+      <c r="I35" s="52" t="str">
         <f>CONCATENATE("  ",E35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
-      </c>
-      <c r="L35" s="18" t="str">
+        <v xml:space="preserve">  0, // #33 = Pedal DB EXIT </v>
+      </c>
+      <c r="J35" s="52" t="str">
         <f>CONCATENATE("  ",C35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #33 = Load SD Scan</v>
+        <v xml:space="preserve">  -1, // #33 = Pedal DB EXIT </v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L35" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #33 = Pedal DB</v>
       </c>
       <c r="M35" s="18" t="s">
-        <v>235</v>
-      </c>
-      <c r="N35" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;loadScanDriver, // Load SD Scan</v>
-      </c>
-      <c r="O35" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P35" s="13" t="str">
-        <f>CONCATENATE("  ",O35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #33 = Load SD Scan</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N35" s="51" t="str">
+        <f>CONCATENATE("  ",M35,", // #",A35," = ",B35,IF(C35&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #33 = Pedal DB EXIT </v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="B36" s="38" t="s">
-        <v>201</v>
+        <v>238</v>
       </c>
       <c r="C36" s="1">
         <v>0</v>
@@ -3476,52 +3386,44 @@
       <c r="F36" s="12">
         <v>0</v>
       </c>
-      <c r="G36" s="12" t="str">
-        <f t="shared" ref="G36:G40" si="7">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B36,"/","")," ","_")))</f>
-        <v>m_flash_sd_scan</v>
-      </c>
-      <c r="H36" s="18" t="str">
-        <f>CONCATENATE("  ",G36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_flash_sd_scan, // #34 = Flash SD Scan</v>
-      </c>
-      <c r="I36" s="1" t="str">
-        <f>CONCATENATE("  { """,B36,""" },  // #",A36," ",IF(C36&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Flash SD Scan" },  // #34 </v>
-      </c>
-      <c r="J36" s="18" t="str">
+      <c r="G36" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "SD Card Info" },  // #34 </v>
+      </c>
+      <c r="H36" s="51" t="str">
         <f>CONCATENATE("  ",D36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
-      </c>
-      <c r="K36" s="18" t="str">
+        <v xml:space="preserve">  0, // #34 = SD Card Info</v>
+      </c>
+      <c r="I36" s="51" t="str">
         <f>CONCATENATE("  ",E36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
-      </c>
-      <c r="L36" s="18" t="str">
+        <v xml:space="preserve">  0, // #34 = SD Card Info</v>
+      </c>
+      <c r="J36" s="51" t="str">
         <f>CONCATENATE("  ",C36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #34 = Flash SD Scan</v>
-      </c>
-      <c r="M36" s="41" t="s">
-        <v>236</v>
-      </c>
-      <c r="N36" s="18" t="str">
+        <v xml:space="preserve">  0, // #34 = SD Card Info</v>
+      </c>
+      <c r="K36" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="L36" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;flashScanDriver, // Flash SD Scan</v>
-      </c>
-      <c r="O36" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P36" s="13" t="str">
-        <f>CONCATENATE("  ",O36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #34 = Flash SD Scan</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+        <v xml:space="preserve">  &amp;sdCardInfo, // SD Card Info</v>
+      </c>
+      <c r="M36" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="N36" s="51" t="str">
+        <f>CONCATENATE("  ",M36,", // #",A36," = ",B36,IF(C36&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #34 = SD Card Info</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="B37" s="38" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -3535,52 +3437,44 @@
       <c r="F37" s="12">
         <v>0</v>
       </c>
-      <c r="G37" s="12" t="str">
-        <f t="shared" si="7"/>
-        <v>m_flash_fpga</v>
-      </c>
-      <c r="H37" s="18" t="str">
-        <f>CONCATENATE("  ",G37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_flash_fpga, // #35 = Flash FPGA</v>
-      </c>
-      <c r="I37" s="1" t="str">
-        <f>CONCATENATE("  { """,B37,""" },  // #",A37," ",IF(C37&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Flash FPGA" },  // #35 </v>
-      </c>
-      <c r="J37" s="18" t="str">
+      <c r="G37" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Load SD Scan" },  // #35 </v>
+      </c>
+      <c r="H37" s="51" t="str">
         <f>CONCATENATE("  ",D37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
-      </c>
-      <c r="K37" s="18" t="str">
+        <v xml:space="preserve">  0, // #35 = Load SD Scan</v>
+      </c>
+      <c r="I37" s="51" t="str">
         <f>CONCATENATE("  ",E37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
-      </c>
-      <c r="L37" s="18" t="str">
+        <v xml:space="preserve">  0, // #35 = Load SD Scan</v>
+      </c>
+      <c r="J37" s="51" t="str">
         <f>CONCATENATE("  ",C37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #35 = Flash FPGA</v>
-      </c>
-      <c r="M37" s="41" t="s">
-        <v>237</v>
-      </c>
-      <c r="N37" s="18" t="str">
+        <v xml:space="preserve">  0, // #35 = Load SD Scan</v>
+      </c>
+      <c r="K37" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="L37" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;flashFPGA, // Flash FPGA</v>
-      </c>
-      <c r="O37" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P37" s="13" t="str">
-        <f>CONCATENATE("  ",O37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #35 = Flash FPGA</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+        <v xml:space="preserve">  &amp;loadScanDriver, // Load SD Scan</v>
+      </c>
+      <c r="M37" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="N37" s="51" t="str">
+        <f>CONCATENATE("  ",M37,", // #",A37," = ",B37,IF(C37&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #35 = Load SD Scan</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="B38" s="38" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C38" s="1">
         <v>0</v>
@@ -3594,52 +3488,44 @@
       <c r="F38" s="12">
         <v>0</v>
       </c>
-      <c r="G38" s="12" t="str">
-        <f t="shared" si="7"/>
-        <v>m_flash_other</v>
-      </c>
-      <c r="H38" s="18" t="str">
-        <f>CONCATENATE("  ",G38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_flash_other, // #36 = Flash Other</v>
-      </c>
-      <c r="I38" s="1" t="str">
-        <f>CONCATENATE("  { """,B38,""" },  // #",A38," ",IF(C38&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Flash Other" },  // #36 </v>
-      </c>
-      <c r="J38" s="18" t="str">
+      <c r="G38" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Flash SD Scan" },  // #36 </v>
+      </c>
+      <c r="H38" s="51" t="str">
         <f>CONCATENATE("  ",D38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #36 = Flash Other</v>
-      </c>
-      <c r="K38" s="18" t="str">
+        <v xml:space="preserve">  0, // #36 = Flash SD Scan</v>
+      </c>
+      <c r="I38" s="51" t="str">
         <f>CONCATENATE("  ",E38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #36 = Flash Other</v>
-      </c>
-      <c r="L38" s="18" t="str">
+        <v xml:space="preserve">  0, // #36 = Flash SD Scan</v>
+      </c>
+      <c r="J38" s="51" t="str">
         <f>CONCATENATE("  ",C38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #36 = Flash Other</v>
-      </c>
-      <c r="M38" s="41" t="s">
-        <v>238</v>
-      </c>
-      <c r="N38" s="18" t="str">
+        <v xml:space="preserve">  0, // #36 = Flash SD Scan</v>
+      </c>
+      <c r="K38" s="41" t="s">
+        <v>234</v>
+      </c>
+      <c r="L38" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;flashOther, // Flash Other</v>
-      </c>
-      <c r="O38" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P38" s="13" t="str">
-        <f>CONCATENATE("  ",O38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #36 = Flash Other</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+        <v xml:space="preserve">  &amp;flashScanDriver, // Flash SD Scan</v>
+      </c>
+      <c r="M38" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="N38" s="51" t="str">
+        <f>CONCATENATE("  ",M38,", // #",A38," = ",B38,IF(C38&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #36 = Flash SD Scan</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
@@ -3653,52 +3539,44 @@
       <c r="F39" s="12">
         <v>0</v>
       </c>
-      <c r="G39" s="12" t="str">
-        <f t="shared" si="7"/>
-        <v>m_reload_fpga</v>
-      </c>
-      <c r="H39" s="18" t="str">
-        <f>CONCATENATE("  ",G39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_reload_fpga, // #37 = Reload FPGA</v>
-      </c>
-      <c r="I39" s="1" t="str">
-        <f>CONCATENATE("  { """,B39,""" },  // #",A39," ",IF(C39&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Reload FPGA" },  // #37 </v>
-      </c>
-      <c r="J39" s="18" t="str">
+      <c r="G39" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Flash FPGA" },  // #37 </v>
+      </c>
+      <c r="H39" s="51" t="str">
         <f>CONCATENATE("  ",D39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
-      </c>
-      <c r="K39" s="18" t="str">
+        <v xml:space="preserve">  0, // #37 = Flash FPGA</v>
+      </c>
+      <c r="I39" s="51" t="str">
         <f>CONCATENATE("  ",E39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
-      </c>
-      <c r="L39" s="18" t="str">
+        <v xml:space="preserve">  0, // #37 = Flash FPGA</v>
+      </c>
+      <c r="J39" s="51" t="str">
         <f>CONCATENATE("  ",C39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #37 = Reload FPGA</v>
+        <v xml:space="preserve">  0, // #37 = Flash FPGA</v>
+      </c>
+      <c r="K39" s="41" t="s">
+        <v>235</v>
+      </c>
+      <c r="L39" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;flashFPGA, // Flash FPGA</v>
       </c>
       <c r="M39" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="N39" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  &amp;organReset, // Reload FPGA</v>
-      </c>
-      <c r="O39" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P39" s="13" t="str">
-        <f>CONCATENATE("  ",O39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #37 = Reload FPGA</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N39" s="51" t="str">
+        <f>CONCATENATE("  ",M39,", // #",A39," = ",B39,IF(C39&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #37 = Flash FPGA</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="B40" s="38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C40" s="1">
         <v>0</v>
@@ -3712,288 +3590,248 @@
       <c r="F40" s="12">
         <v>0</v>
       </c>
-      <c r="G40" s="12" t="str">
-        <f t="shared" si="7"/>
-        <v>m_test</v>
-      </c>
-      <c r="H40" s="18" t="str">
-        <f>CONCATENATE("  ",G40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_test, // #38 = Test</v>
-      </c>
-      <c r="I40" s="1" t="str">
-        <f>CONCATENATE("  { """,B40,""" },  // #",A40," ",IF(C40&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Test" },  // #38 </v>
-      </c>
-      <c r="J40" s="18" t="str">
+      <c r="G40" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Flash Other" },  // #38 </v>
+      </c>
+      <c r="H40" s="51" t="str">
         <f>CONCATENATE("  ",D40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #38 = Test</v>
-      </c>
-      <c r="K40" s="18" t="str">
+        <v xml:space="preserve">  0, // #38 = Flash Other</v>
+      </c>
+      <c r="I40" s="51" t="str">
         <f>CONCATENATE("  ",E40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #38 = Test</v>
-      </c>
-      <c r="L40" s="18" t="str">
+        <v xml:space="preserve">  0, // #38 = Flash Other</v>
+      </c>
+      <c r="J40" s="51" t="str">
         <f>CONCATENATE("  ",C40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #38 = Test</v>
+        <v xml:space="preserve">  0, // #38 = Flash Other</v>
+      </c>
+      <c r="K40" s="41" t="s">
+        <v>236</v>
+      </c>
+      <c r="L40" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;flashOther, // Flash Other</v>
       </c>
       <c r="M40" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N40" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O40" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P40" s="13" t="str">
-        <f>CONCATENATE("  ",O40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #38 = Test</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N40" s="51" t="str">
+        <f>CONCATENATE("  ",M40,", // #",A40," = ",B40,IF(C40&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #38 = Flash Other</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="B41" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="C41" s="22">
-        <v>-1</v>
-      </c>
-      <c r="D41" s="22">
-        <v>0</v>
-      </c>
-      <c r="E41" s="22">
-        <v>0</v>
-      </c>
-      <c r="F41" s="22">
-        <v>0</v>
-      </c>
-      <c r="G41" s="26" t="str">
-        <f>CONCATENATE("m_back_",A41)</f>
-        <v>m_back_39</v>
-      </c>
-      <c r="H41" s="26" t="str">
-        <f>CONCATENATE("  ",G41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_39, // #39 = Utilities EXIT </v>
-      </c>
-      <c r="I41" s="22" t="str">
-        <f>CONCATENATE("  { """,B41,""" },  // #",A41," ",IF(C41&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Utilities" },  // #39  EXIT SUBM</v>
-      </c>
-      <c r="J41" s="26" t="str">
+      <c r="B41" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0</v>
+      </c>
+      <c r="D41" s="12">
+        <v>0</v>
+      </c>
+      <c r="E41" s="12">
+        <v>0</v>
+      </c>
+      <c r="F41" s="12">
+        <v>0</v>
+      </c>
+      <c r="G41" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Reload FPGA" },  // #39 </v>
+      </c>
+      <c r="H41" s="51" t="str">
         <f>CONCATENATE("  ",D41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #39 = Utilities EXIT </v>
-      </c>
-      <c r="K41" s="26" t="str">
+        <v xml:space="preserve">  0, // #39 = Reload FPGA</v>
+      </c>
+      <c r="I41" s="51" t="str">
         <f>CONCATENATE("  ",E41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #39 = Utilities EXIT </v>
-      </c>
-      <c r="L41" s="26" t="str">
+        <v xml:space="preserve">  0, // #39 = Reload FPGA</v>
+      </c>
+      <c r="J41" s="51" t="str">
         <f>CONCATENATE("  ",C41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #39 = Utilities EXIT </v>
+        <v xml:space="preserve">  0, // #39 = Reload FPGA</v>
+      </c>
+      <c r="K41" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="L41" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  &amp;organReset, // Reload FPGA</v>
       </c>
       <c r="M41" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N41" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O41" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P41" s="13" t="str">
-        <f>CONCATENATE("  ",O41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #39 = Utilities EXIT </v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N41" s="51" t="str">
+        <f>CONCATENATE("  ",M41,", // #",A41," = ",B41,IF(C41&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #39 = Reload FPGA</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="B42" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="C42" s="20">
-        <v>0</v>
-      </c>
-      <c r="D42" s="20">
-        <v>0</v>
-      </c>
-      <c r="E42" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G42" s="12" t="str">
-        <f>CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B42,"/","")," ","_")))</f>
-        <v>m_kbd_driver</v>
-      </c>
-      <c r="H42" s="18" t="str">
-        <f>CONCATENATE("  ",G42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_kbd_driver, // #40 = Kbd Driver</v>
-      </c>
-      <c r="I42" s="1" t="str">
-        <f>CONCATENATE("  { """,B42,""" },  // #",A42," ",IF(C42&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Kbd Driver" },  // #40 </v>
-      </c>
-      <c r="J42" s="18" t="str">
+      <c r="B42" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="C42" s="1">
+        <v>0</v>
+      </c>
+      <c r="D42" s="12">
+        <v>0</v>
+      </c>
+      <c r="E42" s="12">
+        <v>0</v>
+      </c>
+      <c r="F42" s="12">
+        <v>0</v>
+      </c>
+      <c r="G42" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Test" },  // #40 </v>
+      </c>
+      <c r="H42" s="51" t="str">
         <f>CONCATENATE("  ",D42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #40 = Kbd Driver</v>
-      </c>
-      <c r="K42" s="18" t="str">
+        <v xml:space="preserve">  0, // #40 = Test</v>
+      </c>
+      <c r="I42" s="51" t="str">
         <f>CONCATENATE("  ",E42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  drv_custom, // #40 = Kbd Driver</v>
-      </c>
-      <c r="L42" s="18" t="str">
+        <v xml:space="preserve">  0, // #40 = Test</v>
+      </c>
+      <c r="J42" s="51" t="str">
         <f>CONCATENATE("  ",C42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #40 = Kbd Driver</v>
+        <v xml:space="preserve">  0, // #40 = Test</v>
+      </c>
+      <c r="K42" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L42" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #40 = Test</v>
       </c>
       <c r="M42" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N42" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O42" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P42" s="13" t="str">
-        <f>CONCATENATE("  ",O42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #40 = Kbd Driver</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N42" s="51" t="str">
+        <f>CONCATENATE("  ",M42,", // #",A42," = ",B42,IF(C42&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #40 = Test</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" s="1">
-        <v>0</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1</v>
-      </c>
-      <c r="E43" s="1">
-        <v>40</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G43" s="12" t="str">
-        <f t="shared" ref="G43:G48" si="8">CONCATENATE("m_",LOWER(SUBSTITUTE(SUBSTITUTE(B43,"/","")," ","_")))</f>
-        <v>m_velocity_min</v>
-      </c>
-      <c r="H43" s="18" t="str">
-        <f>CONCATENATE("  ",G43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_velocity_min, // #41 = Velocity Min</v>
-      </c>
-      <c r="I43" s="1" t="str">
-        <f>CONCATENATE("  { """,B43,""" },  // #",A43," ",IF(C43&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Velocity Min" },  // #41 </v>
-      </c>
-      <c r="J43" s="18" t="str">
+      <c r="B43" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="C43" s="22">
+        <v>-1</v>
+      </c>
+      <c r="D43" s="22">
+        <v>0</v>
+      </c>
+      <c r="E43" s="22">
+        <v>0</v>
+      </c>
+      <c r="F43" s="22">
+        <v>0</v>
+      </c>
+      <c r="G43" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Utilities" },  // #41  EXIT SUBM</v>
+      </c>
+      <c r="H43" s="52" t="str">
         <f>CONCATENATE("  ",D43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  1, // #41 = Velocity Min</v>
-      </c>
-      <c r="K43" s="18" t="str">
+        <v xml:space="preserve">  0, // #41 = Utilities EXIT </v>
+      </c>
+      <c r="I43" s="52" t="str">
         <f>CONCATENATE("  ",E43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  40, // #41 = Velocity Min</v>
-      </c>
-      <c r="L43" s="18" t="str">
+        <v xml:space="preserve">  0, // #41 = Utilities EXIT </v>
+      </c>
+      <c r="J43" s="52" t="str">
         <f>CONCATENATE("  ",C43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #41 = Velocity Min</v>
+        <v xml:space="preserve">  -1, // #41 = Utilities EXIT </v>
+      </c>
+      <c r="K43" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L43" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #41 = Utilities</v>
       </c>
       <c r="M43" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N43" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O43" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P43" s="13" t="str">
-        <f>CONCATENATE("  ",O43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #41 = Velocity Min</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N43" s="51" t="str">
+        <f>CONCATENATE("  ",M43,", // #",A43," = ",B43,IF(C43&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #41 = Utilities EXIT </v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C44" s="1">
-        <v>0</v>
-      </c>
-      <c r="D44" s="1">
-        <v>1</v>
-      </c>
-      <c r="E44" s="1">
-        <v>40</v>
+      <c r="B44" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="20">
+        <v>0</v>
+      </c>
+      <c r="D44" s="20">
+        <v>0</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>38</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G44" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v>m_velocity_maxadj</v>
-      </c>
-      <c r="H44" s="18" t="str">
-        <f>CONCATENATE("  ",G44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_velocity_maxadj, // #42 = Velocity MaxAdj</v>
-      </c>
-      <c r="I44" s="1" t="str">
-        <f>CONCATENATE("  { """,B44,""" },  // #",A44," ",IF(C44&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Velocity MaxAdj" },  // #42 </v>
-      </c>
-      <c r="J44" s="18" t="str">
+        <v>31</v>
+      </c>
+      <c r="G44" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Kbd Driver" },  // #42 </v>
+      </c>
+      <c r="H44" s="51" t="str">
         <f>CONCATENATE("  ",D44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  1, // #42 = Velocity MaxAdj</v>
-      </c>
-      <c r="K44" s="18" t="str">
+        <v xml:space="preserve">  0, // #42 = Kbd Driver</v>
+      </c>
+      <c r="I44" s="51" t="str">
         <f>CONCATENATE("  ",E44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  40, // #42 = Velocity MaxAdj</v>
-      </c>
-      <c r="L44" s="18" t="str">
+        <v xml:space="preserve">  drv_custom, // #42 = Kbd Driver</v>
+      </c>
+      <c r="J44" s="51" t="str">
         <f>CONCATENATE("  ",C44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #42 = Velocity MaxAdj</v>
+        <v xml:space="preserve">  0, // #42 = Kbd Driver</v>
+      </c>
+      <c r="K44" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L44" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #42 = Kbd Driver</v>
       </c>
       <c r="M44" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N44" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O44" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P44" s="13" t="str">
-        <f>CONCATENATE("  ",O44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #42 = Velocity MaxAdj</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+        <v>258</v>
+      </c>
+      <c r="N44" s="51" t="str">
+        <f>CONCATENATE("  ",M44,", // #",A44," = ",B44,IF(C44&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;boardInfo.scan_driverIdx, // #42 = Kbd Driver</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C45" s="1">
         <v>0</v>
@@ -4002,175 +3840,151 @@
         <v>1</v>
       </c>
       <c r="E45" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G45" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v>m_velocity_slope</v>
-      </c>
-      <c r="H45" s="18" t="str">
-        <f>CONCATENATE("  ",G45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_velocity_slope, // #43 = Velocity Slope</v>
-      </c>
-      <c r="I45" s="1" t="str">
-        <f>CONCATENATE("  { """,B45,""" },  // #",A45," ",IF(C45&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Velocity Slope" },  // #43 </v>
-      </c>
-      <c r="J45" s="18" t="str">
+        <v>35</v>
+      </c>
+      <c r="G45" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Velocity Min" },  // #43 </v>
+      </c>
+      <c r="H45" s="51" t="str">
         <f>CONCATENATE("  ",D45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  1, // #43 = Velocity Slope</v>
-      </c>
-      <c r="K45" s="18" t="str">
+        <v xml:space="preserve">  1, // #43 = Velocity Min</v>
+      </c>
+      <c r="I45" s="51" t="str">
         <f>CONCATENATE("  ",E45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  30, // #43 = Velocity Slope</v>
-      </c>
-      <c r="L45" s="18" t="str">
+        <v xml:space="preserve">  40, // #43 = Velocity Min</v>
+      </c>
+      <c r="J45" s="51" t="str">
         <f>CONCATENATE("  ",C45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #43 = Velocity Slope</v>
+        <v xml:space="preserve">  0, // #43 = Velocity Min</v>
+      </c>
+      <c r="K45" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L45" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #43 = Velocity Min</v>
       </c>
       <c r="M45" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N45" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O45" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P45" s="13" t="str">
-        <f>CONCATENATE("  ",O45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #43 = Velocity Slope</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N45" s="51" t="str">
+        <f>CONCATENATE("  ",M45,", // #",A45," = ",B45,IF(C45&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #43 = Velocity Min</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="C46" s="1">
         <v>0</v>
       </c>
       <c r="D46" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E46" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G46" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v>m_upper_base</v>
-      </c>
-      <c r="H46" s="18" t="str">
-        <f>CONCATENATE("  ",G46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_upper_base, // #44 = Upper Base</v>
-      </c>
-      <c r="I46" s="1" t="str">
-        <f>CONCATENATE("  { """,B46,""" },  // #",A46," ",IF(C46&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Upper Base" },  // #44 </v>
-      </c>
-      <c r="J46" s="18" t="str">
+        <v>36</v>
+      </c>
+      <c r="G46" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Velocity MaxAdj" },  // #44 </v>
+      </c>
+      <c r="H46" s="51" t="str">
         <f>CONCATENATE("  ",D46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  12, // #44 = Upper Base</v>
-      </c>
-      <c r="K46" s="18" t="str">
+        <v xml:space="preserve">  1, // #44 = Velocity MaxAdj</v>
+      </c>
+      <c r="I46" s="51" t="str">
         <f>CONCATENATE("  ",E46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  60, // #44 = Upper Base</v>
-      </c>
-      <c r="L46" s="18" t="str">
+        <v xml:space="preserve">  40, // #44 = Velocity MaxAdj</v>
+      </c>
+      <c r="J46" s="51" t="str">
         <f>CONCATENATE("  ",C46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #44 = Upper Base</v>
+        <v xml:space="preserve">  0, // #44 = Velocity MaxAdj</v>
+      </c>
+      <c r="K46" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L46" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #44 = Velocity MaxAdj</v>
       </c>
       <c r="M46" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N46" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O46" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P46" s="13" t="str">
-        <f>CONCATENATE("  ",O46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #44 = Upper Base</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+      <c r="N46" s="51" t="str">
+        <f>CONCATENATE("  ",M46,", // #",A46," = ",B46,IF(C46&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #44 = Velocity MaxAdj</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
       </c>
       <c r="D47" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E47" s="1">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G47" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v>m_lower_base</v>
-      </c>
-      <c r="H47" s="18" t="str">
-        <f>CONCATENATE("  ",G47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_lower_base, // #45 = Lower Base</v>
-      </c>
-      <c r="I47" s="1" t="str">
-        <f>CONCATENATE("  { """,B47,""" },  // #",A47," ",IF(C47&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Lower Base" },  // #45 </v>
-      </c>
-      <c r="J47" s="18" t="str">
+        <v>37</v>
+      </c>
+      <c r="G47" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Velocity Slope" },  // #45 </v>
+      </c>
+      <c r="H47" s="51" t="str">
         <f>CONCATENATE("  ",D47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  12, // #45 = Lower Base</v>
-      </c>
-      <c r="K47" s="18" t="str">
+        <v xml:space="preserve">  1, // #45 = Velocity Slope</v>
+      </c>
+      <c r="I47" s="51" t="str">
         <f>CONCATENATE("  ",E47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  60, // #45 = Lower Base</v>
-      </c>
-      <c r="L47" s="18" t="str">
+        <v xml:space="preserve">  30, // #45 = Velocity Slope</v>
+      </c>
+      <c r="J47" s="51" t="str">
         <f>CONCATENATE("  ",C47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #45 = Lower Base</v>
+        <v xml:space="preserve">  0, // #45 = Velocity Slope</v>
+      </c>
+      <c r="K47" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L47" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #45 = Velocity Slope</v>
       </c>
       <c r="M47" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N47" s="18" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O47" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P47" s="13" t="str">
-        <f>CONCATENATE("  ",O47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #45 = Lower Base</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+      <c r="N47" s="51" t="str">
+        <f>CONCATENATE("  ",M47,", // #",A47," = ",B47,IF(C47&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;organModel.fatarVelocityFac, // #45 = Velocity Slope</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
-        <f>A47+1</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C48" s="1">
         <v>0</v>
@@ -4182,130 +3996,222 @@
         <v>60</v>
       </c>
       <c r="F48" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G48" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Upper Base" },  // #46 </v>
+      </c>
+      <c r="H48" s="51" t="str">
+        <f>CONCATENATE("  ",D48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  12, // #46 = Upper Base</v>
+      </c>
+      <c r="I48" s="51" t="str">
+        <f>CONCATENATE("  ",E48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  60, // #46 = Upper Base</v>
+      </c>
+      <c r="J48" s="51" t="str">
+        <f>CONCATENATE("  ",C48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #46 = Upper Base</v>
+      </c>
+      <c r="K48" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L48" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #46 = Upper Base</v>
+      </c>
+      <c r="M48" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="N48" s="51" t="str">
+        <f>CONCATENATE("  ",M48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;midiSettings.channel, // #46 = Upper Base</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="1">
+        <v>0</v>
+      </c>
+      <c r="D49" s="1">
+        <v>12</v>
+      </c>
+      <c r="E49" s="1">
+        <v>60</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Lower Base" },  // #47 </v>
+      </c>
+      <c r="H49" s="51" t="str">
+        <f>CONCATENATE("  ",D49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  12, // #47 = Lower Base</v>
+      </c>
+      <c r="I49" s="51" t="str">
+        <f>CONCATENATE("  ",E49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  60, // #47 = Lower Base</v>
+      </c>
+      <c r="J49" s="51" t="str">
+        <f>CONCATENATE("  ",C49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #47 = Lower Base</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L49" s="51" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve">  NULL, // #47 = Lower Base</v>
+      </c>
+      <c r="M49" s="49" t="s">
+        <v>259</v>
+      </c>
+      <c r="N49" s="51" t="str">
+        <f>CONCATENATE("  ",M49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;midiSettings.channelLower, // #47 = Lower Base</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <f>A49+1</f>
+        <v>48</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="1">
+        <v>0</v>
+      </c>
+      <c r="D50" s="1">
+        <v>12</v>
+      </c>
+      <c r="E50" s="1">
+        <v>60</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G48" s="12" t="str">
-        <f t="shared" si="8"/>
-        <v>m_pedal_base</v>
-      </c>
-      <c r="H48" s="18" t="str">
-        <f>CONCATENATE("  ",G48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_pedal_base, // #46 = Pedal Base</v>
-      </c>
-      <c r="I48" s="1" t="str">
-        <f>CONCATENATE("  { """,B48,""" },  // #",A48," ",IF(C48&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "Pedal Base" },  // #46 </v>
-      </c>
-      <c r="J48" s="18" t="str">
-        <f>CONCATENATE("  ",D48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  12, // #46 = Pedal Base</v>
-      </c>
-      <c r="K48" s="18" t="str">
-        <f>CONCATENATE("  ",E48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  60, // #46 = Pedal Base</v>
-      </c>
-      <c r="L48" s="18" t="str">
-        <f>CONCATENATE("  ",C48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #46 = Pedal Base</v>
-      </c>
-      <c r="M48" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N48" s="18" t="str">
+      <c r="G50" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "Pedal Base" },  // #48 </v>
+      </c>
+      <c r="H50" s="51" t="str">
+        <f>CONCATENATE("  ",D50,", // #",A50," = ",B50,IF(C50&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  12, // #48 = Pedal Base</v>
+      </c>
+      <c r="I50" s="51" t="str">
+        <f>CONCATENATE("  ",E50,", // #",A50," = ",B50,IF(C50&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  60, // #48 = Pedal Base</v>
+      </c>
+      <c r="J50" s="51" t="str">
+        <f>CONCATENATE("  ",C50,", // #",A50," = ",B50,IF(C50&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #48 = Pedal Base</v>
+      </c>
+      <c r="K50" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L50" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O48" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P48" s="13" t="str">
-        <f>CONCATENATE("  ",O48,", // #",A48," = ",B48,IF(C48&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #46 = Pedal Base</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
-        <f>A48+1</f>
-        <v>47</v>
-      </c>
-      <c r="B49" s="22" t="s">
+        <v xml:space="preserve">  NULL, // #48 = Pedal Base</v>
+      </c>
+      <c r="M50" s="49" t="s">
+        <v>260</v>
+      </c>
+      <c r="N50" s="51" t="str">
+        <f>CONCATENATE("  ",M50,", // #",A50," = ",B50,IF(C50&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  &amp;midiSettings.channelPedal, // #48 = Pedal Base</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <f>A50+1</f>
+        <v>49</v>
+      </c>
+      <c r="B51" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C49" s="22">
+      <c r="C51" s="22">
         <v>-1</v>
       </c>
-      <c r="D49" s="22">
-        <v>0</v>
-      </c>
-      <c r="E49" s="22">
-        <v>0</v>
-      </c>
-      <c r="F49" s="22">
-        <v>0</v>
-      </c>
-      <c r="G49" s="26" t="str">
-        <f>CONCATENATE("m_back_",A49)</f>
-        <v>m_back_47</v>
-      </c>
-      <c r="H49" s="26" t="str">
-        <f>CONCATENATE("  ",G49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  m_back_47, // #47 = (Keyboard) EXIT </v>
-      </c>
-      <c r="I49" s="22" t="str">
-        <f>CONCATENATE("  { """,B49,""" },  // #",A49," ",IF(C49&lt;0," EXIT SUBM",""))</f>
-        <v xml:space="preserve">  { "(Keyboard)" },  // #47  EXIT SUBM</v>
-      </c>
-      <c r="J49" s="26" t="str">
-        <f>CONCATENATE("  ",D49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #47 = (Keyboard) EXIT </v>
-      </c>
-      <c r="K49" s="26" t="str">
-        <f>CONCATENATE("  ",E49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  0, // #47 = (Keyboard) EXIT </v>
-      </c>
-      <c r="L49" s="26" t="str">
-        <f>CONCATENATE("  ",C49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  -1, // #47 = (Keyboard) EXIT </v>
-      </c>
-      <c r="M49" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="N49" s="18" t="str">
+      <c r="D51" s="22">
+        <v>0</v>
+      </c>
+      <c r="E51" s="22">
+        <v>0</v>
+      </c>
+      <c r="F51" s="22">
+        <v>0</v>
+      </c>
+      <c r="G51" s="50" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve">  { "(Keyboard)" },  // #49  EXIT SUBM</v>
+      </c>
+      <c r="H51" s="52" t="str">
+        <f>CONCATENATE("  ",D51,", // #",A51," = ",B51,IF(C51&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #49 = (Keyboard) EXIT </v>
+      </c>
+      <c r="I51" s="52" t="str">
+        <f>CONCATENATE("  ",E51,", // #",A51," = ",B51,IF(C51&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  0, // #49 = (Keyboard) EXIT </v>
+      </c>
+      <c r="J51" s="52" t="str">
+        <f>CONCATENATE("  ",C51,", // #",A51," = ",B51,IF(C51&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  -1, // #49 = (Keyboard) EXIT </v>
+      </c>
+      <c r="K51" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="L51" s="51" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  NULL,</v>
-      </c>
-      <c r="O49" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="P49" s="13" t="str">
-        <f>CONCATENATE("  ",O49,", // #",A49," = ",B49,IF(C49&lt;0," EXIT ",""))</f>
-        <v xml:space="preserve">  NULL, // #47 = (Keyboard) EXIT </v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H50" s="15" t="s">
+        <v xml:space="preserve">  NULL, // #49 = (Keyboard)</v>
+      </c>
+      <c r="M51" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="N51" s="51" t="str">
+        <f>CONCATENATE("  ",M51,", // #",A51," = ",B51,IF(C51&lt;0," EXIT ",""))</f>
+        <v xml:space="preserve">  NULL, // #49 = (Keyboard) EXIT </v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="I50" s="1" t="s">
+      <c r="H52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="J50" s="1" t="s">
+      <c r="I52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="K50" s="1" t="s">
+      <c r="J52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="L50" s="1" t="s">
+      <c r="K52" s="1"/>
+      <c r="L52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="M50" s="1"/>
-      <c r="N50" s="1" t="s">
+      <c r="M52" s="1"/>
+      <c r="N52" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="O50" s="1"/>
-      <c r="P50" s="1" t="s">
-        <v>20</v>
-      </c>
+    </row>
+    <row r="54" spans="1:14" s="34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="43"/>
+      <c r="E54" s="44"/>
+      <c r="F54" s="44"/>
+      <c r="G54" s="44"/>
+      <c r="H54" s="44"/>
+      <c r="K54" s="45"/>
+      <c r="M54" s="45"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>